<commit_message>
commit after running apply-names
</commit_message>
<xml_diff>
--- a/Excel/3_5_Enteric_Swine_WIP_v02.xlsx
+++ b/Excel/3_5_Enteric_Swine_WIP_v02.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\htdocs\zneagcrc\GAF-VEERG-Functions\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37C85E99-C83A-42F8-878A-59CDAA561384}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92456BE4-F994-42AA-B62B-D1785BC62230}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="990" yWindow="510" windowWidth="37170" windowHeight="19920" activeTab="3" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
+    <workbookView xWindow="585" yWindow="495" windowWidth="37785" windowHeight="19140" activeTab="3" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="71" r:id="rId1"/>
@@ -6310,7 +6310,7 @@
     <tableColumn id="1" xr3:uid="{A1AC17BE-6F0C-4EA3-88D1-F15B8A0AA6A1}" name="Class">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Swine.SourceData_Swine_VolatileSolids_Data(), Table_SourceData_Swine_VolatileSolids[[#Headers],[Class]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{539845C7-E401-474C-86C5-B676BBD1B040}" name="VSj" dataDxfId="43" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{539845C7-E401-474C-86C5-B676BBD1B040}" name="VSj" dataDxfId="80" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Swine.SourceData_Swine_VolatileSolids_Data(), Table_SourceData_Swine_VolatileSolids[[#Headers],[Class]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6341,20 +6341,20 @@
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="27" xr:uid="{1333872B-E46C-4DC7-8E2D-1F3D704794C8}" name="Table_SourceData_Swine_FracGASM28" displayName="Table_SourceData_Swine_FracGASM28" ref="D111:F117" totalsRowShown="0" dataDxfId="25" dataCellStyle="Content normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="27" xr:uid="{1333872B-E46C-4DC7-8E2D-1F3D704794C8}" name="Table_SourceData_Swine_FracGASM28" displayName="Table_SourceData_Swine_FracGASM28" ref="D111:F117" totalsRowShown="0" dataDxfId="62" dataCellStyle="Content normal">
   <autoFilter ref="D111:F117" xr:uid="{1333872B-E46C-4DC7-8E2D-1F3D704794C8}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{6DD7EF85-D333-4B03-BD58-78D84BEEC9B4}" name="MMSm" dataDxfId="24" dataCellStyle="Content normal">
+    <tableColumn id="1" xr3:uid="{6DD7EF85-D333-4B03-BD58-78D84BEEC9B4}" name="MMSm" dataDxfId="61" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Swine.SourceData_Swine_NitrousOxideEFs_Data(), Table_SourceData_Swine_FracGASM28[[#Headers],[MMSm]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{F61F4819-1794-4A31-843F-5F15C9F3C95F}" name="EFmT" dataDxfId="23" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{F61F4819-1794-4A31-843F-5F15C9F3C95F}" name="EFmT" dataDxfId="60" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Swine.SourceData_Swine_NitrousOxideEFs_Data(), Table_SourceData_Swine_FracGASM28[[#Headers],[MMSm]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{B97B38DF-3EA9-445C-BD0D-2CBB24B993D8}" name="NIR reference" dataDxfId="22" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{B97B38DF-3EA9-445C-BD0D-2CBB24B993D8}" name="NIR reference" dataDxfId="59" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Swine.SourceData_Swine_NitrousOxideEFs_Data(), Table_SourceData_Swine_FracGASM28[[#Headers],[MMSm]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6398,7 +6398,7 @@
     <tableColumn id="1" xr3:uid="{39C5E3A8-688C-4C4E-A337-E32C77B7769F}" name="Livestock type j">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Swine.SourceData_Swine_AverageLiveweight_Data(),Table_SourceData_Swine_Liveweight[[#Headers],[Livestock type j]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{37866161-8EEC-44E3-8B1D-0210A7AFC89C}" name="Average liveweight (kg)" dataDxfId="21" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{37866161-8EEC-44E3-8B1D-0210A7AFC89C}" name="Average liveweight (kg)" dataDxfId="58" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Swine.SourceData_Swine_AverageLiveweight_Data(),Table_SourceData_Swine_Liveweight[[#Headers],[Livestock type j]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6514,49 +6514,49 @@
     <tableColumn id="1" xr3:uid="{71F77FEF-5DA5-48FC-A4EC-D6565B8E968A}" name="Climate zone" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{533F9369-8EBA-4392-808C-6F82710A50B9}" name="MAT" totalsRowDxfId="80" totalsRowCellStyle="Content bold">
+    <tableColumn id="2" xr3:uid="{533F9369-8EBA-4392-808C-6F82710A50B9}" name="MAT" totalsRowDxfId="57" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{E9080D07-580D-4AFF-9E53-17CD4467293E}" name="MAP" totalsRowDxfId="79" totalsRowCellStyle="Content bold">
+    <tableColumn id="3" xr3:uid="{E9080D07-580D-4AFF-9E53-17CD4467293E}" name="MAP" totalsRowDxfId="56" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{34AC0E99-27E9-4F30-8647-90F9BA108B62}" name="Frost days per year" totalsRowDxfId="78" totalsRowCellStyle="Content bold">
+    <tableColumn id="4" xr3:uid="{34AC0E99-27E9-4F30-8647-90F9BA108B62}" name="Frost days per year" totalsRowDxfId="55" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{C3EBF4E5-C730-497B-A70D-9A7FF2DD3CD5}" name="Elevation" totalsRowDxfId="77" totalsRowCellStyle="Content bold">
+    <tableColumn id="5" xr3:uid="{C3EBF4E5-C730-497B-A70D-9A7FF2DD3CD5}" name="Elevation" totalsRowDxfId="54" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{BFD65F2C-CCA4-4893-81D0-318F6ADAABE9}" name="MAP:PET" totalsRowDxfId="76" totalsRowCellStyle="Content bold">
+    <tableColumn id="6" xr3:uid="{BFD65F2C-CCA4-4893-81D0-318F6ADAABE9}" name="MAP:PET" totalsRowDxfId="53" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{BC9C9862-34FA-47DB-9248-2D7316D968C5}" name="Min temp" totalsRowDxfId="75" totalsRowCellStyle="Content bold">
+    <tableColumn id="7" xr3:uid="{BC9C9862-34FA-47DB-9248-2D7316D968C5}" name="Min temp" totalsRowDxfId="52" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{CE4FF499-BA21-4502-9E55-81F8B39B8CF4}" name="Max temp" totalsRowDxfId="74" totalsRowCellStyle="Content bold">
+    <tableColumn id="8" xr3:uid="{CE4FF499-BA21-4502-9E55-81F8B39B8CF4}" name="Max temp" totalsRowDxfId="51" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{B5278575-0B92-45C9-84B2-A1E944E98820}" name="Min rainfall" totalsRowDxfId="73" totalsRowCellStyle="Content bold">
+    <tableColumn id="9" xr3:uid="{B5278575-0B92-45C9-84B2-A1E944E98820}" name="Min rainfall" totalsRowDxfId="50" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{F9EF9A9E-D211-4A99-A455-772A6AAF236E}" name="Max rainfall" totalsRowDxfId="72" totalsRowCellStyle="Content bold">
+    <tableColumn id="10" xr3:uid="{F9EF9A9E-D211-4A99-A455-772A6AAF236E}" name="Max rainfall" totalsRowDxfId="49" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{862E5ADE-479F-49C7-AD94-EF751714E0A6}" name="Min frost days" totalsRowDxfId="71" totalsRowCellStyle="Content bold">
+    <tableColumn id="11" xr3:uid="{862E5ADE-479F-49C7-AD94-EF751714E0A6}" name="Min frost days" totalsRowDxfId="48" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{68486057-8901-4C62-BEF4-640DC77809F7}" name="Max frost days" totalsRowDxfId="70" totalsRowCellStyle="Content bold">
+    <tableColumn id="15" xr3:uid="{68486057-8901-4C62-BEF4-640DC77809F7}" name="Max frost days" totalsRowDxfId="47" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{21997671-A002-47F3-834F-FA3ABF166EED}" name="Min elevation" totalsRowDxfId="69" totalsRowCellStyle="Content bold">
+    <tableColumn id="12" xr3:uid="{21997671-A002-47F3-834F-FA3ABF166EED}" name="Min elevation" totalsRowDxfId="46" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{5B1B4A66-D90F-4082-809F-58DD0FD24EB8}" name="Max elevation" totalsRowDxfId="68" totalsRowCellStyle="Content bold">
+    <tableColumn id="16" xr3:uid="{5B1B4A66-D90F-4082-809F-58DD0FD24EB8}" name="Max elevation" totalsRowDxfId="45" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{DEB9DEC0-2E93-4A31-ACA3-AB7A4B7B16F7}" name="Min MAP:PET" totalsRowDxfId="67" totalsRowCellStyle="Content bold">
+    <tableColumn id="13" xr3:uid="{DEB9DEC0-2E93-4A31-ACA3-AB7A4B7B16F7}" name="Min MAP:PET" totalsRowDxfId="44" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{3E216ACC-D918-4D1F-A39C-7415BE8D20B3}" name="Max MAP:PET" totalsRowDxfId="66" totalsRowCellStyle="Content bold">
+    <tableColumn id="17" xr3:uid="{3E216ACC-D918-4D1F-A39C-7415BE8D20B3}" name="Max MAP:PET" totalsRowDxfId="43" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6582,31 +6582,31 @@
     <tableColumn id="1" xr3:uid="{948C8C81-0F25-4404-945E-CD16BE93BFBF}" name="MMS">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Swine.SourceData_Swine_MMS_MCFs_Data(),Table_SourceData_Swine_MMSMCF[[#Headers],[MMS]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{CC6F19AB-67BC-413A-9108-447CB795CC02}" name="NSW" dataDxfId="42" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{CC6F19AB-67BC-413A-9108-447CB795CC02}" name="NSW" dataDxfId="79" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Swine.SourceData_Swine_MMS_MCFs_Data(),Table_SourceData_Swine_MMSMCF[[#Headers],[MMS]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{EFE4C41A-233A-4E7D-912F-E949B7110A0A}" name="ACT" dataDxfId="41" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{EFE4C41A-233A-4E7D-912F-E949B7110A0A}" name="ACT" dataDxfId="78" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Swine.SourceData_Swine_MMS_MCFs_Data(),Table_SourceData_Swine_MMSMCF[[#Headers],[MMS]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{90D72B45-949A-49D4-8B76-EF78C1A193C9}" name="QLD" dataDxfId="40" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{90D72B45-949A-49D4-8B76-EF78C1A193C9}" name="QLD" dataDxfId="77" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Swine.SourceData_Swine_MMS_MCFs_Data(),Table_SourceData_Swine_MMSMCF[[#Headers],[MMS]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{D7D725B2-0CF9-4EB2-A5C1-09EDA961537A}" name="NT" dataDxfId="39" dataCellStyle="Content normal">
+    <tableColumn id="5" xr3:uid="{D7D725B2-0CF9-4EB2-A5C1-09EDA961537A}" name="NT" dataDxfId="76" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Swine.SourceData_Swine_MMS_MCFs_Data(),Table_SourceData_Swine_MMSMCF[[#Headers],[MMS]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{2934DF60-275E-438D-A730-DD780A8931E8}" name="SA" dataDxfId="38" dataCellStyle="Content normal">
+    <tableColumn id="6" xr3:uid="{2934DF60-275E-438D-A730-DD780A8931E8}" name="SA" dataDxfId="75" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Swine.SourceData_Swine_MMS_MCFs_Data(),Table_SourceData_Swine_MMSMCF[[#Headers],[MMS]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{29BE3DB6-3057-4DB9-9C8B-816C15103256}" name="TAS" dataDxfId="37" dataCellStyle="Content normal">
+    <tableColumn id="7" xr3:uid="{29BE3DB6-3057-4DB9-9C8B-816C15103256}" name="TAS" dataDxfId="74" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Swine.SourceData_Swine_MMS_MCFs_Data(),Table_SourceData_Swine_MMSMCF[[#Headers],[MMS]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{FF50759B-240C-4451-AB1C-3143673818F2}" name="VIC" dataDxfId="36" dataCellStyle="Content normal">
+    <tableColumn id="8" xr3:uid="{FF50759B-240C-4451-AB1C-3143673818F2}" name="VIC" dataDxfId="73" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Swine.SourceData_Swine_MMS_MCFs_Data(),Table_SourceData_Swine_MMSMCF[[#Headers],[MMS]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{F164F2B6-4BA2-43CA-8A29-E52D5447FFC0}" name="WA" dataDxfId="35" dataCellStyle="Content normal">
+    <tableColumn id="9" xr3:uid="{F164F2B6-4BA2-43CA-8A29-E52D5447FFC0}" name="WA" dataDxfId="72" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Swine.SourceData_Swine_MMS_MCFs_Data(),Table_SourceData_Swine_MMSMCF[[#Headers],[MMS]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{F171BCD0-98D2-4E5E-AC27-147712A91756}" name="NIR definition" dataDxfId="34" dataCellStyle="Content normal">
+    <tableColumn id="10" xr3:uid="{F171BCD0-98D2-4E5E-AC27-147712A91756}" name="NIR definition" dataDxfId="71" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Swine.SourceData_Swine_MMS_MCFs_Data(),Table_SourceData_Swine_MMSMCF[[#Headers],[MMS]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6624,7 +6624,7 @@
     <tableColumn id="1" xr3:uid="{CDBBD1AA-A706-451F-ABDE-23C23829872B}" name="Climate zone" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{FF8BE4D4-1976-4E42-8770-483FC880BDB4}" name="Wet or Dry Zone" totalsRowDxfId="65" totalsRowCellStyle="Content bold">
+    <tableColumn id="2" xr3:uid="{FF8BE4D4-1976-4E42-8770-483FC880BDB4}" name="Wet or Dry Zone" totalsRowDxfId="42" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6730,7 +6730,7 @@
     <tableColumn id="1" xr3:uid="{34AD6582-8E95-4448-A250-240E89847E4A}" name="Is in leaching zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{C3940927-214E-4C98-86AE-ADACF192BCA9}" name="FracWET" dataDxfId="64">
+    <tableColumn id="2" xr3:uid="{C3940927-214E-4C98-86AE-ADACF192BCA9}" name="FracWET" dataDxfId="41">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6778,7 +6778,7 @@
     <tableColumn id="1" xr3:uid="{8D4CCA43-B7CF-49EB-9E74-60A53ACA8E4D}" name="Irrigation type i">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{778FEAF3-8D02-41F3-92B0-ED66A58F2CDD}" name="FracWET" dataDxfId="63" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{778FEAF3-8D02-41F3-92B0-ED66A58F2CDD}" name="FracWET" dataDxfId="40" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6796,7 +6796,7 @@
     <tableColumn id="1" xr3:uid="{11AAB06B-7F71-4384-947E-E0AE7E030BAF}" name="Climate zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Data(), Table_SourceData_EFPastureRangeAndPaddock[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{7A26D427-C856-4145-9747-F08CCA41A6F5}" name="EFPRP" dataDxfId="62" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{7A26D427-C856-4145-9747-F08CCA41A6F5}" name="EFPRP" dataDxfId="39" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Data(), Table_SourceData_EFPastureRangeAndPaddock[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6814,7 +6814,7 @@
     <tableColumn id="1" xr3:uid="{4489322D-5AE6-40C1-BEED-B2944D80F65F}" name="Month">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{1213DFA2-5F54-4F6A-911F-1A1A0FF066AC}" name="Season" dataDxfId="61" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{1213DFA2-5F54-4F6A-911F-1A1A0FF066AC}" name="Season" dataDxfId="38" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6860,49 +6860,49 @@
     <tableColumn id="1" xr3:uid="{DA0B8804-E50D-49C3-BBD5-777B3DD714CB}" name="Temperature zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{CBF1A988-17D4-4C8D-BB65-F3054B9BA01B}" name="MAT (ºC)" dataDxfId="60" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{CBF1A988-17D4-4C8D-BB65-F3054B9BA01B}" name="MAT (ºC)" dataDxfId="37" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{7DC93EB0-E255-4399-A86A-9372E6369FFB}" name="Anaerobic lagoon" dataDxfId="59" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{7DC93EB0-E255-4399-A86A-9372E6369FFB}" name="Anaerobic lagoon" dataDxfId="36" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{2176C1B0-8CD0-499A-8540-4B7AC2E2E8A7}" name="Digester / covered lagoons" dataDxfId="58" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{2176C1B0-8CD0-499A-8540-4B7AC2E2E8A7}" name="Digester / covered lagoons" dataDxfId="35" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{62C02B10-F291-41FE-9EC4-A8CBFAA750DE}" name="Liquid systems" dataDxfId="57" dataCellStyle="Content normal">
+    <tableColumn id="5" xr3:uid="{62C02B10-F291-41FE-9EC4-A8CBFAA750DE}" name="Liquid systems" dataDxfId="34" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{E8F63C19-A7C5-4FDE-A285-A2C9EA3B1394}" name="Daily spread" dataDxfId="56" dataCellStyle="Content normal">
+    <tableColumn id="6" xr3:uid="{E8F63C19-A7C5-4FDE-A285-A2C9EA3B1394}" name="Daily spread" dataDxfId="33" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{DF2A7BD1-FEFB-4A0A-A696-FAC1125D9A62}" name="Composting (passive windrow)" dataDxfId="55" dataCellStyle="Content normal">
+    <tableColumn id="7" xr3:uid="{DF2A7BD1-FEFB-4A0A-A696-FAC1125D9A62}" name="Composting (passive windrow)" dataDxfId="32" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{28CA7996-BCA8-4516-88C7-D142D109F9BE}" name="Solid storage" dataDxfId="54" dataCellStyle="Content normal">
+    <tableColumn id="8" xr3:uid="{28CA7996-BCA8-4516-88C7-D142D109F9BE}" name="Solid storage" dataDxfId="31" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{F3C7333B-9136-4A1B-A4B4-C2B38790829B}" name="Pit storage" dataDxfId="53" dataCellStyle="Content normal">
+    <tableColumn id="9" xr3:uid="{F3C7333B-9136-4A1B-A4B4-C2B38790829B}" name="Pit storage" dataDxfId="30" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{39AA5B79-C37A-45B6-B1DB-FDEC803C706B}" name="Deep litter" dataDxfId="52" dataCellStyle="Content normal">
+    <tableColumn id="10" xr3:uid="{39AA5B79-C37A-45B6-B1DB-FDEC803C706B}" name="Deep litter" dataDxfId="29" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{34E8694A-1411-49D8-B40C-7120CFAED38C}" name="Poultry manure with bedding" dataDxfId="51" dataCellStyle="Content normal">
+    <tableColumn id="11" xr3:uid="{34E8694A-1411-49D8-B40C-7120CFAED38C}" name="Poultry manure with bedding" dataDxfId="28" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{B9D74DB6-031B-4B4F-8C82-B23E803E6B65}" name="Poultry manure without bedding" dataDxfId="50" dataCellStyle="Content normal">
+    <tableColumn id="12" xr3:uid="{B9D74DB6-031B-4B4F-8C82-B23E803E6B65}" name="Poultry manure without bedding" dataDxfId="27" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{DF8CC021-5152-48D6-BAE8-74164E9BCBEE}" name="Direct processing" dataDxfId="49" dataCellStyle="Content normal">
+    <tableColumn id="13" xr3:uid="{DF8CC021-5152-48D6-BAE8-74164E9BCBEE}" name="Direct processing" dataDxfId="26" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{5E638F19-942A-4CD1-8FC4-E477F63A4622}" name="Direct application" dataDxfId="48" dataCellStyle="Content normal">
+    <tableColumn id="14" xr3:uid="{5E638F19-942A-4CD1-8FC4-E477F63A4622}" name="Direct application" dataDxfId="25" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{AF2FEB88-FFD6-4F0D-B66E-0D753D371417}" name="Pasture range and paddock" dataDxfId="47" dataCellStyle="Content normal">
+    <tableColumn id="15" xr3:uid="{AF2FEB88-FFD6-4F0D-B66E-0D753D371417}" name="Pasture range and paddock" dataDxfId="24" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{4CD5B05A-0860-45F3-AF07-E9628AFCE640}" name="MAT raw" dataDxfId="46" dataCellStyle="Content normal">
+    <tableColumn id="16" xr3:uid="{4CD5B05A-0860-45F3-AF07-E9628AFCE640}" name="MAT raw" dataDxfId="23" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6920,7 +6920,7 @@
     <tableColumn id="1" xr3:uid="{50356E5B-3129-47A2-8B24-08A73DEA3863}" name="Climate Zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Data(), Table_SourceData_Common_EFOrganicFertCropResidues[[#Headers],[Climate Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{A304323C-8D8C-483A-947E-6C61A5529433}" name="EFNi &amp; EFN2Oi" dataDxfId="45" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{A304323C-8D8C-483A-947E-6C61A5529433}" name="EFNi &amp; EFN2Oi" dataDxfId="22" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFOrganicFertiliserAndCropResidues_Data(), Table_SourceData_Common_EFOrganicFertCropResidues[[#Headers],[Climate Zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6936,7 +6936,7 @@
     <filterColumn colId="2" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="3">
-    <tableColumn id="2" xr3:uid="{80EBB5A3-AF38-4828-A77A-5F6DD7E49B3F}" name="Description" dataDxfId="44" dataCellStyle="Content normal"/>
+    <tableColumn id="2" xr3:uid="{80EBB5A3-AF38-4828-A77A-5F6DD7E49B3F}" name="Description" dataDxfId="21" dataCellStyle="Content normal"/>
     <tableColumn id="1" xr3:uid="{5C065004-98BF-4E2D-98A7-5F09CC477E38}" name="ID"/>
     <tableColumn id="3" xr3:uid="{FC3B7793-2EF6-4110-A0DB-654BAA6B8A02}" name="Score"/>
   </tableColumns>
@@ -7071,7 +7071,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="24" xr:uid="{61D86DCB-D80D-4593-96F3-A897FC93073F}" name="Table_SourceData_Swine_NitrogenInWaste" displayName="Table_SourceData_Swine_NitrogenInWaste" ref="D89:G93" totalsRowShown="0" dataDxfId="33" dataCellStyle="Content normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="24" xr:uid="{61D86DCB-D80D-4593-96F3-A897FC93073F}" name="Table_SourceData_Swine_NitrogenInWaste" displayName="Table_SourceData_Swine_NitrogenInWaste" ref="D89:G93" totalsRowShown="0" dataDxfId="70" dataCellStyle="Content normal">
   <autoFilter ref="D89:G93" xr:uid="{61D86DCB-D80D-4593-96F3-A897FC93073F}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -7079,16 +7079,16 @@
     <filterColumn colId="3" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{1C4094D2-E798-4EA4-8FBC-50FBA0E527D4}" name="Class" dataDxfId="32" dataCellStyle="Content normal">
+    <tableColumn id="1" xr3:uid="{1C4094D2-E798-4EA4-8FBC-50FBA0E527D4}" name="Class" dataDxfId="69" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Swine.SourceData_Swine_NitrogenInWaste_Data(), Table_SourceData_Swine_NitrogenInWaste[[#Headers],[Class]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{0BD1910A-3F15-4C45-9A95-D2ADDB197E82}" name="NWj" dataDxfId="31" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{0BD1910A-3F15-4C45-9A95-D2ADDB197E82}" name="NWj" dataDxfId="68" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Swine.SourceData_Swine_NitrogenInWaste_Data(), Table_SourceData_Swine_NitrogenInWaste[[#Headers],[Class]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{06D949C0-1431-4E8B-9FED-E08C8D4D7E61}" name="NWj Daily" dataDxfId="30" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{06D949C0-1431-4E8B-9FED-E08C8D4D7E61}" name="NWj Daily" dataDxfId="67" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Swine.SourceData_Swine_NitrogenInWaste_Data(), Table_SourceData_Swine_NitrogenInWaste[[#Headers],[Class]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{5C9C6F5B-830D-4A53-BEF6-FDE389E9F8CC}" name="Class name" dataDxfId="29" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{5C9C6F5B-830D-4A53-BEF6-FDE389E9F8CC}" name="Class name" dataDxfId="66" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Swine.SourceData_Swine_NitrogenInWaste_Data(), Table_SourceData_Swine_NitrogenInWaste[[#Headers],[Class]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -7097,16 +7097,16 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="25" xr:uid="{E34928EB-73E5-43B2-830B-089F30DA4EF0}" name="Table_SourceData_Swine_FeedIntake" displayName="Table_SourceData_Swine_FeedIntake" ref="D78:E82" totalsRowShown="0" dataDxfId="28" dataCellStyle="Content normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="25" xr:uid="{E34928EB-73E5-43B2-830B-089F30DA4EF0}" name="Table_SourceData_Swine_FeedIntake" displayName="Table_SourceData_Swine_FeedIntake" ref="D78:E82" totalsRowShown="0" dataDxfId="65" dataCellStyle="Content normal">
   <autoFilter ref="D78:E82" xr:uid="{E34928EB-73E5-43B2-830B-089F30DA4EF0}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{CAC8EB28-568F-4E9F-8E36-EBDFF74A58D3}" name="Class" dataDxfId="27" dataCellStyle="Content normal">
+    <tableColumn id="1" xr3:uid="{CAC8EB28-568F-4E9F-8E36-EBDFF74A58D3}" name="Class" dataDxfId="64" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Swine.SourceData_Swine_FeedIntake_Data(), Table_SourceData_Swine_FeedIntake[[#Headers],[Class]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{2CE09F11-701B-40A5-9E2D-B745C440FD8B}" name="Ij" dataDxfId="26" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{2CE09F11-701B-40A5-9E2D-B745C440FD8B}" name="Ij" dataDxfId="63" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Swine.SourceData_Swine_FeedIntake_Data(), Table_SourceData_Swine_FeedIntake[[#Headers],[Class]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -9817,7 +9817,7 @@
     </row>
     <row r="6" spans="1:19" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D6" s="41" t="str">
-        <f>"Average duration of stay between " &amp; TEXT(X_Cell_Site_StartDate, "dd mmm yy") &amp; " and " &amp; TEXT('Input - Site'!$E$13, "dd mmm yy")</f>
+        <f>"Average duration of stay between " &amp; TEXT(X_Cell_Site_StartDate, "dd mmm yy") &amp; " and " &amp; TEXT(X_Cell_Site_EndDate, "dd mmm yy")</f>
         <v>Average duration of stay between 01 Jan 24 and 31 Dec 24</v>
       </c>
       <c r="E6" s="58">
@@ -9840,7 +9840,7 @@
     </row>
     <row r="7" spans="1:19" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D7" s="41" t="str">
-        <f>"Average number of head between " &amp; TEXT(X_Cell_Site_StartDate, "dd mmm yy") &amp; " and " &amp; TEXT('Input - Site'!$E$13, "dd mmm yy")</f>
+        <f>"Average number of head between " &amp; TEXT(X_Cell_Site_StartDate, "dd mmm yy") &amp; " and " &amp; TEXT(X_Cell_Site_EndDate, "dd mmm yy")</f>
         <v>Average number of head between 01 Jan 24 and 31 Dec 24</v>
       </c>
       <c r="E7" s="58">
@@ -19066,30 +19066,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7291119c-fce9-4911-96ae-b800be5dccd8">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgAFwAdQAwADAAMgA3AEYAcgB5AFwAdQAwADAAMgA3ACAAdABvACAAXAB1ADAAMAAyADcARAByAHkAXAB1ADAAMAAyADcALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIAVwBlAHQAIABvAHIAIABEAHIAeQAgAFoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAGkAbgAgAE0AQQBUACAAdgBhAGwAdQBlACAAZgBvAHIAIAB3AGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABjAGgAYQBuAGcAZQBkACAAMQAwACAAdABvACAAMQAxAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAG0AaQBuACAAYQBuAGQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIABmAG8AcgAgAE0AQQBUACwAIABNAEEAUAAsACAAZgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgAsACAAZQBsAGUAdgBhAHQAaQBvAG4ALAAgAE0AQQBQADoAUABFAFQAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAcwAgAGYAcgBvAG0AIAByAGUAYQBsACAAYwBsAGkAbQBhAHQAZQAgAGQAYQB0AGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBBAEYAIABhAGMAYwBlAHAAdABzACAAcgBhAGkAbgBmAGEAbABsACAAYQBzACAAYQAgAHAAcgBvAHgAeQAgAGYAbwByACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUAFwAIgAsACAAXAAiAE0AQQBQAFwAIgAsACAAXAAiAEYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIAXAAiACwAIABcACIARQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAHQAZQBtAHAAXAAiACwAIABcACIATQBhAHgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AaQBuACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AYQB4ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AaQBuACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGEAeAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBpAG4AIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGEAeAAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADIAMAAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAG0AIAAtACAAZCIgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwAC4AMAAwADEALAAgADIAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0AGUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFQAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAUAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEUAVAAgAD0AIABwAG8AdABlAG4AdABpAGEAbAAgAGUAdgBhAHAAbwB0AHIAYQBuAHMAcABpAHIAYQB0AGkAbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAE0AQQBUACAAbQBpAG4AIABhAG4AZAAgAE0AQQBUACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AZQBkAGkAYQBuACAAQQBuAG4AdQBhAGwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAAoAE0AQQBUACkAXAAiACwAIABcACIATQBpAG4AIABNAEEAVABcACIALAAgAFwAIgBNAGEAeAAgAE0AQQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiIAAyADYAIABDAFwAIgAsACAAMgA2ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgAFwAIgAxADUAIAAtACAAMgA1ACAAQwBcACIALAAgADEANQAsACAAMgA1AC4AOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIiAAMQA0ACAAQwBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEANAAuADkAOQA5AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABaAG8AbgBlAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAXAB1ADAAMAAzAGUAIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAXAB1ADAAMAAzAGUAowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABkAG8AZQBzACAAbgBvAHQAIABvAGMAYwB1AHIAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAGQiowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBzACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAWQBlAHMAIAAtACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvACAALQAgAG4AbwB0ACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAZABhAHQAYQAgAHMAYwBvAHIAZQBzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFgAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAdABhACAAcwBvAHUAcgBjAGUAXAAiACwAIABcACIARABhAHQAYQAgAHMAYwBvAHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBuAHQAZQByAG4AYQB0AGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUAIABvAHIAIAByAGUAZwBpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGkAbgB0AGUAbgBzAGkAdAB5ACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIABhAHAAcAByAG8AdgBlAGQAIABtAGUAdABoAG8AZABcACIALAAgADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBlAHIAaQBmAGkAZQBkACAAYwByAGUAZABlAG4AdABpAGEAbAAgAG0AYQB0AGMAaABpAG4AZwAgAEkAUwBPADEANAAwADYANwBcACIALAAgADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAAoADMALgBEAC4AYgAuADIAKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBMAEUAQQBDAEgAXAAiACwAMAAuADIANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABFAHEAdQBhAHQAaQBvAG4AIAAzAC4ARAAuAEIAXwAxADAAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAGwAZQBhAGMAaABcACIALAAwAC4AMAAxADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcAG4ATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADQALAAgADUALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAGoAXAAiACwAXAAiAEUARgBOADIATwBcACIALAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5AFwAIgAsACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAA1ADkALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAXAAiACwAMAAuADAAMAA3ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABsAG8AdwAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAMgA5ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAOAAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAMAAuADAAMQA5ADkALAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsADAALgAwADAANQAzACwAIABcACIAQwBvAHQAdABvAG4AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAMAAuADAAMAA2ADQALAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABjAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnACkAXAAiACwAMAAuADAAMAAzACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBDAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABzAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnACkAXAAiACwAMAAuADAAMAA1ACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBTAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAMAAuADAAMAAyADYALAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABkAHUAcABsAGkAYwBhAHQAZQAgAFwAdQAwADAAMgA3AEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcAHUAMAAwADIANwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcAcAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcAHUAMAAwADIANwAsACAAXAB1ADAAMAAyADcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcAHUAMAAwADIANwAgAGEAbgBkACAAXAB1ADAAMAAyADcAaQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AG4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAdQAwADAAMgA3ACAAcgBvAHcAIAB3AGkAdABoACAAcwBhAG0AZQAgAEUARgAgAGYAbwByACAAbABvAHcAIABhAG4AZAAgAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXABuAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXABuAEkAUABDAEMAOgAgAE4AMgBPACAARQBNAEkAUwBTAEkATwBOAFMAIABGAFIATwBNACAATQBBAE4AQQBHAEUARAAgAFMATwBJAEwAUwAsACAAQQBOAEQAIABDAE8AMgAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAEwASQBNAEUAIABBAE4ARAAgAFUAUgBFAEEAIABBAFAAUABMAEkAQwBBAFQASQBPAE4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAFcARQBUACAAZgBvAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBkAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAQwBoAGEAcAB0AGUAcgAgADEALAAgAHMAZQBjAHQAaQBvAG4AIAAxAC4AOAAuADIAIABMAGUAYQBjAGgAaQBuAGcALAAgAGMAbABpAG0AYQB0AGUAIABhAG4AZAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEkAUABDAEMAIAAyADAAMQA5ACAAUgBlAGYAaQBuAGUAbQBlAG4AdAAgAFYAbwBsAHUAbQBlACAANAA6ACAAQwBoAGEAcAB0AGUAcgAgADEAMQA6ACAATgAyAE8AIABFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABNAGEAbgBhAGcAZQBkACAAUwBvAGkAbABzACwAIABhAG4AZAAgAEMATwAyACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATABpAG0AZQAgAGEAbgBkACAAVQByAGUAYQAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIAB0AHkAcABlACAAaQByAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAaQBwACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBwAHIAaQBuAGsAbABlAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAcgBmAGEAYwBlACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwB0AGgAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABUAGEAYgBsAGUAIABjAHIAZQBhAHQAZQBkACAAYgBhAHMAZQBkACAAbwBuACAAVgBFAEUAUgBHACAAdABlAHgAdAAgAFwAdQAwADAAMgA3AEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuAFwAdQAwADAAMgA3AFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAOgAgAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAFAAUgBQACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAFAAUgBQAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEMAaABhAG4AZwBlAGQAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAB1ADAAMAAyADcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAdQAwADAAMgA3ACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AbwBuAHQAaABzACAAdABvACAAUwBlAGEAcwBvAG4AcwAgAE0AYQBwAHAAaQBuAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAG8AbgB0AGgAXAAiACwAIABcACIAUwBlAGEAcwBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAYQBuAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAZQBiAHIAdQBhAHIAeQBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAHIAYwBoAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHAAcgBpAGwAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQB5AFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbgBlAFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbAB5AFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAZwB1AHMAdABcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAHAAdABlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AYwB0AG8AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB2AGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABlAGMAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAbgB1AHIAZQAgAE0AYQBuAGEAZwBlAG0AZQBuAHQAIAATICAATQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHAAZQByACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGkAbQApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgA4AC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAxACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAIAAoALoAQwApAFwAIgAsACAAXAAiAFUAbgBjAG8AdgBlAHIAZQBkACAAYQBuAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAUwBsAHUAcgByAHkAIAAoAHcAaQB0AGgAbwB1AHQAIABuAGEAdAB1AHIAYQBsACAAYwByAHUAcwB0ACkAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAGIAKQBcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABTAHQAbwByAGEAZwBlACAAXAB1ADAAMAAzAGMAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AFAAbwB1AGwAdAByAHkAIAB3AGkAdABoACAAYQBuAGQAIAB3AGkAdABoAG8AdQB0ACAAbABpAHQAdABlAHIAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHcAaQB0AGgAIABzAGUAcABhAHIAYQB0AGUAIABOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE0AQQBUACAAcgBhAHcAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAbABsAG8AdwAgAGwAbwBvAGsAdQBwACAAbwBmACAAbgB1AG0AYgBlAHIAcwAuAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBuAGQAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAcgBlAHQAdQByAG4AZQBkACAAdABvACAAdABoAGUAIABzAG8AaQBsAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYATgBpACAAXAB1ADAAMAAyADYAIABFAEYATgAyAE8AaQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADEALgA0AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBOAGkAIABcAHUAMAAwADIANgAgAEUARgBOADIATwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAE4AMgBPACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUATgAyAE8AOgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXABuAEcAVwBQAE4AMgBPADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBOADIATwAsACAARwBXAFAAXwBOADIATwAsAFwAbgAgACAAIAAgAEUAXwBOADIATwAgACoAIABHAFcAUABfAE4AMgBPAFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAE4AMgBPACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AE4AMgBPAH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AE4AMgBPAH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBOADIATwBcACIALABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAATgAyAE8AXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAEMASAA0ACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUAQwBIADQAOgAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXABuAEcAVwBQAEMASAA0ADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBDAEgANAAsACAARwBXAFAAXwBDAEgANAAsAFwAbgAgACAAIAAgAEUAXwBDAEgANAAgACoAIABHAFcAUABfAEMASAA0AFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEMASAA0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AEMASAA0AH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AEMASAA0AH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBDAEgANABcACIALABcACIATQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAAQwBIADQAXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQAgAGQAYQB0AGEAIAB0AGgAYQB0ACAAaQBzACAAYwBvAG0AbQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAbABpAHYAZQBzAHQAbwBjAGsAIAB0AHkAcABlAHMAXABuAEUAeABjAGUAbAAgAG0AbwBkAHUAbABlACAAbgBhAG0AZQA6ACAAUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlADoAIABOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcAG4ATgBJAFIAXwAyADAAMgAzAF8AVgBvAGwAMQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBcAG4ARgByAGEAYwBXAEUAVABNAE0AUwBpACAAPQAgAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4AKABUAGEAYgBsAGUAIABBADUALgA1AC4AMQAwAC4AMgAgAGkAcwAgAHIAZQBmAGUAcgBlAG4AYwBlAGQAIABpAG4AIABOAEkAUgAgAGIAdQB0ACAAMQAgAGkAcwAgAHUAcwBlAGQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAxACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXABuAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTACAAPQAgADAALgAwADIAIAAoAEcAZwAgAE4ALwBHAGcAIABhAHAAcABsAGkAZQBkACkAIAAoAEMAUwAgAEUARgAsACAAcwBvAHUAcgBjAGUAIABJAFAAQwBDACAAKAAyADAAMQA5ACkAKQAgAFwAbgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAbABvAHMAdAAgAHQAaAByAG8AdQBnAGgAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABsAG8AcwB0ACAAdABoAHIAbwB1AGcAaAAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA4ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAIAAwAC4AMAAwADUAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwAFwAIgAsACAAMAAuADAAMAA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAgADAALgAwADAAMQA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcABcACIALAAgADAALgAwADAANAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAIABjAGEAbgBlAFwAIgAsACAAMAAuADAAMQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsACAAMAAuADAAMAA1ADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBlAFwAIgAsACAAMAAuADAAMAA2ADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXABuAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVgBhAGkAcgBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE0AUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAAVABhAGIAbABlACAANQAuADEAMgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAOQAsACAAMwAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB5AG0AYgBvAGwAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgAgACgAbQA9ADEAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADIAXAAiACwAIABcACIATABpAHEAdQBpAGQAIABzAHkAcwB0AGUAbQBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwAgACgAbQA9ADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADMAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAG0APQAzACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGEAXAAiACwAIABcACIAUwB1AG0AcAAgAGEAbgBkACAAZABpAHMAcABlAHIAcwBhAGwAIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbAAgAHMAeQBzAHQAZQBtACAAKABtAD0AMwBhACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGIAXAAiACwAIABcACIARAByAGEAaQBuAHMAIAB0AG8AIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAEQAcgBhAGkAbgBzACAAdABvACAAcABhAGQAZABvAGMAawAgACgAbQA9ADMAYgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIANABcACIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAIAAoAG0APQA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA1AFwAIgAsACAAXAAiAEQAcgB5AGwAbwB0ACAAKABmAGUAZQBkACAAcABhAGQAKQBcACIALAAgAFwAIgBEAHIAeQBsAG8AdAAgACgAZgBlAGUAZAAgAHAAYQBkACkAIAAoAG0APQA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA2AFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQAgACgAbQA9ADYAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADcAXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEQAaQBnAGUAcwB0AGUAcgAgAC8AIABjAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AcwAgACgAbQA9ADcAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADgAXAAiACwAIABcACIARABlAGUAcAAgAGwAaQB0AHQAZQByAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgAgACgAbQA9ADgAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADkAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQAgACgAbQA9ADkAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMABcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwAgACgAbQA9ADEAMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnACAAKABtAD0AMQAxACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADEAYQBcACIALAAgAFwAIgBCAGUAbAB0ACAAbQBhAG4AdQByAGUAIAByAGUAbQBvAHYAYQBsAFwAIgAsACAAXAAiAEIAZQBsAHQAIABtAGEAbgB1AHIAZQAgAHIAZQBtAG8AdgBhAGwAIAAoAG0APQAxADEAYQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAGIAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABzAHQAbwByAGUAZAAgAGkAbgAgAGgAbwB1AHMAZQBcACIALAAgAFwAIgBNAGEAbgB1AHIAZQAgAHMAdABvAHIAZQBkACAAaQBuACAAaABvAHUAcwBlACAAKABtAD0AMQAxAGIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAKABtAD0AMQAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADMAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAAoAG0APQAxADMAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEANABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACAAcgBhAG4AZwBlACAAYQBuAGQAIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAIAAoAG0APQAxADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQgBlAGUAZgAgAGMAYQB0AHQAbABlACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBfAFYAYQBpAHIAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAaQBmAGUAYwB5AGMAbABlAHMALgAgACgAMgAwADIANgApAC4AIABHAHIAZQBlAG4AaABvAHUAcwBlACAARwBhAHMAIABFAG0AaQBzAHMAaQBvAG4AIABJAG4AdABlAG4AcwBpAHQAaQBlAHMAIABmAG8AcgAgAE0AYQB0AGUAcgBpAGEAbAAgAEkAbgBwAHUAdABzACAAdABvACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAEEAZwByAGkAYwB1AGwAdAB1AHIAZQAsACAARgBpAHMAaABlAHIAaQBlAHMAIABhAG4AZAAgAEYAbwByAGUAcwB0AHIAeQAuACAAVgBlAHIAcwBpAG8AbgAgADQAOAAuACAAZABvAGkAIAAxADAALgA1ADIAOAAxAC8AegBlAG4AbwBkAG8ALgAxADkANgA1ADYANQA4ADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAXAAiACwAIABcACIAUwBvAHUAcgBjAGUAIAByAGUAZwBpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAYQB0AHQAbABlACwAIABmAG8AcgAgAG0AYQBuAHUAZgBhAGMAdAB1AHIAaQBuAGcAIABiAGUAZQBmAFwAIgAsACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBhAHQAdABsAGUALAAgAGYAbwByACAAcAByAGkAbQBlACAAYgBlAGUAZgBcACIALAAgAFwAIgBOAFMAVwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAYQB0AHQAbABlACwAIAB3AGUAYQBuAGUAcgBzAFwAIgAsACAAXAAiAE4AVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFEATABEAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAVABBAFMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBWAEkAQwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFcAQQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBDAGgAaQBjAGsAZQBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEMAaABpAGMAawBlAG4AcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBoAGkAYwBrAGUAbgBzACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQwBoAGkAYwBrAGUAbgBzAF8AVgBhAGkAcgBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEMAaABpAGMAawBlAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQwBoAGkAYwBrAGUAbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAaQBmAGUAYwB5AGMAbABlAHMALgAgACgAMgAwADIANgApAC4AIABHAHIAZQBlAG4AaABvAHUAcwBlACAARwBhAHMAIABFAG0AaQBzAHMAaQBvAG4AIABJAG4AdABlAG4AcwBpAHQAaQBlAHMAIABmAG8AcgAgAE0AYQB0AGUAcgBpAGEAbAAgAEkAbgBwAHUAdABzACAAdABvACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAEEAZwByAGkAYwB1AGwAdAB1AHIAZQAsACAARgBpAHMAaABlAHIAaQBlAHMAIABhAG4AZAAgAEYAbwByAGUAcwB0AHIAeQAuACAAVgBlAHIAcwBpAG8AbgAgADQAOAAuACAAZABvAGkAIAAxADAALgA1ADIAOAAxAC8AegBlAG4AbwBkAG8ALgAxADkANgA1ADYANQA4ADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBDAGgAaQBjAGsAZQBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUAByAG8AZAB1AGMAdABcACIALAAgAFwAIgBTAG8AdQByAGMAZQAgAHIAZQBnAGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBoAGkAYwBrAGUAbgBzAFwAIgAsACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEQAYQBpAHIAeQBjAGEAdAB0AGwAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIABwAHIAbwBkAHUAYwB0AHMAIABmAG8AcgAgAHMAYwBvAHAAZQAgADMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXwBWAGEAaQByAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8ARABhAGkAcgB5AGMAYQB0AHQAbABlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATABpAGYAZQBjAHkAYwBsAGUAcwAuACAAKAAyADAAMgA2ACkALgAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABHAGEAcwAgAEUAbQBpAHMAcwBpAG8AbgAgAEkAbgB0AGUAbgBzAGkAdABpAGUAcwAgAGYAbwByACAATQBhAHQAZQByAGkAYQBsACAASQBuAHAAdQB0AHMAIAB0AG8AIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAQQBnAHIAaQBjAHUAbAB0AHUAcgBlACwAIABGAGkAcwBoAGUAcgBpAGUAcwAgAGEAbgBkACAARgBvAHIAZQBzAHQAcgB5AC4AIABWAGUAcgBzAGkAbwBuACAANAA4AC4AIABkAG8AaQAgADEAMAAuADUAMgA4ADEALwB6AGUAbgBvAGQAbwAuADEAOQA2ADUANgA1ADgAMABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEQAYQBpAHIAeQBjAGEAdAB0AGwAZQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AFwAIgAsACAAXAAiAFMAbwB1AHIAYwBlACAAcgBlAGcAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAaQByAHkAIABjAG8AdwBzAFwAIgAsACAAXAAiAFYASQBDAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBQAGkAZwBzACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUABpAGcAcwBfAFYAYQBpAHIAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAaQBmAGUAYwB5AGMAbABlAHMALgAgACgAMgAwADIANgApAC4AIABHAHIAZQBlAG4AaABvAHUAcwBlACAARwBhAHMAIABFAG0AaQBzAHMAaQBvAG4AIABJAG4AdABlAG4AcwBpAHQAaQBlAHMAIABmAG8AcgAgAE0AYQB0AGUAcgBpAGEAbAAgAEkAbgBwAHUAdABzACAAdABvACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAEEAZwByAGkAYwB1AGwAdAB1AHIAZQAsACAARgBpAHMAaABlAHIAaQBlAHMAIABhAG4AZAAgAEYAbwByAGUAcwB0AHIAeQAuACAAVgBlAHIAcwBpAG8AbgAgADQAOAAuACAAZABvAGkAIAAxADAALgA1ADIAOAAxAC8AegBlAG4AbwBkAG8ALgAxADkANgA1ADYANQA4ADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAXAAiACwAIABcACIAUwBvAHUAcgBjAGUAIAByAGUAZwBpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAaQBnAHMAXAAiACwAIABcACIAQQB1AHMAdAByAGEAbABpAGEAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUwBoAGUAZQBwAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBTAGgAZQBlAHAAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFMAaABlAGUAcAAgAHAAcgBvAGQAdQBjAHQAcwAgAGYAbwByACAAcwBjAG8AcABlACAAMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFMAaABlAGUAcABfAFYAYQBpAHIAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBTAGgAZQBlAHAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFMAaABlAGUAcABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBMAGkAZgBlAGMAeQBjAGwAZQBzAC4AIAAoADIAMAAyADYAKQAuACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAEcAYQBzACAARQBtAGkAcwBzAGkAbwBuACAASQBuAHQAZQBuAHMAaQB0AGkAZQBzACAAZgBvAHIAIABNAGEAdABlAHIAaQBhAGwAIABJAG4AcAB1AHQAcwAgAHQAbwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABBAGcAcgBpAGMAdQBsAHQAdQByAGUALAAgAEYAaQBzAGgAZQByAGkAZQBzACAAYQBuAGQAIABGAG8AcgBlAHMAdAByAHkALgAgAFYAZQByAHMAaQBvAG4AIAA0ADgALgAgAGQAbwBpACAAMQAwAC4ANQAyADgAMQAvAHoAZQBuAG8AZABvAC4AMQA5ADYANQA2ADUAOAAwAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUwBoAGUAZQBwAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAXAAiACwAIABcACIAUwBvAHUAcgBjAGUAIAByAGUAZwBpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAaABlAGUAcAAsACAAZgBvAHIAIABtAHUAdAB0AG8AbgBcACIALAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAaABlAGUAcAAsACAAZgBvAHIAIABwAHIAaQBtAGUAIABsAGEAbQBiAFwAIgAsACAAXAAiAE4AUwBXAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAUQBMAEQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBTAEEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFYASQBDAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAVwBBAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFIATwBXACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwAKQAgACsAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACAALQAgADEAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAVABhAGIAbABlAEgAZQBhAGQAZQByAEMAZQBsAGwALABcAG4AIAAgAEMATwBMAFUATQBOACgAVABhAGIAbABlAEgAZQBhAGQAZQByAEMAZQBsAGwAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAHIAYQB5AEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIABBAHIAcgBhAHkARABhAHQAYQAsACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkALAAgAFsAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQBdACwAXABuACAASQBGAEUAUgBSAE8AUgAoAFwAbgAgACAAIAAgACAASQBOAEQARQBYACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFUATgBJAFEAVQBFACgAQQByAHIAYQB5AEQAYQB0AGEAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIATwBXACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABDAE8ATABVAE0ATgAoACkALQBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5ACkALAAgADEALAAgAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALAAgAFwAIgBcACIAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABJAEYAKABJAFMATgBVAE0AQgBFAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkAXABuACAAIAAgACAAKQAsACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQAsACAAMAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAVAB3AG8AQwBvAGwAdQBtAG4AcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkARgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIAAoAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlADEAKQAqACgATABvAG8AawB1AHAAQQByAHIAYQB5ADIAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgApACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAVgBhAGwAdQBlAEkARgBGAGEAbABzAGUAKQAsACAAXAAiAFwAIgAsACAAVgBhAGwAdQBlAEkARgBGAGEAbABzAGUAKQApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATwBuAGUAQwBvAGwAdQBtAG4AQQBuAGQASABlAGEAZABlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABbAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlAF0ALABcAG4AIAAgACAAIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBmAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBmAEYAYQBsAHMAZQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHAAbABpAHQAUwB0AHIAaQBuAGcASQBuAHQAbwBBAHIAcgBhAHkAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABDAGUAbABsACwAIABEAGUAbABpAG0AaQB0AGUAcgAsACAAWwBDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQBdACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyAF0ALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSAFgATQBMACgAXABuACAAIAAgACAAIAAgACAAIABcACIAXAB1ADAAMAAzAGMAdABcAHUAMAAwADMAZQBcAHUAMAAwADMAYwBzAFwAdQAwADAAMwBlAFwAIgAgAFwAdQAwADAAMgA2AFwAbgAgACAAIAAgACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAUwBVAEIAUwBUAEkAVABVAFQARQAoAEMAZQBsAGwALABDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQAsAFwAIgBcACIAKQAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEQAZQBsAGkAbQBpAHQAZQByACwAXAAiAFwAdQAwADAAMwBjAC8AcwBcAHUAMAAwADMAZQBcAHUAMAAwADMAYwBzAFwAdQAwADAAMwBlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgACkAIABcAHUAMAAwADIANgBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcAHUAMAAwADMAYwAvAHMAXAB1ADAAMAAzAGUAXAB1ADAAMAAzAGMALwB0AFwAdQAwADAAMwBlAFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAC8ALwBzAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAYQB2AGcAVABlAG0AcAAsAGEAdgBnAFIAYQBpAG4ALABmAHIAbwBzAHQARABhAHkAcwAsAGUAbABlAHYALABtAGEAcABfAHAAZQB0ACwAXABuACAAIAAgACAAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkALABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQAsAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABtAGEAeABFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBQAEUAVABBAHIAcgBhAHkALABtAGEAeABQAEUAVABBAHIAcgBhAHkALABcAG4AIAAgACAAIABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AGEAdgBnAFQAZQBtAHAAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBhAHYAZwBSAGEAaQBuACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AZgByAG8AcwB0AEQAYQB5AHMAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABGAHIAbwBzAHQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AZQBsAGUAdgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AZQBsAGUAdgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAFAARQBUAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AbQBhAHAAXwBwAGUAdAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFAARQBUAEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AbQBhAHAAXwBwAGUAdAApACwAXABuACAAIAAgACAAIAAgACAAIABUAEEASwBFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgAYwBsAGkAbQBhAHQAZQBaAG8AbgBlAEEAcgByAGEAeQAsAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAMQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAEkAdABlAG0ARgByAG8AbQBNAGkAbgBNAGEAeABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATQBpAG4AQQByAHIAYQB5ACwAIABNAGEAeABBAHIAcgBhAHkALAAgAEkAdABlAG0AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBpAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGEAeABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACwAXABuACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgAoAEkAdABlAG0AQQByAHIAYQB5ACwAIABtAGEAcwBrACwAIABcACIATgBvACAAbQBhAHQAYwBoAFwAIgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABDAHIAaQB0AGUAcgBpAGEAMQAsACAAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkALAAgAFEAdQBhAG4AdABpAHQAeQAsACAAWwBNAHUAbAB0AGkAcABsAGkAZQByAF0ALAAgAFsAQwByAGkAdABlAHIAaQBhADIAXQAsAFsAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AF0ALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAbQB1AGwAdABpAHAAbABpAGUAcgAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABNAHUAbAB0AGkAcABsAGkAZQByACkALAAxACwATQB1AGwAdABpAHAAbABpAGUAcgApACwAXABuACAAIAAgACAAcQB1AGEAbgB0AGkAdAB5ACwAIABRAHUAYQBuAHQAaQB0AHkAKgBNAHUAbAB0AGkAcABsAGkAZQByACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAxACkALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMgAsAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwByAGkAdABlAHIAaQBhADIAKQAsADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMgApACkALABcAG4AIAAgACAAIABTAFUATQBQAFIATwBEAFUAQwBUACgAYwByAGkAdABlAHIAaQBhADEAKgBjAHIAaQB0AGUAcgBpAGEAMgAqAHEAdQBhAG4AdABpAHQAeQApAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAXAB1ADAAMAAzAGMAIABTACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAXAB1ADAAMAAzAGUAIABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAE0AQQBYACgAMAAsAGwAYQBzAHQAWQBlAGEAcgAtAGYAaQByAHMAdABZAGUAYQByACsAMQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBQAGUAcgBpAG8AZABzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAIAAvACoAaABlAGwAcABlAHIAOgAgAGUAbgBkACAAZABhAHQAZQAgAGYAbwByACAAYQAgAHIAZQBwAG8AcgB0AGkAbgBnACAAcABlAHIAaQBvAGQAIABzAHQAYQByAHQAaQBuAGcAIABhAHQAIABhACAAZwBpAHYAZQBuACAAZABhAHQAZQAqAC8AXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALAAgAC8AKgBvAG4AbAB5ACAAbgBlAGUAZAAgAHQAbwAgAGwAbwBvAGsAIABiAGEAYwBrACAAMwA2ADUAIABkAGEAeQBzACgAbQBhAHgAIABvAHYAZQByAGwAYQBwACAAdwBpAG4AZABvAHcAKQAqAC8AXABuACAAIAAgACAAIAAgACAAIABBACwAUwAtADMANgA1ACwAXABuACAAIAAgACAAIAAgACAAIAB5AGEALABZAEUAQQBSACgAQQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AGIALABZAEUAQQBSACgARQApACwAIAAvACoAaQBmACAAdABoAGUAIABhAG4AYwBoAG8AcgAgAGYAbwByACAAeQBhACAAZQBuAGQAcwAgAGIAZQBmAG8AcgBlACAAUwAsAGkAdAAgAGMAYQBuAFwAdQAwADAAMgA3AHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAbgBlAHgAdAAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQBcAHUAMAAwADMAYwBTACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGIAIABzAHQAYQByAHQAcwAgAGEAZgB0AGUAcgAgAEUALABpAHQAIABjAGEAbgBcAHUAMAAwADIANwB0ACAAbwB2AGUAcgBsAGEAcAA7ACAAbQBvAHYAZQAgAHQAbwAgAHAAcgBlAHYAaQBvAHUAcwAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQBcAHUAMAAwADMAZQBFACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4ALABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQByAHMALABTAEUAUQBVAEUATgBDAEUAKABuACwAMQAsAGYAaQByAHMAdABZAGUAYQByACwAMQApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwAsAEQAQQBUAEUAKAB5AHIAcwAsAG0ALABkACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMALABNAEEAUAAoAHMAdABhAHIAdABzACwAUABlAHIAaQBvAGQARQBuAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAdABhAGcALABJAEYAKABzAHQAYQByAHQAcwA9AFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcACIAIAAoAFQAaABpAHMAIAByAGUAcABvAHIAdABpAG4AZwAgAGMAeQBjAGwAZQApAFwAIgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMAVABlAHgAdAAsAFQARQBYAFQAKABzAHQAYQByAHQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMAVABlAHgAdAAsAFQARQBYAFQAKABlAG4AZABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAbgA9ADAALABcACIAXAAiACwASABTAFQAQQBDAEsAKABzAHQAYQByAHQAcwBUAGUAeAB0ACAAXAB1ADAAMAAyADYAIABcACIAIAB0AG8AIABcACIAIABcAHUAMAAwADIANgAgAGUAbgBkAHMAVABlAHgAdAAgAFwAdQAwADAAMgA2ACAAdABhAGcAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlAFwAbgA9AEwAQQBNAEIARABBACgARgB1AG4AYwB0AGkAbwBuACwAIABUAEUAWABUAEIARQBGAE8AUgBFACgARgBPAFIATQBVAEwAQQBUAEUAWABUACgARgB1AG4AYwB0AGkAbwBuACkALAAgAFwAIgAoAFwAIgApACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZABBAHIAcgBhAHkALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQAsAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABJAEYAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAD0AXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBBAG4AeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAIAA9ACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgAMQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBBAHIAcgBhAHkAPQBQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQA9AEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQA9AFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAgACsAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQAXAB1ADAAMAAzAGUAMAAsACAAMQAsACAAMAApAFwAbgAgACAAIAAgACkAKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBDAG8AbgB2AGUAcgB0AFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAFQAbwBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlACwAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAQQByAHIAYQB5ACwAIABTAHQAYQB0AGUAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlACwAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAFwAbgA9AEwAQQBNAEIARABBACgAVABhAHIAZwBlAHQAQwBlAGwAbAAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABzAGgALAAgAFQARQBYAFQAQQBGAFQARQBSACgAQwBFAEwATAAoAFwAIgBmAGkAbABlAG4AYQBtAGUAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALAAgAFwAIgBdAFwAIgApACwAXABuACAAIAAgACAAYQBkAGQAcgAsACAAQwBFAEwATAAoAFwAIgBhAGQAZAByAGUAcwBzAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAXABuACAAIAAgACAAXAAiACMAXAB1ADAAMAAyADcAXAAiACAAXAB1ADAAMAAyADYAIABzAGgAIABcAHUAMAAwADIANgAgAFwAIgBcAHUAMAAwADIANwAhAFwAIgAgAFwAdQAwADAAMgA2ACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawBEAGkAZgBmAGUAcgBlAG4AdABTAGgAZQBlAHQAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwBcACIAIABcAHUAMAAwADIANgAgAGEAZABkAHIAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADEAXwAyAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAXABuACAAIAAgACAAQwBIAE8ATwBTAEUAQwBPAEwAUwAoAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsACAAMQAsACAAMgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADMAXwA0AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAXABuACAAIAAgACAAQwBIAE8ATwBTAEUAQwBPAEwAUwAoAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsACAAMwAsACAANAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEcAZQB0AE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACwAIABNAE0AUwAsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAXABuACAAIAAgACAAIAAgACAAIABNAEUARABJAEEATgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAE8AVQBOAEQAKABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgADAAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAE0ASQBOACgAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBBAFgAKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATQBNAFMALAAgAE0ATQBTAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBSAGUAcwB1AGwAdABzAEkAdABlAG0ARgByAG8AbQBFAHEAdQBhAHQAaQBvAG4AVABpAHQAbABlAEEAbgBkAFMAbwB1AHIAYwBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABpAHQAbABlAEMAZQBsAGwALAAgAFMAbwB1AHIAYwBlAEMAZQBsAGwALABcAG4AIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgATABFAEYAVAAoAFMAbwB1AHIAYwBlAEMAZQBsAGwALAAgAEYASQBOAEQAKABcACIALABcACIALAAgAFMAbwB1AHIAYwBlAEMAZQBsAGwAKQAgAC0AMQApACwAIABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAXAAiACwAIABcACIAXAAiACkAIABcAHUAMAAwADIANgAgAFwAIgAgAFwAIgAgAFwAdQAwADAAMgA2ACAAVABpAHQAbABlAEMAZQBsAGwAXABuACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAgACsAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQAXAB1ADAAMAAzAGUAMAAsACAAMQAsACAAMAApAFwAbgAgACAAIAAgACkAKQA7AFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEMAYQBsAGMAdQBsAGEAdABlAEgAYQByAHYAZQBzAHQASQBuAGQAZQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQwByAG8AcABUAHkAcABlACwAIABDAHIAbwBwAFQAeQBwAGUAQQByAHIAYQB5ACwAIABSAGUAcwBpAGQAdQBlAEMAcgBvAHAAUgBhAHQAaQBvAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgADEALwAoADEAKwBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAEMAcgBvAHAAVAB5AHAAZQAsACAAQwByAG8AcABUAHkAcABlAEEAcgByAGEAeQAsACAAUgBlAHMAaQBkAHUAZQBDAHIAbwBwAFIAYQB0AGkAbwBBAHIAcgBhAHkAKQApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBSAGUAcwBpAGQAdQBlAEMAcgBvAHAAUgBhAHQAaQBvAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAASABhAHIAdgBlAHMAdABJAG4AZABlAHgALABcAG4AIAAgACAAIAAoADEALQBIAGEAcgB2AGUAcwB0AEkAbgBkAGUAeAApAC8ASABhAHIAdgBlAHMAdABJAG4AZABlAHgAXABuACkAOwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBGAHIAYQBjAHQAaQBvAG4AUgBlAHMAaQBkAHUAZQBSAGUAbQBvAHYAZQBkAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABvAHQAYQBsAFIAZQBzAGkAZAB1AGUALAAgAEEAbQBvAHUAbgB0AFIAZQBtAG8AdgBlAGQALABcAG4AIAAgACAAIAAoAEEAbQBvAHUAbgB0AFIAZQBtAG8AdgBlAGQAKgAxADAAXgAzACkALwAoAFQAbwB0AGEAbABSAGUAcwBpAGQAdQBlACoAMQAwAF4AMwApAFwAbgApACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAIABkAGEAdABhACAARgBvAHIAIABTAHcAaQBuAGUAXABuAEUAeABjAGUAbAAgAG0AbwBkAHUAbABlACAAbgBhAG0AZQA6ACAAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAXABuAFYAUwBqAFwAbgBrAGcALwBoAGUAYQBkAC8AZABhAHkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAUwB3AGkAbgBlACAALQAgAFYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZABzACAAKABWAFMAagApACAALQAgADIAMAAyADAAIAB0AG8AIAAyADAAMgA0AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnAC8AaABlAGEAZAAvAGQAYQB5AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4ANgAuADEAOgAgAFMAdwBpAG4AZQAgAC0AIABJAG4AdABhAGsAZQAgAGEAbgBkACAAbQBhAG4AdQByAGUAIABjAGgAYQByAGEAYwB0AGUAcgBpAHMAdABpAGMAcwAgAGQAZQByAGkAdgBlAGQAIABmAHIAbwBtACAAUABpAGcAQgBhAGwAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAE8AbgBsAHkAIAB1AHMAZQBzACAAZABhAHQAYQAgAGYAbwByACAAMgAwADIAMAAtADIAMAAyADQALgAgAFUAcwBlACAAXAB1ADAAMAAyADcAUwBsAGEAdQBnAGgAdABlAHIAIABwAGkAZwBzAFwAdQAwADAAMgA3ACAAZABhAHQAYQAgAGYAbwByACAAXAB1ADAAMAAyADcATwB0AGgAZQByACAAagA9ADQAXAB1ADAAMAAyADcAIABjAGwAYQBzAHMALgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAYQBzAHMAXAAiACwAIABcACIAVgBTAGoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAbwBhAHIAcwBcACIALAAgADAALgA0ADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHcAcwBcACIALAAgADAALgA0ADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBpAGwAdABzAFwAIgAsACAAMAAuADUANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAHQAaABlAHIAcwBcACIALAAgADAALgAzADkAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ARgBlAGUAZABJAG4AdABhAGsAZQBcAG4ASQBqAFwAbgBrAGcALwBoAGUAYQBkAC8AZABhAHkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFMAdwBpAG4AZQAgAC0AIABGAGUAZQBkACAAaQBuAHQAYQBrAGUAIAAtACAAaQBuAGcAZQBzAHQAZQBkACAAYQBzACAAZgBlAGQAIAAgACgASQBqACkAIAAtACAAMgAwADIAMAAgAHQAbwAgADIAMAAyADQAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBGAGUAZQBkAEkAbgB0AGEAawBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnAC8AaABlAGEAZAAvAGQAYQB5AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ARgBlAGUAZABJAG4AdABhAGsAZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADYALgAxADoAIABTAHcAaQBuAGUAIAAtACAASQBuAHQAYQBrAGUAIABhAG4AZAAgAG0AYQBuAHUAcgBlACAAYwBoAGEAcgBhAGMAdABlAHIAaQBzAHQAaQBjAHMAIABkAGUAcgBpAHYAZQBkACAAZgByAG8AbQAgAFAAaQBnAEIAYQBsAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ARgBlAGUAZABJAG4AdABhAGsAZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAATwBuAGwAeQAgAHUAcwBlAHMAIABkAGEAdABhACAAZgBvAHIAIAAyADAAMgAwAC0AMgAwADIANAAuACAAVQBzAGUAIABcAHUAMAAwADIANwBTAGwAYQB1AGcAaAB0AGUAcgAgAHAAaQBnAHMAXAB1ADAAMAAyADcAIABkAGEAdABhACAAZgBvAHIAIABcAHUAMAAwADIANwBPAHQAaABlAHIAIABqAD0ANABcAHUAMAAwADIANwAgAGMAbABhAHMAcwAuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ARgBlAGUAZABJAG4AdABhAGsAZQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAYQBzAHMAXAAiACwAIABcACIASQBqAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBCAG8AYQByAHMAXAAiACwAIAAyAC4ANgAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAbwB3AHMAXAAiACwAMgAuADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAGkAbAB0AHMAXAAiACwAIAAyAC4ANQAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AdABoAGUAcgBzAFwAIgAsACAAMQAuADcAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE4AaQB0AHIAbwBnAGUAbgBJAG4AVwBhAHMAdABlAFwAbgBOAFcAagBcAG4AawBnAC8AaABlAGEAZAAvAGQAYQB5AFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBOAGkAdAByAG8AZwBlAG4ASQBuAFcAYQBzAHQAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAUwB3AGkAbgBlACAALQAgAE4AaQB0AHIAbwBnAGUAbgAgAGkAbgAgAHcAYQBzAHQAZQAgACgATgBXAGoAKQAgAC0AIAAyADAAMgAwACAAdABvACAAMgAwADIANABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE4AaQB0AHIAbwBnAGUAbgBJAG4AVwBhAHMAdABlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnAC8AaABlAGEAZAAvAGQAYQB5AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATgBpAHQAcgBvAGcAZQBuAEkAbgBXAGEAcwB0AGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgA2AC4AMQA6ACAAUwB3AGkAbgBlACAALQAgAEkAbgB0AGEAawBlACAAYQBuAGQAIABtAGEAbgB1AHIAZQAgAGMAaABhAHIAYQBjAHQAZQByAGkAcwB0AGkAYwBzACAAZABlAHIAaQB2AGUAZAAgAGYAcgBvAG0AIABQAGkAZwBCAGEAbABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE4AaQB0AHIAbwBnAGUAbgBJAG4AVwBhAHMAdABlAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBOACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABPAG4AbAB5ACAAdQBzAGUAcwAgAGQAYQB0AGEAIABmAG8AcgAgADIAMAAyADAALQAyADAAMgA0AC4AIABVAHMAZQAgAFwAdQAwADAAMgA3AFMAbABhAHUAZwBoAHQAZQByACAAcABpAGcAcwBcAHUAMAAwADIANwAgAGQAYQB0AGEAIABmAG8AcgAgAFwAdQAwADAAMgA3AE8AdABoAGUAcgAgAGoAPQA0AFwAdQAwADAAMgA3ACAAYwBsAGEAcwBzAC4AIABBAGQAZABlAGQAIABcAHUAMAAwADIANwBOAFcAagAgAGQAYQBpAGwAeQBcAHUAMAAwADIANwAgAGMAbwBsAHUAbQBuACAAdABvACAAcAByAG8AdgBpAGQAZQAgAGQAYQBpAGwAeQAgAHYAYQBsAHUAZQAgAGYAbwByACAATwB0AGgAZQByAHMAIABjAGwAYQBzAHMALgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AEMAbABhAHMAcwAgAG4AYQBtAGUAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE4AaQB0AHIAbwBnAGUAbgBJAG4AVwBhAHMAdABlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADQALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABhAHMAcwBcACIALAAgAFwAIgBOAFcAagBcACIALAAgAFwAIgBOAFcAagAgAGQAYQBpAGwAeQBcACIALAAgAFwAIgBDAGwAYQBzAHMAIABuAGEAbQBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBCAG8AYQByAHMAXAAiACwAIAAwAC4AMAA0ADYALAAgADAALgAwADQANgAsACAAXAAiAEIAbwBhAHIAcwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHcAcwBcACIALAAwAC4AMAA0ADkALAAgADAALgAwADQAOQAsACAAXAAiAFMAbwB3AHMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAaQBsAHQAcwBcACIALAAgADAALgAwADQANgAsACAAMAAuADAANAA2ACwAIABcACIARwBpAGwAdABzAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAHQAaABlAHIAcwAgACgAawBnAC8AaABlAGEAZAAvAHkAZQBhAHIAKQBcACIALAAgADEAMQAuADQALAAgADAALgAwADMAMQAyACwAIABcACIATwB0AGgAZQByAHMAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAEYAcgBhAGMAdABpAG8AbgBOAFYAbwBsAGEAdABpAGwAaQBzAGUAZABcAG4ARgByAGEAYwBHAEEAUwBNAG0AVABcAG4AKABrAGcAIABOAEgAMwAtAE4AIAArACAATgBPAHgALQBOACkALwBrAGcATgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ARgByAGEAYwB0AGkAbwBuAE4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBTAHcAaQBuAGUAIAAtACAARgByAGEAYwB0AGkAbwBuACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAdgBvAGwAYQB0AGkAbABpAHMAZQBkACAAKABGAHIAYQBjAEcAQQBTAE0AbQBUACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBGAHIAYQBjAHQAaQBvAG4ATgBWAG8AbABhAHQAaQBsAGkAcwBlAGQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4ASAAzAC0ATgAgACsAIABOAE8AeAAtAE4AKQAvAGsAZwBOAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ARgByAGEAYwB0AGkAbwBuAE4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4ANgAuADIAOgAgAFMAdwBpAG4AZQAgAC0AIABGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdgBvAGwAYQB0AGkAbABpAHMAZQBkACAAYgB5ACAATQBNAFMAIAAoACgAawBnACAATgBIADMALQBOACAAKwAgAE4ATwB4AC0ATgApAC8AawBnAE4AKQAgACgARgByAGEAYwBHAEEAUwBNAG0AVAApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ARgByAGEAYwB0AGkAbwBuAE4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBOACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABcAHUAMAAwADIANwBOAEkAUgAgAHIAZQBmAGUAcgBlAG4AYwBlACAAYwBvAGwAdQBtAG4AIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBGAHIAYQBjAHQAaQBvAG4ATgBWAG8AbABhAHQAaQBsAGkAcwBlAGQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANwAsACAAMwAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBNAFMAbQBcACIALAAgAFwAIgBGAHIAYQBjAEcAQQBTAE0AbQBUAFwAIgAsACAAXAAiAE4ASQBSACAAcgBlAGYAZQByAGUAbgBjAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AdQB0AGQAbwBvAHIAIAAoAEQAcgB5ACAAbABvAHQAKQBcACIALAAgADAALgAzACwAIABcACIARAByAHkAbABvAHQAIAAoAGYAZQBlAGQAIABwAGEAZAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGUAZQBwACAAbABpAHQAdABlAHIAXAAiACwAIAAwAC4AMQAyADUALAAgAFwAIgBEAGUAZQBwACAAbABpAHQAdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABvAGMAawBwAGkAbABlACAAKABTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlACkAXAAiACwAIAAwAC4AMgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAZgBmAGwAdQBlAG4AdAAgAHAAbwBuAGQAIAAoAFUAbgBjAG8AdgBlAHIAZQBkACAAYQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgApAFwAIgAsACAAMAAuADUANQAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAZABpAGcAZQBzAHQAZQByACAALwAgAEMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBcACIALAAgADAALAAgAFwAIgBEAGkAZwBlAHMAdABlAHIAIAAvACAAYwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAHMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAaABvAHIAdAAgAEgAUgBUACAAdABhAG4AawAgAHMAdABvAHIAYQBnAGUAIABcAHUAMAAwADMAYwAgADEAIABtAG8AbgB0AGgAIAAoAHAAaQB0ACAAcwB0AG8AcgBhAGcAZQApAFwAIgAsACAAMAAuADIANQAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXABuAEYAcgBhAGMARwBBAFMATQBtAFQAXABuAGsAZwBOADIATwAgAC0AIABOACAALwAgAGsAZwBOAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAUwB3AGkAbgBlACAALQAgAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABFAEYAcwAgAGIAeQAgAE0ATQBTACAAKABFAEYAbQBUACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwBOADIATwAgAC0AIABOACAALwAgAGsAZwBOAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgA2AC4AMwA6ACAAUwB3AGkAbgBlACAALQAgAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABFAEYAcwAgAGIAeQAgAE0ATQBTACAAKABrAGcATgAyAE8ALQBOAC8AawBnAE4AKQAgACgARQBGAG0AVAApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE4ASQBSACAAcgBlAGYAZQByAGUAbgBjAGUAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADcALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0ATQBTAG0AXAAiACwAIABcACIARQBGAG0AVABcACIALAAgAFwAIgBOAEkAUgAgAHIAZQBmAGUAcgBlAG4AYwBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAHUAdABkAG8AbwByACAAKABEAHIAeQAgAGwAbwB0ACkAXAAiACwAIAAwAC4AMAAyACwAIABcACIARAByAHkAbABvAHQAIAAoAGYAZQBlAGQAIABwAGEAZAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGUAZQBwACAAbABpAHQAdABlAHIAXAAiACwAIAAwAC4AMAAxACwAIABcACIARABlAGUAcAAgAGwAaQB0AHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAbwBjAGsAcABpAGwAZQAgACgAUwBvAGwAaQBkACAAcwB0AG8AcgBhAGcAZQApAFwAIgAsACAAMAAuADAAMAA1ACwAIABcACIAUwBvAGwAaQBkACAAcwB0AG8AcgBhAGcAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBmAGYAbAB1AGUAbgB0ACAAcABvAG4AZAAgACgAVQBuAGMAbwB2AGUAcgBlAGQAIABhAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuACkAXAAiACwAIAAwACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABkAGkAZwBlAHMAdABvAHIAIAAvACAAQwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAFwAIgAsACAAMAAsACAAXAAiAEQAaQBnAGUAcwB0AGUAcgAgAC8AIABjAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AcwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBoAG8AcgB0ACAASABSAFQAIAB0AGEAbgBrACAAcwB0AG8AcgBhAGcAZQAgAFwAdQAwADAAMwBjACAAMQAgAG0AbwBuAHQAaAAgACgAcABpAHQAIABzAHQAbwByAGEAZwBlACkAXAAiACwAIAAwAC4AMAAwADIALAAgAFwAIgBQAGkAdAAgAHMAdABvAHIAYQBnAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAFwAbgBCADAAXABuAG0AMwAgAEMASAA0AC8AawBnACAAVgBTAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuAHMAIABwAG8AdABlAG4AdABpAGEAbAAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAIABwAGUAcgAgAGsAaQBsAG8AZwByAGEAbQAgAG8AZgAgAHYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZABzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEIAMABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAbQAzACAAQwBIADQAIAAvACAAawBnACAAVgBTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIASQBQAEMAQwAgACgAMgAwADEAOQApACwAIABDAGgAYQBwAHQAZQByACAAMQAwACAAWwA0AF0AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMQA5ACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATQBNAFMAXwBNAEMARgBzAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADYALgA0ADoAIABTAHcAaQBuAGUAIAAtACAATQBDAEYAcwAgACgATQBDAEYAaQBtACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE0ATQBTAF8ATQBDAEYAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQAgAGEAbgBkACAAbQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAcwB5AHMAdABlAG0ALgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE0ATQBTAF8ATQBDAEYAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATQBNAFMAXwBNAEMARgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4ANgAuADQAOgAgAFMAdwBpAG4AZQAgAC0AIABNAEMARgBzACAAKABNAEMARgBpAG0AKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE0ATQBTAF8ATQBDAEYAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQQBkAGQAZQBkACAAYwBvAGwAdQBtAG4AcwAgAGYAbwByACAAQQBDAFQALAAgAHMAcABsAGkAdAAgAFEATABEACAAYQBuAGQAIABOAFQALgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAGMAbwBsAHUAbQBuACAAdwBpAHQAaAAgAE0ATQBTACAAbgBhAG0AZQBzACAAdABoAGEAdAAgAG0AYQB0AGMAaAAgAE4ASQBSACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATQBNAFMAXwBNAEMARgBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADEAMAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBNAFMAXAAiACwAIABcACIATgBTAFcAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAUQBMAEQAXAAiACwAIABcACIATgBUAFwAIgAsACAAXAAiAFMAQQBcACIALAAgAFwAIgBUAEEAUwBcACIALAAgAFwAIgBWAEkAQwBcACIALAAgAFwAIgBXAEEAXAAiACwAIABcACIATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAHUAdABkAG8AbwByACAAKABEAHIAeQAgAGwAbwB0ACkAXAAiACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIAAwAC4AMAAzACwAIAAwAC4AMAAzACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIABcACIARAByAHkAbABvAHQAIAAoAGYAZQBlAGQAIABwAGEAZAApAFwAIgA7ACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgADAALgAwADQALAAgADAALgAwADQALAAgADAALgAwADQALAAgADAALgAwADQALAAgADAALgAwADQALAAgADAALgAwADQALAAgADAALgAwADQALAAgADAALgAwADQALAAgAFwAIgBEAGUAZQBwACAAbABpAHQAdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABvAGMAawBwAGkAbABlACAAKABTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlACkAXAAiACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIABcACIAUwBvAGwAaQBkACAAcwB0AG8AcgBhAGcAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBmAGYAbAB1AGUAbgB0ACAAcABvAG4AZAAgACgAVQBuAGMAbwB2AGUAcgBlAGQAIABhAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuACkAXAAiACwAIAAwAC4ANwA1ACwAIAAwAC4ANwA1ACwAIAAwAC4ANwA4ACwAIAAwAC4ANwA4ACwAIAAwAC4ANwA1ACwAIAAwAC4ANwAwACwAIAAwAC4ANwA0ACwAIAAwAC4ANwA2ACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABkAGkAZwBlAHMAdABlAHIAIAAvACAAQwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAFwAIgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMQAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMQAsACAAMAAuADEALAAgADAALgAxACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgA7ACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAaABvAHIAdAAgAEgAUgBUACAAdABhAG4AawAgAHMAdABvAHIAYQBnAGUAIABcAHUAMAAwADMAYwAgADEAIABtAG8AbgB0AGgAIAAoAHAAaQB0ACAAcwB0AG8AcgBhAGcAZQApAFwAIgAsACAAMAAuADAAMwAsACAAMAAuADAAMwAsACAAMAAuADAAMwAsACAAMAAuADAAMwAsACAAMAAuADAAMwAsACAAMAAuADAAMwAsACAAMAAuADAAMwAsACAAMAAuADAAMwAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQBcACIAOwAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGkAcgBlAGMAdAAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgAgAHQAbwAgAHMAbwBpAGwAXAAiACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAEEAdgBlAHIAYQBnAGUATABpAHYAZQB3AGUAaQBnAGgAdABcAG4AVwBjAG8AXABuAGsAZwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8AQQB2AGUAcgBhAGcAZQBMAGkAdgBlAHcAZQBpAGcAaAB0AF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBTAHcAaQBuAGUAIAAtACAAQQB2AGUAcgBhAGcAZQAgAGwAaQB2AGUAdwBlAGkAZwBoAHQAIAAoAGkAbgB2AGUAbgB0AG8AcgB5ACAAZABlAGYAYQB1AGwAdABzACkAIAAoAGsAZwApACAAKABXAGMAbwApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8AQQB2AGUAcgBhAGcAZQBMAGkAdgBlAHcAZQBpAGcAaAB0AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8AQQB2AGUAcgBhAGcAZQBMAGkAdgBlAHcAZQBpAGcAaAB0AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4ANgAuADUAOgAgAFMAdwBpAG4AZQAgAC0AIABBAHYAZQByAGEAZwBlACAAbABpAHYAZQB3AGUAaQBnAGgAdAAgACgAaQBuAHYAZQBuAHQAbwByAHkAIABkAGUAZgBhAHUAbAB0AHMAKQAgACgAawBnACkAIAAoAFcAYwBvACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBBAHYAZQByAGEAZwBlAEwAaQB2AGUAdwBlAGkAZwBoAHQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIALgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAEEAdgBlAHIAYQBnAGUATABpAHYAZQB3AGUAaQBnAGgAdABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGkAdgBlAHMAdABvAGMAawAgAFQAeQBwAGUAIABqAFwAIgAsACAAXAAiAEEAdgBlAHIAYQBnAGUAIABMAGkAdgBlAHcAZQBpAGcAaAB0ACAAKABrAGcAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHcAcwBcACIALAAgADEAOAA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAbwBhAHIAcwBcACIALAAgADIAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAaQBsAHQAcwBcACIALAAgADEAMgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAbABhAHUAZwBoAHQAZQByACAAcABpAGcAcwBcACIALAAgADMAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAGwAYQB1AGcAaAB0AGUAcgAgAHAAaQBnAHMAIABhAHQAIAB0AHUAcgBuAG8AZgBmAFwAIgAsACAAOQA3AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AcwBcAG4ANAAuADUAIABTAHcAaQBuAGUAIABGAGkAZwB1AHIAZQAgADQALgA4AFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFMAdwBpAG4AZQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQBzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8AUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADUAIABTAHcAaQBuAGUAIABGAGkAZwB1AHIAZQAgADQALgA4AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8AUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8AUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG4AdgBlAG4AdABpAG8AbgBhAGwAIABoAG8AdQBzAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGUAZQBwACAAbABpAHQAdABlAHIAIABoAG8AdQBzAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAHUAdABkAG8AbwByAC8AZgByAGUAZQAgAHIAYQBuAGcAZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAHIAeQBsAG8AdABNAE0AUwBcAG4ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXABuAGYAcgBhAGMAdABpAG8AbgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAHIAeQBsAG8AdABNAE0AUwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAbABvAHMAdAAgAHQAaAByAG8AdQBnAGgAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmACAAZgBvAHIAIABkAHIAeQBsAG8AdAAgAE0ATQBTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAHIAeQBsAG8AdABNAE0AUwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBGAHIAYQBjAEwARQBBAEMASABfAEQAcgB5AGwAbwB0AE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAHIAeQBsAG8AdABNAE0AUwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4ANQAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAHIAeQBsAG8AdABNAE0AUwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFADoAIABUAGUAeAB0ACAAcgBlAGYAZQByAHMAIAB0AG8AIABcAHUAMAAwADIANwBzAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAdQAwADAAMgA3ACAATQBNAFMALAAgAGIAdQB0ACAAZQBxAHUAYQB0AGkAbwBuACAAcgBlAGYAZQByAHMAIAB0AG8AIABcAHUAMAAwADIANwBkAHIAeQBsAG8AdABcAHUAMAAwADIANwAgAE0ATQBTAC4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBGAHIAYQBjAEwARQBBAEMASABfAEQAcgB5AGwAbwB0AE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMAAyACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATQBlAGcAYQBqAG8AdQBsAGUAcwBQAGUAcgBLAGkAbABvAGcAcgBhAG0ATQBlAHQAaABhAG4AZQBcAG4ARgBcAG4ATQBKAC8AawBnACAAQwBIADQAXABuAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBNAGUAZwBhAGoAbwB1AGwAZQBzAFAAZQByAEsAaQBsAG8AZwByAGEAbQBNAGUAdABoAGEAbgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGUAZwBhAGoAbwB1AGwAZQBzACAAcABlAHIAIABrAGkAbABvAGcAcgBhAG0AIABvAGYAIABtAGUAdABoAGEAbgBlAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATQBlAGcAYQBqAG8AdQBsAGUAcwBQAGUAcgBLAGkAbABvAGcAcgBhAG0ATQBlAHQAaABhAG4AZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE0AZQBnAGEAagBvAHUAbABlAHMAUABlAHIASwBpAGwAbwBnAHIAYQBtAE0AZQB0AGgAYQBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAEoAIAAvACAAawBnACAAQwBIADQAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBNAGUAZwBhAGoAbwB1AGwAZQBzAFAAZQByAEsAaQBsAG8AZwByAGEAbQBNAGUAdABoAGEAbgBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADMALgA1AC4AMgAuADMAIABDAE8ATgBTAFQAQQBOAFQAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBNAGUAZwBhAGoAbwB1AGwAZQBzAFAAZQByAEsAaQBsAG8AZwByAGEAbQBNAGUAdABoAGEAbgBlAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATQBlAGcAYQBqAG8AdQBsAGUAcwBQAGUAcgBLAGkAbABvAGcAcgBhAG0ATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgANQA1AC4AMgAyACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAFMAdwBpAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAzAC4ANQA6ACAARQBuAHQAZQByAGkAYwAgAE0AZQB0AGgAYQBuAGUAIAAtACAAUwB3AGkAbgBlAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAzAC4ANQAuADEALgAxACAATQBlAHQAaABvAGQAIAAxACAALQAgAEUAbgB0AGUAcgBpAGMAIABTAHcAaQBuAGUAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwAzAF8ANQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAFwAbgBUAG8AdABhAGwAIABhAG4AbgB1AGEAbAAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgByAG8AbQAgAGUAbgB0AGUAcgBpAGMAIABmAGUAcgBtAGUAbgB0AGEAdABpAG8AbgAgAGkAbgAgAHMAdwBpAG4AZQBcAG4ARQBfAGUAbgB0AGUAcgBpAGMAXABuAHQAIABDAEgANABcAG4ARQBfAHsAZQBuAHQAZQByAGkAYwB9AD0AXABcAHMAdQBtAF8AewBqAH0AKABOAF8AagBcAFwAdABpAG0AZQBzACAATQBfAGoAXABcAHQAaQBtAGUAcwAgAEQAXwBqACkAXABcAHQAaQBtAGUAcwAgADEAMABeAHsALQAzAH0AXABuAE4AXwBqACAAPQAgAG4AdQBtAGIAZQByAHMAIABvAGYAIABzAHcAaQBuAGUAIABvAGYAIABlAGEAYwBoACAAYwBsAGEAcwBzACAAKABoAGUAYQBkACkAXABuAE0AXwBqACAAPQAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAKABrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQApAFwAbgBEAF8AagAgAD0AIAB0AGgAZQAgAGEAdgBlAHIAYQBnAGUAIABuAHUAbQBiAGUAcgAgAG8AZgAgAGQAYQB5AHMAIABvAG4AIABmAGEAcgBtACAAZgBvAHIAIABlAGEAYwBoACAAcwB3AGkAbgBlACAAYwBsAGEAcwBzACAAKABkAGEAeQBzACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADUAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABOAF8AagAsACAATQBfAGoALAAgAEQAXwBqACwAXABuACAAIAAgACAAKABOAF8AagAgACoAIABNAF8AagAgACoAIABEAF8AagApACAAKgAgADEAMAAgAF4AIAAtADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8ANQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAG8AdABhAGwAIABhAG4AbgB1AGEAbAAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgByAG8AbQAgAGUAbgB0AGUAcgBpAGMAIABmAGUAcgBtAGUAbgB0AGEAdABpAG8AbgAgAGkAbgAgAHMAdwBpAG4AZQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADUAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAGUAbgB0AGUAcgBpAGMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwA1AF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBIADQAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwA1AF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADUALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAxACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwA1AF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwA1AF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AewBlAG4AdABlAHIAaQBjAH0APQBcAFwAcwB1AG0AXABcAG4AbwBsAGkAbQBpAHQAcwBfAGoAKABOAF8AagBcAFwAdABpAG0AZQBzACAATQBfAGoAXABcAHQAaQBtAGUAcwAgAEQAXwBqACkAXABcAHQAaQBtAGUAcwAgADEAMABeAHsALQAzAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwA1AF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBfAGoAXAAiACwAIABcACIAbgB1AG0AYgBlAHIAcwAgAG8AZgAgAHMAdwBpAG4AZQAgAG8AZgAgAGUAYQBjAGgAIABjAGwAYQBzAHMAXAAiACwAIABcACIAaABlAGEAZABcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AXwBqAFwAIgAsACAAXAAiAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuAFwAIgAsACAAXAAiAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAAMwAuADUALgAxAC4AMQAsACAAKAAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAXwBqAFwAIgAsACAAXAAiAHQAaABlACAAYQB2AGUAcgBhAGcAZQAgAG4AdQBtAGIAZQByACAAbwBmACAAZABhAHkAcwAgAG8AbgAgAGYAYQByAG0AIABmAG8AcgAgAGUAYQBjAGgAIABzAHcAaQBuAGUAIABjAGwAYQBzAHMAXAAiACwAIABcACIAZABhAHkAcwBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMwBfADUAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBcAG4AVABvAHQAYQBsACAAZABhAGkAbAB5ACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAG8AZgAgAGUAbgB0AGUAcgBpAGMAIABtAGUAdABoAGEAbgBlACAAbwBmACAAcwB3AGkAbgBlAFwAbgBNAF8AagBcAG4AawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXABuAE0AXwBqAD0AXABcAGYAcgBhAGMAewBJAF8AagBcAFwAdABpAG0AZQBzACAAMQA4AC4ANgBcAFwAdABpAG0AZQBzACAAMAAuADAAMAA3AH0AewBGAH0AXABuAEkAXwBqACAAPQAgAGQAYQBpAGwAeQAgAGYAZQBlAGQAIABpAG4AZwBlAHMAdABlAGQAIABiAHkAIABlAGEAYwBoACAAcwB3AGkAbgBlACAAYwBsAGEAcwBzACAAKABrAGcALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ARgAgAD0AIABtAGUAZwBhAGoAbwB1AGwAZQBzACAAcABlAHIAIABrAGkAbABvAGcAcgBhAG0AIABvAGYAIABtAGUAdABoAGEAbgBlACAAKABNAEoALwBrAGcAIABDAEgANAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADMAXwA1AF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAASQBfAGoALAAgAEYALABcAG4AIAAgACAAIAAoAEkAXwBqACAAKgAgADEAOAAuADYAIAAqACAAMAAuADAAMAA3ACkAIAAvACAARgBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwA1AF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAbwB0AGEAbAAgAGQAYQBpAGwAeQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABvAGYAIABlAG4AdABlAHIAaQBjACAAbQBlAHQAaABhAG4AZQAgAG8AZgAgAHMAdwBpAG4AZQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADUAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBfAGoAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwA1AF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADUAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4ANQAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADIAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADUAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADUAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AXwBqAD0AXABcAGYAcgBhAGMAewBJAF8AagBcAFwAdABpAG0AZQBzACAAMQA4AC4ANgBcAFwAdABpAG0AZQBzACAAMAAuADAAMAA3AH0AewBGAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwA1AF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBfAGoAXAAiACwAIABcACIAZABhAGkAbAB5ACAAZgBlAGUAZAAgAGkAbgBnAGUAcwB0AGUAZAAgAGIAeQAgAGUAYQBjAGgAIABzAHcAaQBuAGUAIABjAGwAYQBzAHMAXAAiACwAIABcACIAawBnAC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAMQA4AC4ANgBcACIALAAgAFwAIgBnAHIAbwBzAHMAIABlAG4AZQByAGcAeQAgACgARwBFACkAIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAZgBlAGUAZABcACIALAAgAFwAIgBNAEoAIABHAEUALwBrAGcAIABmAGUAZQBkAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAMAAuADAAMAA3AFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAEcARQAgAGkAbgB0AGEAawBlACAAYwBvAG4AdgBlAHIAdABlAGQAIAB0AG8AIABtAGUAdABoAGEAbgBlACAAYgB5ACAAcwB3AGkAbgBlAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAXAAiACwAIABcACIAbQBlAGcAYQBqAG8AdQBsAGUAcwAgAHAAZQByACAAawBpAGwAbwBnAHIAYQBtACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIALAAgAFwAIgBNAEoALwBrAGcAIABDAEgANABcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ANAAuADUAOgAgAFMAdwBpAG4AZQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ANAAuADUALgAxAC4AMQAgAE0AZQB0AGgAbwBkACAAMQAgABQgIABNAGEAbgB1AHIAZQAgAE0AZQB0AGgAYQBuAGUAIABTAHcAaQBuAGUAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAXABuAFQAbwB0AGEAbAAgAGEAbgBuAHUAYQBsACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdABcAG4ARQBDAEgANABcAG4AdAAgAEMASAA0AFwAbgB7AEUAfQBfAHsAQwBIADQAfQA9AFwAXABzAHUAbQBfAHsAagB9ACgARABfAHsAagB9AFwAXAB0AGkAbQBlAHMAIABNAF8AewBtAGoAfQBcAFwAdABpAG0AZQBzACAATgBfAHsAagB9ACkAXABcAHQAaQBtAGUAcwAxADAAXgB7AC0AMwB9AFwAbgBEAGoAIAA9ACAAbABlAG4AZwB0AGgAIABvAGYAIABzAHQAYQB5ACAAbwBmACAAZQBhAGMAaAAgAGMAbABhAHMAcwAgAG8AZgAgAHMAdwBpAG4AZQAgADoAIABkAGEAeQBzAFwAbgBNAG0AagAgAD0AIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIABtAGEAbgB1AHIAZQAgAGkAbgAgAGUAYQBjAGgAIABzAHcAaQBuAGUAIABjAGwAYQBzAHMAIAA6ACAAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXABuAE4AagAgAD0AIABuAHUAbQBiAGUAcgBzACAAbwBmACAAcwB3AGkAbgBlACAAaQBuACAAZQBhAGMAaAAgAGMAbABhAHMAcwAgADoAIABoAGUAYQBkAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABEAGoALAAgAE0AbQBqACwAIABOAGoALABcAG4AIAAgACAAIABEAGoAIAAqACAATQBtAGoAIAAqACAATgBqACAAKgAgADEAMAAgAF4AIAAtADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAbwB0AGEAbAAgAGEAbgBuAHUAYQBsACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEMASAA0AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBIADQAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4ANQAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADEAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB7AEUAfQBfAHsAQwBIADQAfQA9AFwAXABzAHUAbQBfAHsAagB9ACgARABfAHsAagB9AFwAXAB0AGkAbQBlAHMAIABNAF8AewBtAGoAfQBcAFwAdABpAG0AZQBzACAATgBfAHsAagB9ACkAXABcAHQAaQBtAGUAcwAxADAAXgB7AC0AMwB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABqAFwAIgAsAFwAIgBsAGUAbgBnAHQAaAAgAG8AZgAgAHMAdABhAHkAIABvAGYAIABlAGEAYwBoACAAYwBsAGEAcwBzACAAbwBmACAAcwB3AGkAbgBlAFwAIgAsACAAXAAiAGQAYQB5AHMAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAG0AagBcACIALABcACIAbQBlAHQAaABhAG4AZQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAHIAbwBtACAAbQBhAG4AdQByAGUAIABpAG4AIABlAGEAYwBoACAAcwB3AGkAbgBlACAAYwBsAGEAcwBzAFwAIgAsACAAXAAiAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAANAAuADUALgAxAC4AMQAgACgAMgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAGoAXAAiACwAXAAiAG4AdQBtAGIAZQByAHMAIABvAGYAIABzAHcAaQBuAGUAIABpAG4AIABlAGEAYwBoACAAYwBsAGEAcwBzAFwAIgAsACAAXAAiAGgAZQBhAGQAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADIAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUABlAHIAQwBsAGEAcwBzAFwAbgBNAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIAB0AGgAZQAgAG0AYQBuAHUAcgBlACAAbwBmACAAZQBhAGMAaAAgAGMAbABhAHMAcwAgAG8AZgAgAHMAdwBpAG4AZQBcAG4ATQBtAGoAXABuAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5AFwAbgBNAF8AewBtAGoAfQA9AFwAXABzAHUAbQBfAHsAbQB9AFwAXABzAHUAbQBfAHsAVAB9AE0AXwB7AGoAbQBUAH0AXABuAE0AagBtAFQAIAA9ACAAbQBlAHQAaABhAG4AZQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAHIAbwBtACAAbQBhAG4AdQByAGUAIABwAGUAcgAgAGMAbABhAHMAcwAsACAATQBNAFMALAAgAGEAbgBkACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAA6ACAAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMgBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAGUAcgBDAGwAYQBzAHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBqAG0AVAAsAFwAbgAgACAAIAAgAFMAVQBNACgATQBqAG0AVAApAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMgBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAGUAcgBDAGwAYQBzAHMAVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBqAG0AVAAxACwAIABNAGoAbQBUADIALABcAG4AIAAgACAAIAAgAFMAVQBNACgATQBqAG0AVAAxACwAIABNAGoAbQBUADIAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADIAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUABlAHIAQwBsAGEAcwBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIAB0AGgAZQAgAG0AYQBuAHUAcgBlACAAbwBmACAAZQBhAGMAaAAgAGMAbABhAHMAcwAgAG8AZgAgAHMAdwBpAG4AZQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMgBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAGUAcgBDAGwAYQBzAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AbQBqAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAyAF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAZQByAEMAbABhAHMAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAyAF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAZQByAEMAbABhAHMAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4ANQAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADIAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMgBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAGUAcgBDAGwAYQBzAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADIAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUABlAHIAQwBsAGEAcwBzAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBfAHsAbQBqAH0APQBcAFwAcwB1AG0AXwB7AG0AfQBcAFwAcwB1AG0AXwB7AFQAfQBNAF8AewBqAG0AVAB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAyAF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAZQByAEMAbABhAHMAcwBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGoAbQBUAFwAIgAsAFwAIgBtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIABtAGEAbgB1AHIAZQAgAHAAZQByACAAYwBsAGEAcwBzACwAIABNAE0AUwAsACAAYQBuAGQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQBcACIALAAgAFwAIgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADQALgA1AC4AMQAuADEAIAAoADMAKQAgAGEAbgBkACAAKAA2ACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAyAF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAZQByAEMAbABhAHMAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFADoAIABTAHAAbABpAHQAIAB2AGEAcgBpAGEAYgBsAGUAIABNAGoAbQAgAGkAbgB0AG8AIABNAGoAbQBUADEAIABhAG4AZAAgAE0AagBtAFQAMgAgAGYAbwByACAAcwB0AGEAZwBlACAAMQAgAGEAbgBkACAAMgAgAE0ATQBTAC4AXAAiACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAzAF8AUwB0AGEAZwBlADEATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFwAbgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAbwBmACAAbQBlAHQAaABhAG4AZQAgAGkAbgAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMQAgAE0ATQBTAFwAbgBNAGkAagBtAFQAMQBcAG4AawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXABuAE0AXwB7AGkAagBtACwAVAA9ADEAfQA9AFYAUwBfAHsAagB9AFwAXAB0AGkAbQBlAHMAIABGAFYAUwBfAHsAagBtACwAVAA9ADEAfQBcAFwAdABpAG0AZQBzACAATQBDAEYAXwB7AGkAbQB9AFwAXAB0AGkAbQBlAHMAIABCAE8AXABcAHQAaQBtAGUAcwAgAFwAXAByAGgAbwBcAG4AVgBTAGoAIAA9ACAAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIABzAHcAaQBuAGUAIABpAG4AIABlAGEAYwBoACAAYwBsAGEAcwBzACAAOgAgAGsAZwAvAGgAZQBhAGQALwBkAGEAeQBcAG4ARgBWAFMAagBtAFQAMQAgAD0AIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIAB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgAGkAbgAgAGUAYQBjAGgAIABwAHIAaQBtAGEAcgB5ACAAcwB5AHMAdABlAG0AIAA6ACAAZgByAGEAYwB0AGkAbwBuAFwAbgBNAEMARgBpAG0AIAA9ACAAbQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdABlAG0AcABlAHIAYQB0AGUAIAB6AG8AbgBlACAAYQBuAGQAIABzAHkAcwB0AGUAbQAgADoAIABmAHIAYQBjAHQAaQBvAG4AXABuAEIATwAgAD0AIABlAG0AaQBzAHMAaQBvAG4AcwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAOgAgAG0AMwAgAEMASAA0AC8AawBnACAAVgBTAFwAbgByAGgAbwAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgADoAIABrAGcALwBtADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABWAFMAagAsACAARgBWAFMAagBtAFQAMQAsACAATQBDAEYAaQBtACwAIABCAE8ALAAgAHIAaABvACwAXABuACAAIAAgACAAVgBTAGoAIAAqACAARgBWAFMAagBtAFQAMQAgACoAIABNAEMARgBpAG0AIAAqACAAQgBPACAAKgAgAHIAaABvAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAUAByAG8AZAB1AGMAdABpAG8AbgAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAIABpAG4AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADEAIABNAE0AUwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBpAGoAbQBUADEAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADMAXwBTAHQAYQBnAGUAMQBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4ANQAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADMAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AXwB7AGkAagBtACwAVAA9ADEAfQA9AFYAUwBfAHsAagB9AFwAXAB0AGkAbQBlAHMAIABGAFYAUwBfAHsAagBtACwAVAA9ADEAfQBcAFwAdABpAG0AZQBzACAATQBDAEYAXwB7AGkAbQB9AFwAXAB0AGkAbQBlAHMAIABCAE8AXABcAHQAaQBtAGUAcwAgAFwAXAByAGgAbwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAFMAagBcACIALABcACIAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIABzAHcAaQBuAGUAIABpAG4AIABlAGEAYwBoACAAYwBsAGEAcwBzAFwAIgAsACAAXAAiAGsAZwAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAVgBTAGoAbQBUADEAXAAiACwAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAHYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZABzACAAaQBuACAAZQBhAGMAaAAgAHAAcgBpAG0AYQByAHkAIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAA0AC4ANQAuADEALgAxACAAKAA0ACkAKAA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQwBGAGkAbQBcACIALABcACIAbQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdABlAG0AcABlAHIAYQB0AGUAIAB6AG8AbgBlACAAYQBuAGQAIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBCAE8AXAAiACwAXAAiAGUAbQBpAHMAcwBpAG8AbgBzACAAcABvAHQAZQBuAHQAaQBhAGwAXAAiACwAIABcACIAbQAzACAAQwBIADQALwBrAGcAIABWAFMAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgByAGgAbwBcACIALABcACIAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAXAAiACwAIABcACIAawBnAC8AbQAzAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA0AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBQAHIAaQBtAGEAcgB5AFMAeQBzAHQAZQBtAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIAB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgAGkAbgAgAGUAYQBjAGgAIABwAHIAaQBtAGEAcgB5ACAAcwB5AHMAdABlAG0AIABvAHQAaABlAHIAIAB0AGgAYQBuACAAcwBvAGwAaQBkACAAcwB0AG8AcgBhAGcAZQBcAG4ARgBWAFMAagBtAFQAMQBcAG4AZgByAGEAYwB0AGkAbwBuAFwAbgBGAFYAUwBfAHsAagBtACwAVAA9ADEAfQA9AE0ATQBTAF8AewBqAG0ALABUAD0AMQB9AFwAXAB0AGkAbQBlAHMAKAAxAC0AUwBTAF8AewBtAH0AKQBcAG4ATQBNAFMAagBtAFQAMQAgAD0AIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABtAGEAbgB1AHIAZQAgAHQAbwAgAGUAYQBjAGgAIABwAHIAaQBtAGEAcgB5ACAATQBNAFMAIABmAG8AcgAgAGUAYQBjAGgAIABjAGwAYQBzAHMAIABwAHIAaQBvAHIAIAB0AG8AIABzAG8AbABpAGQAIABzAGUAcABhAHIAYQB0AGkAbwBuACAAOgAgAGYAcgBhAGMAdABpAG8AbgBcAG4AUwBTAG0AIAA9ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkAHMAIABzAGUAcABhAHIAYQB0AGUAZAAgAHQAbwAgAHMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAIABmAG8AcgAgAGUAYQBjAGgAIABNAE0AUwAgADoAIABmAHIAYQBjAHQAaQBvAG4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANABfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAUAByAGkAbQBhAHIAeQBTAHkAcwB0AGUAbQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAE0AUwBqAG0AVAAxACwAIABTAFMAbQAsAFwAbgAgACAAIAAgAE0ATQBTAGoAbQBUADEAIAAqACAAKAAxACAALQAgAFMAUwBtACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA0AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBQAHIAaQBtAGEAcgB5AFMAeQBzAHQAZQBtAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIAB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgAGkAbgAgAGUAYQBjAGgAIABwAHIAaQBtAGEAcgB5ACAAcwB5AHMAdABlAG0AIABvAHQAaABlAHIAIAB0AGgAYQBuACAAcwBvAGwAaQBkACAAcwB0AG8AcgBhAGcAZQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANABfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAUAByAGkAbQBhAHIAeQBTAHkAcwB0AGUAbQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBWAFMAagBtAFQAMQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANABfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAUAByAGkAbQBhAHIAeQBTAHkAcwB0AGUAbQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANABfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAUAByAGkAbQBhAHIAeQBTAHkAcwB0AGUAbQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4ANQAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADQAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANABfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAUAByAGkAbQBhAHIAeQBTAHkAcwB0AGUAbQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANABfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAUAByAGkAbQBhAHIAeQBTAHkAcwB0AGUAbQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAVgBTAF8AewBqAG0ALABUAD0AMQB9AD0ATQBNAFMAXwB7AGoAbQAsAFQAPQAxAH0AXABcAHQAaQBtAGUAcwAoADEALQBTAFMAXwB7AG0AfQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA0AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBQAHIAaQBtAGEAcgB5AFMAeQBzAHQAZQBtAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0ATQBTAGoAbQBUADEAXAAiACwAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG0AYQBuAHUAcgBlACAAdABvACAAZQBhAGMAaAAgAHAAcgBpAG0AYQByAHkAIABNAE0AUwAgAGYAbwByACAAZQBhAGMAaAAgAGMAbABhAHMAcwAgAHAAcgBpAG8AcgAgAHQAbwAgAHMAbwBsAGkAZAAgAHMAZQBwAGEAcgBhAHQAaQBvAG4AXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBTAG0AXAAiACwAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAHYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZABzACAAcwBlAHAAYQByAGEAdABlAGQAIAB0AG8AIABzAG8AbABpAGQAIABzAHQAbwByAGEAZwBlACAAZgBvAHIAIABlAGEAYwBoACAATQBNAFMAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADQAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFAAcgBpAG0AYQByAHkAUwB5AHMAdABlAG0AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA1AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkAHMAIABpAG4AIABzAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAbgBGAFYAUwBqAG0ANABUADEAXABuAGYAcgBhAGMAdABpAG8AbgBcAG4ARgBWAFMAXwB7AGoALABtAD0ANAAsAFQAPQAxAH0APQBNAE0AUwBfAHsAagAsAG0APQA0ACwAVAA9ADEAfQArACgATQBNAFMAXwB7AGoALABtAD0AMQAsADcALAA5ACwAVAA9ADEAfQBcAFwAdABpAG0AZQBzACAAUwBTAF8AewBtAH0AKQBcAG4ATQBNAFMAagBtADQAVAAxACAAPQAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG0AYQBuAHUAcgBlACAAaQBuACAAcwBvAGwAaQBkACAAcwB0AG8AcgBhAGcAZQAgAHAAcgBpAG0AYQByAHkAIABzAHkAcwB0AGUAbQAgADoAIABmAHIAYQBjAHQAaQBvAG4AXABuAE0ATQBTAGoAbQAxADcAOQBUADEAIAA9ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAbQBhAG4AdQByAGUAIABpAG4AIABNAE0AUwAgADEALAAgADcALAAgAGEAbgBkACAAOQAgAGkAbgAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMQAgADoAIABmAHIAYQBjAHQAaQBvAG4AXABuAFMAUwBtACAAPQAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAHYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZABzACAAcwBlAHAAYQByAGEAdABlAGQAIAB0AG8AIABzAG8AbABpAGQAIABzAHQAbwByAGEAZwBlACAAZgBvAHIAIABlAGEAYwBoACAATQBNAFMAIAA6ACAAZgByAGEAYwB0AGkAbwBuAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADUAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0ATQBTAGoAbQA0AFQAMQAsACAATQBNAFMAagBtADEANwA5AFQAMQAsACAAUwBTAG0ALABcAG4AIAAgACAAIABNAE0AUwBqAG0ANABUADEAIAArACAAKABNAE0AUwBqAG0AMQA3ADkAVAAxACAAKgAgAFMAUwBtACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA1AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAE0AUwBqAG0ANABUADEALABcAG4AIAAgACAAIABNAE0AUwBqAG0AVAAxAF8AMQAsACAATQBNAFMAagBtAFQAMQBfADIALAAgAE0ATQBTAGoAbQBUADEAXwAzACwAIABNAE0AUwBqAG0AVAAxAF8ANAAsACAATQBNAFMAagBtAFQAMQBfADUALABcAG4AIAAgACAAIABTAFMAagBtAFQAMQBfADEALAAgAFMAUwBqAG0AVAAxAF8AMgAsACAAUwBTAGoAbQBUADEAXwAzACwAIABTAFMAagBtAFQAMQBfADQALAAgAFMAUwBqAG0AVAAxAF8ANQAsAFwAbgAgACAAIAAgACAAIABNAE0AUwBqAG0ANABUADEAIAArACAAXABuACAAIAAgACAAIAAgACgATQBNAFMAagBtAFQAMQBfADEAIAAqACAAUwBTAGoAbQBUADEAXwAxACkAIAArACAAXABuACAAIAAgACAAIAAgACgATQBNAFMAagBtAFQAMQBfADIAIAAqACAAUwBTAGoAbQBUADEAXwAyACkAIAArACAAXABuACAAIAAgACAAIAAgACgATQBNAFMAagBtAFQAMQBfADMAIAAqACAAUwBTAGoAbQBUADEAXwAzACkAIAArAFwAbgAgACAAIAAgACAAIAAoAE0ATQBTAGoAbQBUADEAXwA0ACAAKgAgAFMAUwBqAG0AVAAxAF8ANAApACAAKwBcAG4AIAAgACAAIAAgACAAKABNAE0AUwBqAG0AVAAxAF8ANQAgACoAIABTAFMAagBtAFQAMQBfADUAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADUAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIAB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgAGkAbgAgAHMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADUAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAFYAUwBqAG0ANABUADEAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADUAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA1AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4ANQAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADUAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADUAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBWAFMAXwB7AGoALABtAD0ANAAsAFQAPQAxAH0APQBNAE0AUwBfAHsAagAsAG0APQA0ACwAVAA9ADEAfQArACgATQBNAFMAXwB7AGoALABtAD0AMQAsADcALAA5ACwAVAA9ADEAfQBcAFwAdABpAG0AZQBzACAAUwBTAF8AewBtAH0AKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAFYAUwBfAHsAagAsAG0APQA0ACwAVAA9ADEAfQA9AE0ATQBTAF8AewBqACwAbQA9ADQALABUAD0AMQB9ACsAKABNAE0AUwBfAHsAagAsAG0APQAxACwAVAA9ADEAfQBcAFwAdABpAG0AZQBzACAAUwBTAF8AewBtAD0AMQAsAFQAPQAxAH0AKQArACgATQBNAFMAXwB7AGoALABtAD0ANwAsAFQAPQAxAH0AXABcAHQAaQBtAGUAcwAgAFMAUwBfAHsAbQA9ADcALABUAD0AMQB9ACkAKwAoAE0ATQBTAF8AewBqACwAbQA9ADkALABUAD0AMQB9AFwAXAB0AGkAbQBlAHMAIABTAFMAXwB7AG0APQA5ACwAVAA9ADEAfQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA1AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE0AUwBqAG0ANABUADEAXAAiACwAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG0AYQBuAHUAcgBlACAAaQBuACAAcwBvAGwAaQBkACAAcwB0AG8AcgBhAGcAZQAgAHAAcgBpAG0AYQByAHkAIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE0AUwBqAG0AMQA3ADkAVAAxAFwAIgAsAFwAIgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABtAGEAbgB1AHIAZQAgAGkAbgAgAE0ATQBTACAAMQAsACAANwAsACAAYQBuAGQAIAA5ACAAaQBuACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAAxAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAUwBtAFwAIgAsAFwAIgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIAB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgAHMAZQBwAGEAcgBhAHQAZQBkACAAdABvACAAcwBvAGwAaQBkACAAcwB0AG8AcgBhAGcAZQAgAGYAbwByACAAZQBhAGMAaAAgAE0ATQBTAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA1AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFADoAIABTAHAAbABpAHQAIABlAHEAdQBhAHQAaQBvAG4AIABmAG8AcgAgAE0ATQBTAG0APQAxACwANwAsADkAIABpAG4AdABvACAAcwBlAHAAYQByAGEAdABlACAAaQB0AGUAbQBzACAAdABvACAAYQBsAGwAbwB3ACAAZgBvAHIAIABjAGEAbABjAHUAbABhAHQAaQBvAG4AXAAiACkAOwBcAG4AIAAgAFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADYAXwBTAHQAYQBnAGUAMgBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXABuAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABvAGYAIABtAGUAdABoAGEAbgBlACAAaQBuACAAZQBhAGMAaAAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMgAgAE0ATQBTAFwAbgBNAGkAagBtAFQAMgBcAG4AawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXABuAE0AXwB7AGkAagBtACwAVAA9ADIAfQA9AFYAUwBUAF8AewBqAG0ALABUAD0AMgB9AFwAXAB0AGkAbQBlAHMAIABCAE8AXABcAHQAaQBtAGUAcwAgAE0ATQBTAF8AewBqAG0ALABUAD0AMgB9AFwAXAB0AGkAbQBlAHMAIABNAEMARgBfAHsAaQBtAH0AXABcAHQAaQBtAGUAcwAgAFwAXAByAGgAbwBcAG4AVgBTAFQAagBtAFQAMgAgAD0AIAB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgAHQAcgBhAG4AcwBmAGUAcgByAGUAZAAgAHQAbwAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMgAgAE0ATQBTACAAOgAgAGsAZwAvAGgAZQBhAGQALwBkAGEAeQBcAG4AQgBPACAAPQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAcABvAHQAZQBuAHQAaQBhAGwAIAA6ACAAbQAzACAAQwBIADQALwBrAGcAIABWAFMAXABuAE0ATQBTAGoAbQBUADIAIAA9ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAbQBhAG4AdQByAGUAIABpAG4AIABlAGEAYwBoACAAcwBlAGMAbwBuAGQAYQByAHkAIABzAHkAcwB0AGUAbQAgADoAIABmAHIAYQBjAHQAaQBvAG4AXABuAE0AQwBGAGkAbQAgAD0AIABtAGUAdABoAGEAbgBlACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAHoAbwBuAGUAIABhAG4AZAAgAHMAeQBzAHQAZQBtACAAOgAgAGYAcgBhAGMAdABpAG8AbgBcAG4AcgBoAG8AIAA9ACAAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAIAA6ACAAawBnAC8AbQAzAFwAbgBpACAAPQAgAHMAdABhAHQAZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA2AF8AUwB0AGEAZwBlADIATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFYAUwBUAGoAbQBUADIALAAgAEIATwAsACAATQBNAFMAagBtAFQAMgAsACAATQBDAEYAaQBtACwAIAByAGgAbwAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgAFYAUwBUAGoAbQBUADIALAAgAEkARgAoAEkAUwBOAFUATQBCAEUAUgAoAFYAUwBUAGoAbQBUADIAKQAsACAAVgBTAFQAagBtAFQAMgAsACAAMAApACwAXABuACAAIAAgACAAIAAgAE0ATQBTAGoAbQBUADIALAAgAEkARgAoAEkAUwBOAFUATQBCAEUAUgAoAE0ATQBTAGoAbQBUADIAKQAsACAATQBNAFMAagBtAFQAMgAsACAAMAApACwAXABuACAAIAAgACAAIAAgAFYAUwBUAGoAbQBUADIAIAAqACAAQgBPACAAKgAgAE0ATQBTAGoAbQBUADIAIAAqACAATQBDAEYAaQBtACAAKgAgAHIAaABvAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA2AF8AUwB0AGEAZwBlADIATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAbwBmACAAbQBlAHQAaABhAG4AZQAgAGkAbgAgAGUAYQBjAGgAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADIAIABNAE0AUwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANgBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBpAGoAbQBUADIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADYAXwBTAHQAYQBnAGUAMgBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANgBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4ANQAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADYAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANgBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANgBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AXwB7AGkAagBtACwAVAA9ADIAfQA9AFYAUwBUAF8AewBqAG0ALABUAD0AMgB9AFwAXAB0AGkAbQBlAHMAIABCAE8AXABcAHQAaQBtAGUAcwAgAE0ATQBTAF8AewBqAG0ALABUAD0AMgB9AFwAXAB0AGkAbQBlAHMAIABNAEMARgBfAHsAaQBtAH0AXABcAHQAaQBtAGUAcwAgAFwAXAByAGgAbwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANgBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAFMAVABqAG0AVAAyAFwAIgAsAFwAIgB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgAHQAcgBhAG4AcwBmAGUAcgByAGUAZAAgAHQAbwAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMgAgAE0ATQBTAFwAIgAsACAAXAAiAGsAZwAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADQALgA1AC4AMQAuADEAIAAoADcAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgBPAFwAIgAsAFwAIgBlAG0AaQBzAHMAaQBvAG4AcwAgAHAAbwB0AGUAbgB0AGkAYQBsAFwAIgAsACAAXAAiAG0AMwAgAEMASAA0AC8AawBnACAAVgBTAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBNAFMAagBtAFQAMgBcACIALABcACIAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAbQBhAG4AdQByAGUAIABpAG4AIABlAGEAYwBoACAAcwBlAGMAbwBuAGQAYQByAHkAIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEMARgBpAG0AXAAiACwAXAAiAG0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHQAZQBtAHAAZQByAGEAdABlACAAegBvAG4AZQAgAGEAbgBkACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAcgBoAG8AXAAiACwAXAAiAGQAZQBuAHMAaQB0AHkAIABvAGYAIABtAGUAdABoAGEAbgBlAFwAIgAsACAAXAAiAGsAZwAvAG0AMwBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAGkAXAAiACwAXAAiAHMAdABhAHQAZQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA2AF8AUwB0AGEAZwBlADIATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AQQByAGcAdQBtAGUAbgB0AHMAXwBNAGUAdABoAG8AZAAyAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAFMAVABqAG0AVAAyAFwAIgAsAFwAIgB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgAHQAcgBhAG4AcwBmAGUAcgByAGUAZAAgAHQAbwAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMgAgAE0ATQBTAFwAIgAsACAAXAAiAGsAZwAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADQALgA1AC4AMQAuADEAIAAoADcAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgBPAFwAIgAsAFwAIgBlAG0AaQBzAHMAaQBvAG4AcwAgAHAAbwB0AGUAbgB0AGkAYQBsAFwAIgAsACAAXAAiAG0AMwAgAEMASAA0AC8AawBnACAAVgBTAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBNAFMAagBtAFQAMgBcACIALABcACIAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAbQBhAG4AdQByAGUAIABpAG4AIABlAGEAYwBoACAAcwBlAGMAbwBuAGQAYQByAHkAIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEMARgBpAG0AXAAiACwAXAAiAG0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHQAZQBtAHAAZQByAGEAdABlACAAegBvAG4AZQAgAGEAbgBkACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAcgBoAG8AXAAiACwAXAAiAGQAZQBuAHMAaQB0AHkAIABvAGYAIABtAGUAdABoAGEAbgBlAFwAIgAsACAAXAAiAGsAZwAvAG0AMwBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQQBUAFwAIgAsAFwAIgBNAGUAYQBuACAAYQBuAG4AdQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAXAAiACwAIABcACIAsABDAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANwBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBUAHIAYQBuAHMAZgBlAHIAcgBlAGQAUwB0AGEAZwBlADIAXABuAFYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZABzACAAdAByAGEAbgBzAGYAZQByAHIAZQBkACAAdABvACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAAyACAATQBNAFMAXABuAFYAUwBUAGkAagBtAFQAMgBcAG4AawBnACAAVgBTAFwAbgBWAFMAVABfAHsAaQBqAG0ALABUAD0AMgB9AD0AVgBTAF8AewBqAH0AXABcAHQAaQBtAGUAcwAgAEYAVgBTAF8AewBqAG0ALABUAD0AMQB9AFwAXAB0AGkAbQBlAHMAKAAxAC0AVgBTAEwAXwB7AG0ALABUAD0AMQB9ACkAXABuAFYAUwBqACAAPQAgAHYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZAAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAHIAbwBtACAAcwB3AGkAbgBlACAAaQBuACAAZQBhAGMAaAAgAGMAbABhAHMAcwAgADoAIABrAGcALwBoAGUAYQBkAC8AZABhAHkAXABuAEYAVgBTAGoAbQBUADEAIAA9ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkAHMAIABpAG4AIABlAGEAYwBoACAAcAByAGkAbQBhAHIAeQAgAHMAeQBzAHQAZQBtACAAOgAgAGYAcgBhAGMAdABpAG8AbgBcAG4AVgBTAEwAbQBUADEAIAA9ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkAHMAIABsAG8AcwB0ACAAZAB1AHIAaQBuAGcAIABzAHQAbwByAGEAZwBlACAAaQBuACAAdABoAGUAIABwAHIAaQBtAGEAcgB5ACAAcwB5AHMAdABlAG0AIAA6ACAAZgByAGEAYwB0AGkAbwBuAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADcAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVAByAGEAbgBzAGYAZQByAHIAZQBkAFMAdABhAGcAZQAyAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFYAUwBqACwAIABGAFYAUwBqAG0AVAAxACwAIABWAFMATABtAFQAMQAsAFwAbgAgACAAIAAgAFYAUwBqACAAKgAgAEYAVgBTAGoAbQBUADEAIAAqACAAKAAxACAALQAgAFYAUwBMAG0AVAAxACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA3AF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFQAcgBhAG4AcwBmAGUAcgByAGUAZABTAHQAYQBnAGUAMgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkAHMAIAB0AHIAYQBuAHMAZgBlAHIAcgBlAGQAIAB0AG8AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADIAIABNAE0AUwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANwBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBUAHIAYQBuAHMAZgBlAHIAcgBlAGQAUwB0AGEAZwBlADIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAUwBUAGkAagBtAFQAMgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANwBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBUAHIAYQBuAHMAZgBlAHIAcgBlAGQAUwB0AGEAZwBlADIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABWAFMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADcAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVAByAGEAbgBzAGYAZQByAHIAZQBkAFMAdABhAGcAZQAyAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgA1AC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgANwApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA3AF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFQAcgBhAG4AcwBmAGUAcgByAGUAZABTAHQAYQBnAGUAMgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANwBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBUAHIAYQBuAHMAZgBlAHIAcgBlAGQAUwB0AGEAZwBlADIAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAFMAVABfAHsAaQBqAG0ALABUAD0AMgB9AD0AVgBTAF8AewBqAH0AXABcAHQAaQBtAGUAcwAgAEYAVgBTAF8AewBqAG0ALABUAD0AMQB9AFwAXAB0AGkAbQBlAHMAKAAxAC0AVgBTAEwAXwB7AG0ALABUAD0AMQB9ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADcAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVAByAGEAbgBzAGYAZQByAHIAZQBkAFMAdABhAGcAZQAyAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAUwBqAFwAIgAsAFwAIgB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgByAG8AbQAgAHMAdwBpAG4AZQAgAGkAbgAgAGUAYQBjAGgAIABjAGwAYQBzAHMAXAAiACwAIABcACIAawBnAC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBWAFMAagBtAFQAMQBcACIALABcACIAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkAHMAIABpAG4AIABlAGEAYwBoACAAcAByAGkAbQBhAHIAeQAgAHMAeQBzAHQAZQBtAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADQALgA1AC4AMQAuADEAIAAoADQAKQAoADUAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBTAEwAbQBUADEAXAAiACwAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAHYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZABzACAAbABvAHMAdAAgAGQAdQByAGkAbgBnACAAcwB0AG8AcgBhAGcAZQAgAGkAbgAgAHQAaABlACAAcAByAGkAbQBhAHIAeQAgAHMAeQBzAHQAZQBtAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBMAG8AbwBrAHUAcABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ANAAuADUAOgAgAFMAdwBpAG4AZQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ANAAuADUALgAxAC4AMwAgAE0AZQB0AGgAbwBkACAAMQAgAC0AIABNAGEAbgB1AHIAZQAgAEQAaQByAGUAYwB0ACAATgAyAE8AIABTAHcAaQBuAGUAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0ATQBNAFMAXABuAFQAbwB0AGEAbAAgAGEAbgBuAHUAYQBsACAAZABpAHIAZQBjAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAAbQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAcwB5AHMAdABlAG0AcwBcAG4ARQBfAE4AMgBPAGQAaQByAFwAbgB0ACAATgAyAE8AXABuAEUAXwB7AE4AMgBPACwAZABpAHIAfQA9AFwAXABzAHUAbQBfAHsAagB9AFwAXABzAHUAbQBfAHsAbQB9AFwAXABzAHUAbQBfAHsAVAB9ACgATQBOAF8AewBqAG0AVAB9AFwAXAB0AGkAbQBlAHMAIABFAEYAXwB7AGoAbQB9AFwAXAB0AGkAbQBlAHMAIABDAF8AewBOADIATwB9ACkAXABcAHQAaQBtAGUAcwAxADAAXgB7AC0AMwB9AFwAbgBNAE4AXwBqAG0AVAAgAD0AIABuAGkAdAByAG8AZwBlAG4AIABwAGUAcgAgAHMAdwBpAG4AZQAgAGMAbABhAHMAcwAsACAATQBNAFMAIABhAG4AZAAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAKABrAGcAIABOACkAXABuAEUARgBfAGoAbQAgAD0AIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAE0ATQBTACAAKABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACkAXABuAEMAXwBOADIATwAgAD0AIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwARABpAHIAZQBjAHQATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBNAE0AUwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAE4AXwBqAG0AVAAsACAARQBGAF8AagBtACwAIABDAF8ATgAyAE8ALABcAG4AIAAgACAAIABNAE4AXwBqAG0AVAAgACoAIABFAEYAXwBqAG0AIAAqACAAQwBfAE4AMgBPACAAKgAgADEAMAAgAF4AIAAtADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0ATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAbwB0AGEAbAAgAGEAbgBuAHUAYQBsACAAZABpAHIAZQBjAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAAbQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAcwB5AHMAdABlAG0AcwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABEAGkAcgBlAGMAdABOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAE0ATQBTAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8ATgAyAE8AZABpAHIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwARABpAHIAZQBjAHQATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBNAE0AUwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABOADIATwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABEAGkAcgBlAGMAdABOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAE0ATQBTAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgA1AC4AMQAuADMALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0ATQBNAFMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwARABpAHIAZQBjAHQATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBNAE0AUwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwB7AE4AMgBPACwAZABpAHIAfQA9AFwAXABzAHUAbQBfAHsAagB9AFwAXABzAHUAbQBfAHsAbQB9AFwAXABzAHUAbQBfAHsAVAB9ACgATQBOAF8AewBqAG0AVAB9AFwAXAB0AGkAbQBlAHMAIABFAEYAXwB7AGoAbQB9AFwAXAB0AGkAbQBlAHMAIABDAF8AewBOADIATwB9ACkAXABcAHQAaQBtAGUAcwAxADAAXgB7AC0AMwB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0ATQBNAFMAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBOAF8AagBtAFQAXAAiACwAIABcACIAbgBpAHQAcgBvAGcAZQBuACAAcABlAHIAIABzAHcAaQBuAGUAIABjAGwAYQBzAHMALAAgAE0ATQBTACAAYQBuAGQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQBcACIALAAgAFwAIgBrAGcAIABOAFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAANAAuADUALgAxAC4AMwAgACgAMgApACgANgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEYAXwBqAG0AXAAiACwAIABcACIAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABNAE0AUwBcACIALAAgAFwAIgBrAGcAIABOADIATwAtAE4ALwBrAGcAIABOAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBfAE4AMgBPAFwAIgAsACAAXAAiAGYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXAAiACwAIABcACIAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADIAXwBTAHQAYQBnAGUAMQBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAFwAbgBOAGkAdAByAG8AZwBlAG4AIABpAG4AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADEAIABNAE0AUwBcAG4ATQBOAF8AagBtAFQAMQBcAG4AawBnACAATgBcAG4ATQBOAF8AewBqAG0ALABUAD0AMQB9AD0AQQBFAF8AewBqAH0AXABcAHQAaQBtAGUAcwAgAEYATgBfAHsAagBtACwAVAA9ADEAfQBcAG4AQQBFAF8AagAgAD0AIAB0AG8AdABhAGwAIABuAGkAdAByAG8AZwBlAG4AIABlAHgAYwByAGUAdABlAGQAIABiAHkAIABlAGEAYwBoACAAcwB3AGkAbgBlACAAYwBsAGEAcwBzACAAKABrAGcAIABOACkAXABuAEYATgBfAGoAbQBUADEAIAA9ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAaQBuACAAZQBhAGMAaAAgAHAAcgBpAG0AYQByAHkAIABNAE0AUwAgAHMAeQBzAHQAZQBtAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADIAXwBTAHQAYQBnAGUAMQBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEEARQBfAGoALAAgAEYATgBfAGoAbQBUADEALABcAG4AIAAgACAAIABBAEUAXwBqACAAKgAgAEYATgBfAGoAbQBUADEAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwAyAF8AUwB0AGEAZwBlADEATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBpAHQAcgBvAGcAZQBuACAAaQBuACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAAxACAATQBNAFMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADIAXwBTAHQAYQBnAGUAMQBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE4AXwBqAG0AVAAxAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwAyAF8AUwB0AGEAZwBlADEATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADIAXwBTAHQAYQBnAGUAMQBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgA1AC4AMQAuADMALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMgApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwAyAF8AUwB0AGEAZwBlADEATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8AMgBfAFMAdABhAGcAZQAxAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE4AXwB7AGoAbQAsAFQAPQAxAH0APQBBAEUAXwB7AGoAfQBcAFwAdABpAG0AZQBzACAARgBOAF8AewBqAG0ALABUAD0AMQB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwAyAF8AUwB0AGEAZwBlADEATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAEUAXwBqAFwAIgAsACAAXAAiAHQAbwB0AGEAbAAgAG4AaQB0AHIAbwBnAGUAbgAgAGUAeABjAHIAZQB0AGUAZAAgAGIAeQAgAGUAYQBjAGgAIABzAHcAaQBuAGUAIABjAGwAYQBzAHMAXAAiACwAIABcACIAawBnACAATgBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADQALgA1AC4AMQAuADMAIAAoADUAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBOAF8AagBtAFQAMQBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABuAGkAdAByAG8AZwBlAG4AIABpAG4AIABlAGEAYwBoACAAcAByAGkAbQBhAHIAeQAgAE0ATQBTACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAANAAuADUALgAxAC4AMwAgACgAMwApACgANAApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADMAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBJAG4AUAByAGkAbQBhAHIAeQBNAE0AUwBcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAaQBuACAAZQBhAGMAaAAgAHAAcgBpAG0AYQByAHkAIABNAE0AUwAgACgAZQB4AGMAbAB1AGQAaQBuAGcAIABzAG8AbABpAGQAIABzAHQAbwByAGEAZwBlACkAXABuAEYATgBfAGoAbQBUADEAXABuAGYAcgBhAGMAdABpAG8AbgBcAG4ARgBOAF8AewBqAG0ALABUAD0AMQB9AD0ATQBNAFMAXwB7AGoAbQAsAFQAPQAxAH0AXABcAHQAaQBtAGUAcwAoADEALQBTAE4AXwB7AG0AfQApAFwAbgBNAE0AUwBfAGoAbQBUADEAIAA9ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAbQBhAG4AdQByAGUAIABpAG4AIABwAHIAaQBtAGEAcgB5ACAATQBNAFMAXABuAFMATgBfAG0AIAA9ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAcwBlAHAAYQByAGEAdABlAGQAIAB0AG8AIABzAG8AbABpAGQAIABzAHQAbwByAGEAZwBlACAAZgBvAHIAIABlAGEAYwBoACAATQBNAFMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8AMwBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEkAbgBQAHIAaQBtAGEAcgB5AE0ATQBTAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0ATQBTAF8AagBtAFQAMQAsACAAUwBOAF8AbQAsAFwAbgAgACAAIAAgAE0ATQBTAF8AagBtAFQAMQAgACoAIAAoADEAIAAtACAAUwBOAF8AbQApAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8AMwBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEkAbgBQAHIAaQBtAGEAcgB5AE0ATQBTAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABuAGkAdAByAG8AZwBlAG4AIABpAG4AIABlAGEAYwBoACAAcAByAGkAbQBhAHIAeQAgAE0ATQBTACAAKABlAHgAYwBsAHUAZABpAG4AZwAgAHMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8AMwBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEkAbgBQAHIAaQBtAGEAcgB5AE0ATQBTAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAE4AXwBqAG0AVAAxAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwAzAF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ASQBuAFAAcgBpAG0AYQByAHkATQBNAFMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADMAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBJAG4AUAByAGkAbQBhAHIAeQBNAE0AUwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4ANQAuADEALgAzACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADMAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8AMwBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEkAbgBQAHIAaQBtAGEAcgB5AE0ATQBTAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwAzAF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ASQBuAFAAcgBpAG0AYQByAHkATQBNAFMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAE4AXwB7AGoAbQAsAFQAPQAxAH0APQBNAE0AUwBfAHsAagBtACwAVAA9ADEAfQBcAFwAdABpAG0AZQBzACgAMQAtAFMATgBfAHsAbQB9ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADMAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBJAG4AUAByAGkAbQBhAHIAeQBNAE0AUwBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE0AUwBfAGoAbQBUADEAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAbQBhAG4AdQByAGUAIABpAG4AIABwAHIAaQBtAGEAcgB5ACAATQBNAFMAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBOAF8AbQBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABuAGkAdAByAG8AZwBlAG4AIABzAGUAcABhAHIAYQB0AGUAZAAgAHQAbwAgAHMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAIABmAG8AcgAgAGUAYQBjAGgAIABNAE0AUwBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADQAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBJAG4AUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG4AaQB0AHIAbwBnAGUAbgAgAGkAbgAgAHMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXABuAEYATgBfAGoAbQA0AFQAMQBcAG4AZgByAGEAYwB0AGkAbwBuAFwAbgBGAE4AXwB7AGoAbQA9ADQALABUAD0AMQB9AD0ATQBNAFMAXwB7AGoAbQA9ADQALABUAD0AMQB9ACsAKABNAE0AUwBfAHsAagBtAD0AMQAsADcALAA5ACwAVAA9ADEAfQBcAFwAdABpAG0AZQBzACAAUwBOAF8AewBtAH0AKQBcAG4ATQBNAFMAXwBqAG0ANABUADEAIAA9ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAbQBhAG4AdQByAGUAIABpAG4AIABzAG8AbABpAGQAIABzAHQAbwByAGEAZwBlACAATQBNAFMAXABuAE0ATQBTAF8AagBtADEANwA5AFQAMQAgAD0AIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABtAGEAbgB1AHIAZQAgAGkAbgAgAHAAcgBpAG0AYQByAHkAIABsAGkAcQB1AGkAZAAgAHMAeQBzAHQAZQBtAHMAIAAoAG0APQAxACwANwAsADkAKQBcAG4AUwBOAF8AbQAgAD0AIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABuAGkAdAByAG8AZwBlAG4AIABzAGUAcABhAHIAYQB0AGUAZAAgAHQAbwAgAHMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAIABmAG8AcgAgAGUAYQBjAGgAIABNAE0AUwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA0AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ASQBuAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0ATQBTAF8AagBtADQAVAAxACwAIABNAE0AUwBfAGoAbQAxADcAOQBUADEALAAgAFMATgBfAG0ALABcAG4AIAAgACAAIABNAE0AUwBfAGoAbQA0AFQAMQAgACsAIAAoAE0ATQBTAF8AagBtADEANwA5AFQAMQAgACoAIABTAE4AXwBtACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA0AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ASQBuAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0ATQBTAF8AagBtADQAVAAxACwAXABuACAAIAAgACAATQBNAFMAagBtAFQAMQBfADEALAAgAE0ATQBTAGoAbQBUADEAXwAyACwAIABNAE0AUwBqAG0AVAAxAF8AMwAsACAATQBNAFMAagBtAFQAMQBfADQALAAgAE0ATQBTAGoAbQBUADEAXwA1ACwAXABuACAAIAAgACAAUwBTAGoAbQBUADEAXwAxACwAIABTAFMAagBtAFQAMQBfADIALAAgAFMAUwBqAG0AVAAxAF8AMwAsACAAUwBTAGoAbQBUADEAXwA0ACwAIABTAFMAagBtAFQAMQBfADUALABcAG4AIAAgACAAIABNAE0AUwBfAGoAbQA0AFQAMQAgACsAIAAoAE0ATQBTAGoAbQBUADEAXwAxACAAKgAgAFMAUwBqAG0AVAAxAF8AMQApACAAKwAgACgATQBNAFMAagBtAFQAMQBfADIAIAAqACAAUwBTAGoAbQBUADEAXwAyACkAIAArACAAKABNAE0AUwBqAG0AVAAxAF8AMwAgACoAIABTAFMAagBtAFQAMQBfADMAKQAgACsAIAAoAE0ATQBTAGoAbQBUADEAXwA0ACAAKgAgAFMAUwBqAG0AVAAxAF8ANAApACAAKwAgACgATQBNAFMAagBtAFQAMQBfADUAIAAqACAAUwBTAGoAbQBUADEAXwA1ACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA0AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ASQBuAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABuAGkAdAByAG8AZwBlAG4AIABpAG4AIABzAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA0AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ASQBuAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAE4AXwBqAG0ANABUADEAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADQAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBJAG4AUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADQAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBJAG4AUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADUALgAxAC4AMwAsACAARQBxAHUAYQB0AGkAbwBuACAAKAA0ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADQAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBJAG4AUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADQAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBJAG4AUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAE4AXwB7AGoAbQA9ADQALABUAD0AMQB9AD0ATQBNAFMAXwB7AGoAbQA9ADQALABUAD0AMQB9ACsAKABNAE0AUwBfAHsAagBtAD0AMQAsADcALAA5ACwAVAA9ADEAfQBcAFwAdABpAG0AZQBzACAAUwBOAF8AewBtAH0AKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8ANABfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEkAbgBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYATgBfAHsAagBtAD0ANAAsAFQAPQAxAH0APQBNAE0AUwBfAHsAagBtAD0ANAAsAFQAPQAxAH0AKwAoAE0ATQBTAF8AewBqACwAbQA9ADEALABUAD0AMQB9AFwAXAB0AGkAbQBlAHMAIABTAFMAXwB7AG0APQAxACwAVAA9ADEAfQApACsAKABNAE0AUwBfAHsAagAsAG0APQA3ACwAVAA9ADEAfQBcAFwAdABpAG0AZQBzACAAUwBTAF8AewBtAD0ANwAsAFQAPQAxAH0AKQArACgATQBNAFMAXwB7AGoALABtAD0AOQAsAFQAPQAxAH0AXABcAHQAaQBtAGUAcwAgAFMAUwBfAHsAbQA9ADkALABUAD0AMQB9ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADQAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBJAG4AUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBNAFMAXwBqAG0ANABUADEAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAbQBhAG4AdQByAGUAIABpAG4AIABzAG8AbABpAGQAIABzAHQAbwByAGEAZwBlACAATQBNAFMAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBNAFMAXwBqAG0AMQA3ADkAVAAxAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG0AYQBuAHUAcgBlACAAaQBuACAAcAByAGkAbQBhAHIAeQAgAGwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwAgACgAbQA9ADEALAA3ACwAOQApAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMATgBfAG0AXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAcwBlAHAAYQByAGEAdABlAGQAIAB0AG8AIABzAG8AbABpAGQAIABzAHQAbwByAGEAZwBlACAAZgBvAHIAIABlAGEAYwBoACAATQBNAFMAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADQAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBJAG4AUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6ACAAUwBwAGwAaQB0ACAAZQBxAHUAYQB0AGkAbwBuACAAZgBvAHIAIABNAE0AUwBtAD0AMQAsADcALAA5ACAAaQBuAHQAbwAgAHMAZQBwAGEAcgBhAHQAZQAgAGkAdABlAG0AcwAgAHQAbwAgAGEAbABsAG8AdwAgAGYAbwByACAAYwBhAGwAYwB1AGwAYQB0AGkAbwBuAFwAIgApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8ANQBfAEEAbgBuAHUAYQBsAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBcAG4AQQBuAG4AdQBhAGwAIABuAGkAdAByAG8AZwBlAG4AIABlAHgAYwByAGUAdABpAG8AbgAgAGYAcgBvAG0AIABlAGEAYwBoACAAcwB3AGkAbgBlACAAZwByAG8AdQBwAFwAbgBBAEUAXwBqAFwAbgBrAGcAIABOAFwAbgBBAEUAXwB7AGoAfQA9AE4AXwB7AGoAfQBcAFwAdABpAG0AZQBzACAATgBXAF8AewBqAH0AXABcAHQAaQBtAGUAcwAgAEQAXwB7AGoAfQBcAG4ATgBfAGoAIAA9ACAAbgB1AG0AYgBlAHIAIABvAGYAIABzAHcAaQBuAGUAIABpAG4AIABlAGEAYwBoACAAZwByAG8AdQBwACAAKABoAGUAYQBkACkAXABuAE4AVwBfAGoAIAA9ACAAbgBpAHQAcgBvAGcAZQBuACAAcAByAG8AZAB1AGMAZQBkACAAaQBuACAAcwB3AGkAbgBlACAAbQBhAG4AdQByAGUAIABhAG4AZAAgAHcAYQBzAHQAZQAgAGYAZQBlAGQAIABpAG4AIABlAGEAYwBoACAAYwBsAGEAcwBzACAAKABrAGcAIABOAC8AaABlAGEAZAAvAGQAYQB5ACkAXABuAEQAXwBqACAAPQAgAGQAdQByAGEAdABpAG8AbgAgAG8AZgAgAHMAdABhAHkAIABvAGYAIABzAHcAaQBuAGUAIABnAHIAbwB1AHAAIAAoAGQAYQB5AHMAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA1AF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE4AXwBqACwAIABOAFcAXwBqACwAIABEAF8AagAsAFwAbgAgACAAIAAgAE4AXwBqACAAKgAgAE4AVwBfAGoAIAAqACAARABfAGoAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA1AF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAG4AbgB1AGEAbAAgAG4AaQB0AHIAbwBnAGUAbgAgAGUAeABjAHIAZQB0AGkAbwBuACAAZgByAG8AbQAgAGUAYQBjAGgAIABzAHcAaQBuAGUAIABnAHIAbwB1AHAAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADUAXwBBAG4AbgB1AGEAbABOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAaQBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEARQBfAGoAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADUAXwBBAG4AbgB1AGEAbABOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA1AF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgA1AC4AMQAuADMALAAgAEUAcQB1AGEAdABpAG8AbgAgACgANQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA1AF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA1AF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBFAF8AewBqAH0APQBOAF8AewBqAH0AXABcAHQAaQBtAGUAcwAgAE4AVwBfAHsAagB9AFwAXAB0AGkAbQBlAHMAIABEAF8AewBqAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADUAXwBBAG4AbgB1AGEAbABOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBfAGoAXAAiACwAIABcACIAbgB1AG0AYgBlAHIAIABvAGYAIABzAHcAaQBuAGUAIABpAG4AIABlAGEAYwBoACAAZwByAG8AdQBwAFwAIgAsACAAXAAiAGgAZQBhAGQAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAFcAXwBqAFwAIgAsACAAXAAiAG4AaQB0AHIAbwBnAGUAbgAgAHAAcgBvAGQAdQBjAGUAZAAgAGkAbgAgAHMAdwBpAG4AZQAgAG0AYQBuAHUAcgBlACAAYQBuAGQAIAB3AGEAcwB0AGUAIABmAGUAZQBkACAAaQBuACAAZQBhAGMAaAAgAGMAbABhAHMAcwBcACIALAAgAFwAIgBrAGcAIABOAC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABfAGoAXAAiACwAIABcACIAZAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAG8AZgAgAHMAdwBpAG4AZQAgAGcAcgBvAHUAcABcACIALAAgAFwAIgBkAGEAeQBzAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA2AF8AUwB0AGEAZwBlADIATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBcAG4ATgBpAHQAcgBvAGcAZQBuACAAaQBuACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAAyACAATQBNAFMAXABuAE0ATgBfAGoAbQBUADIAXABuAGsAZwAgAE4AXABuAE0ATgBfAHsAagBtACwAVAA9ADIAfQA9AE4AVABfAHsAagBtACwAVAA9ADIAfQBcAFwAdABpAG0AZQBzACAATQBNAFMAXwB7AGoAbQAsAFQAPQAyAH0AXABuAE4AVABfAGoAbQBUADIAIAA9ACAAbgBpAHQAcgBvAGcAZQBuACAAdAByAGEAbgBzAGYAZQByAHIAZQBkACAAdABvACAAcwBlAGMAbwBuAGQAYQByAHkAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAE0ATQBTACAAKABrAGcAIABOACkAXABuAE0ATQBTAF8AagBtAFQAMgAgAD0AIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABtAGEAbgB1AHIAZQAgAGkAbgAgAGUAYQBjAGgAIABzAGUAYwBvAG4AZABhAHIAeQAgAHMAeQBzAHQAZQBtAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADYAXwBTAHQAYQBnAGUAMgBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE4AVABfAGoAbQBUADIALAAgAE0ATQBTAF8AagBtAFQAMgAsAFwAbgAgACAAIAAgAE4AVABfAGoAbQBUADIAIAAqACAATQBNAFMAXwBqAG0AVAAyAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8ANgBfAFMAdABhAGcAZQAyAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwBnAGUAbgAgAGkAbgAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMgAgAE0ATQBTAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA2AF8AUwB0AGEAZwBlADIATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBOAF8AagBtAFQAMgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8ANgBfAFMAdABhAGcAZQAyAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA2AF8AUwB0AGEAZwBlADIATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4ANQAuADEALgAzACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADYAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8ANgBfAFMAdABhAGcAZQAyAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADYAXwBTAHQAYQBnAGUAMgBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBOAF8AewBqAG0ALABUAD0AMgB9AD0ATgBUAF8AewBqAG0ALABUAD0AMgB9AFwAXAB0AGkAbQBlAHMAIABNAE0AUwBfAHsAagBtACwAVAA9ADIAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8ANgBfAFMAdABhAGcAZQAyAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBUAF8AagBtAFQAMgBcACIALAAgAFwAIgBuAGkAdAByAG8AZwBlAG4AIAB0AHIAYQBuAHMAZgBlAHIAcgBlAGQAIAB0AG8AIABzAGUAYwBvAG4AZABhAHIAeQAgAHQAcgBlAGEAdABtAGUAbgB0ACAATQBNAFMAXAAiACwAIABcACIAawBnACAATgBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADQALgA1AC4AMQAuADMAIAAoADcAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBNAFMAXwBqAG0AVAAyAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG0AYQBuAHUAcgBlACAAaQBuACAAZQBhAGMAaAAgAHMAZQBjAG8AbgBkAGEAcgB5ACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA3AF8ATgBpAHQAcgBvAGcAZQBuAFQAcgBhAG4AcwBmAGUAcgByAGUAZABUAG8AUwB0AGEAZwBlADIATQBNAFMAXABuAE4AaQB0AHIAbwBnAGUAbgAgAHQAcgBhAG4AcwBmAGUAcgByAGUAZAAgAHQAbwAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMgAgAE0ATQBTAFwAbgBOAFQAXwBqAG0AVAAyAFwAbgBrAGcAIABOAFwAbgBOAFQAXwB7AGoAbQAsAFQAPQAyAH0APQBNAE4AXwB7AGoAbQAsAFQAPQAxAH0AXABcAHQAaQBtAGUAcwAoADEALQBGAHIAYQBjAEcAQQBTAE0AXwB7AG0ALABUAD0AMQB9AC0ARQBGAF8AewBtACwAVAA9ADEAfQApAFwAbgBNAE4AXwBqAG0AVAAxACAAPQAgAG4AaQB0AHIAbwBnAGUAbgAgAHAAZQByACAAcwB3AGkAbgBlACAAYwBsAGEAcwBzACAAaQBuACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAAxACAATQBNAFMAIAAoAGsAZwAgAE4AKQBcAG4ARgByAGEAYwBHAEEAUwBNAG0AVAAxACAAPQAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB2AG8AbABhAHQAaQBsAGkAcwBlAGQAIABmAHIAbwBtACAATQBNAFMAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGEAdAAgAHMAdABhAGcAZQAgADEAXABuAEUARgBfAG0AVAAxACAAPQAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAATQBNAFMAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGEAdAAgAHMAdABhAGcAZQAgADEAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8ANwBfAE4AaQB0AHIAbwBnAGUAbgBUAHIAYQBuAHMAZgBlAHIAcgBlAGQAVABvAFMAdABhAGcAZQAyAE0ATQBTAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0ATgBfAGoAbQBUADEALAAgAEYAcgBhAGMARwBBAFMATQBtAFQAMQAsACAARQBGAF8AbQBUADEALABcAG4AIAAgACAAIABNAE4AXwBqAG0AVAAxACAAKgAgACgAMQAgAC0AIABGAHIAYQBjAEcAQQBTAE0AbQBUADEAIAAtACAARQBGAF8AbQBUADEAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADcAXwBOAGkAdAByAG8AZwBlAG4AVAByAGEAbgBzAGYAZQByAHIAZQBkAFQAbwBTAHQAYQBnAGUAMgBNAE0AUwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBpAHQAcgBvAGcAZQBuACAAdAByAGEAbgBzAGYAZQByAHIAZQBkACAAdABvACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAAyACAATQBNAFMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADcAXwBOAGkAdAByAG8AZwBlAG4AVAByAGEAbgBzAGYAZQByAHIAZQBkAFQAbwBTAHQAYQBnAGUAMgBNAE0AUwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBUAF8AagBtAFQAMgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8ANwBfAE4AaQB0AHIAbwBnAGUAbgBUAHIAYQBuAHMAZgBlAHIAcgBlAGQAVABvAFMAdABhAGcAZQAyAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8ANwBfAE4AaQB0AHIAbwBnAGUAbgBUAHIAYQBuAHMAZgBlAHIAcgBlAGQAVABvAFMAdABhAGcAZQAyAE0ATQBTAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgA1AC4AMQAuADMALAAgAEUAcQB1AGEAdABpAG8AbgAgACgANwApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA3AF8ATgBpAHQAcgBvAGcAZQBuAFQAcgBhAG4AcwBmAGUAcgByAGUAZABUAG8AUwB0AGEAZwBlADIATQBNAFMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADcAXwBOAGkAdAByAG8AZwBlAG4AVAByAGEAbgBzAGYAZQByAHIAZQBkAFQAbwBTAHQAYQBnAGUAMgBNAE0AUwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AVABfAHsAagBtACwAVAA9ADIAfQA9AE0ATgBfAHsAagBtACwAVAA9ADEAfQBcAFwAdABpAG0AZQBzACgAMQAtAEYAcgBhAGMARwBBAFMATQBfAHsAbQAsAFQAPQAxAH0ALQBFAEYAXwB7AG0ALABUAD0AMQB9ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADcAXwBOAGkAdAByAG8AZwBlAG4AVAByAGEAbgBzAGYAZQByAHIAZQBkAFQAbwBTAHQAYQBnAGUAMgBNAE0AUwBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE4AXwBqAG0AVAAxAFwAIgAsACAAXAAiAG4AaQB0AHIAbwBnAGUAbgAgAHAAZQByACAAcwB3AGkAbgBlACAAYwBsAGEAcwBzACAAaQBuACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAAxACAATQBNAFMAXAAiACwAIABcACIAawBnACAATgBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADQALgA1AC4AMQAuADMAIAAoADIAKQAoADYAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBHAEEAUwBNAG0AVAAxAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB2AG8AbABhAHQAaQBsAGkAcwBlAGQAIABmAHIAbwBtACAATQBNAFMAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGEAdAAgAHMAdABhAGcAZQAgADEAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEwAbwBvAGsAdQBwAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEYAXwBtAFQAMQBcACIALAAgAFwAIgBuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAE0ATQBTACAAdAByAGUAYQB0AG0AZQBuAHQAIABhAHQAIABzAHQAYQBnAGUAIAAxAFwAIgAsACAAXAAiAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AXAAiACwAIABcACIATABvAG8AawB1AHAAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8ATQBNAFMAXwBTAHcAaQBuAGUAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA0AC4ANQA6ACAAUwB3AGkAbgBlAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA0AC4ANQAuADEALgA1ACAATQBlAHQAaABvAGQAIAAxACAALQAgAE0AYQBuAHUAcgBlACAAQQB0AG0AbwBzAHAAaABlAHIAaQBjACAARABlAHAAbwBzAGkAdABpAG8AbgAgAFMAdwBpAG4AZQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADUAXwBfADEAXwBBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAE0ATQBTAFwAbgBBAG4AbgB1AGEAbAAgAGEAdABtAG8AcwBwAGgAZQByAGkAYwAgAGQAZQBwAG8AcwBpAHQAaQBvAG4AIABlAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABNAE0AUwBcAG4ARQBfAE4AMgBPAE0ATQBTAGEAZABcAG4AdAAgAE4AMgBPAFwAbgBFAF8AewBOADIATwAsAGEAZAB9AD0ATQBNAFMAXwB7AEEAVABNAE8AUwB9AFwAXAB0AGkAbQBlAHMAIABFAEYAXwB7AE4AMgBPAH0AXABcAHQAaQBtAGUAcwAgAEMAXwB7AE4AMgBPAH0AXABcAHQAaQBtAGUAcwAgADEAMABeAHsALQAzAH0AXABuAE0ATQBTAF8AQQBUAE0ATwBTACAAPQAgAG0AYQBzAHMAIABvAGYAIABOACAAdgBvAGwAYQB0AGkAbABpAHMAZQBkACAAZgByAG8AbQAgAE0ATQBTACAAKABrAGcAIABOACkAXABuAEUARgBfAE4AMgBPACAAPQAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAYQB0AG0AbwBzAHAAaABlAHIAaQBjACAAZABlAHAAbwBzAGkAdABpAG8AbgAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApAFwAbgBDAF8ATgAyAE8AIAA9ACAAZgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAATgAyAE8AIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANQBfAF8AMQBfAEEAbgBuAHUAYQBsAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0ATQBNAFMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBNAFMAXwBBAFQATQBPAFMALAAgAEUARgBfAE4AMgBPACwAIABDAF8ATgAyAE8ALABcAG4AIAAgACAAIABNAE0AUwBfAEEAVABNAE8AUwAgACoAIABFAEYAXwBOADIATwAgACoAIABDAF8ATgAyAE8AIAAqACAAMQAwACAAXgAgAC0AMwBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADUAXwBfADEAXwBBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAE0ATQBTAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAG4AbgB1AGEAbAAgAGEAdABtAG8AcwBwAGgAZQByAGkAYwAgAGQAZQBwAG8AcwBpAHQAaQBvAG4AIABlAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABNAE0AUwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANQBfAF8AMQBfAEEAbgBuAHUAYQBsAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0ATQBNAFMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwBOADIATwBNAE0AUwBhAGQAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADUAXwBfADEAXwBBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAE4AMgBPAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA1AF8AXwAxAF8AQQBuAG4AdQBhAGwAQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBNAE0AUwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4ANQAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADEAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANQBfAF8AMQBfAEEAbgBuAHUAYQBsAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0ATQBNAFMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADUAXwBfADEAXwBBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAE0ATQBTAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAHsATgAyAE8ALABhAGQAfQA9AE0ATQBTAF8AewBBAFQATQBPAFMAfQBcAFwAdABpAG0AZQBzACAARQBGAF8AewBOADIATwB9AFwAXAB0AGkAbQBlAHMAIABDAF8AewBOADIATwB9AFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA1AF8AXwAxAF8AQQBuAG4AdQBhAGwAQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBNAE0AUwBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE0AUwBfAEEAVABNAE8AUwBcACIALAAgAFwAIgBtAGEAcwBzACAAbwBmACAATgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGYAcgBvAG0AIABNAE0AUwBcACIALAAgAFwAIgBrAGcAIABOAFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAANAAuADUALgAxAC4ANQAgACgAMgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEYAXwBOADIATwBcACIALAAgAFwAIgBuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGEAdABtAG8AcwBwAGgAZQByAGkAYwAgAGQAZQBwAG8AcwBpAHQAaQBvAG4AXAAiACwAIABcACIAawBnACAATgAyAE8ALQBOAC8AawBnACAATgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAXwBOADIATwBcACIALAAgAFwAIgBmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIALAAgAFwAIgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAGoAXAAiACwAIABcACIAcAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAaQByAFwAIgAsACAAXAAiAGkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAHIAXAAiACwAIABcACIAcgBhAGkAbgBmAGEAbABsACAAcgBlAGcAaQBvAG4AXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADUAXwBfADIAXwBUAG8AdABhAGwATgBpAHQAcgBvAGcAZQBuAFYAbwBsAGEAdABpAGwAaQBzAGUAZABGAHIAbwBtAE0ATQBTAFwAbgBUAG8AdABhAGwAIABuAGkAdAByAG8AZwBlAG4AIAB2AG8AbABhAHQAaQBsAGkAcwBlAGQAIABmAHIAbwBtACAATQBNAFMAXABuAE0ATQBTAF8AQQBUAE0ATwBTAFwAbgBrAGcAIABOAFwAbgBNAE0AUwBfAHsAQQBUAE0ATwBTAH0APQBcAFwAcwB1AG0AXwB7AGoAfQBcAFwAcwB1AG0AXwB7AG0AfQBcAFwAcwB1AG0AXwB7AFQAfQAoAE0ATgBfAHsAagBtAFQAfQBcAFwAdABpAG0AZQBzACAARgByAGEAYwBHAEEAUwBNAF8AewBtAFQAfQApAFwAbgBNAE4AXwBqAG0AVAAgAD0AIABuAGkAdAByAG8AZwBlAG4AIABwAGUAcgAgAHMAdwBpAG4AZQAgAGMAbABhAHMAcwAsACAATQBNAFMAIABhAG4AZAAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAKABrAGcAIABOACkAXABuAEYAcgBhAGMARwBBAFMATQBtAFQAIAA9ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGkAbgAgAGUAYQBjAGgAIABNAE0AUwAgACgAKABrAGcAIABOAEgAMwAtAE4AIAArACAATgBPAHgALQBOACkALwBrAGcAIABOACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANQBfAF8AMgBfAFQAbwB0AGEAbABOAGkAdAByAG8AZwBlAG4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAEYAcgBvAG0ATQBNAFMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBOAF8AagBtAFQALAAgAEYAcgBhAGMARwBBAFMATQBtAFQALABcAG4AIAAgACAAIABNAE4AXwBqAG0AVAAgACoAIABGAHIAYQBjAEcAQQBTAE0AbQBUAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANQBfAF8AMgBfAFQAbwB0AGEAbABOAGkAdAByAG8AZwBlAG4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAEYAcgBvAG0ATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAbwB0AGEAbAAgAG4AaQB0AHIAbwBnAGUAbgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGYAcgBvAG0AIABNAE0AUwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANQBfAF8AMgBfAFQAbwB0AGEAbABOAGkAdAByAG8AZwBlAG4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAEYAcgBvAG0ATQBNAFMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0ATQBTAF8AQQBUAE0ATwBTAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA1AF8AXwAyAF8AVABvAHQAYQBsAE4AaQB0AHIAbwBnAGUAbgBWAG8AbABhAHQAaQBsAGkAcwBlAGQARgByAG8AbQBNAE0AUwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADUAXwBfADIAXwBUAG8AdABhAGwATgBpAHQAcgBvAGcAZQBuAFYAbwBsAGEAdABpAGwAaQBzAGUAZABGAHIAbwBtAE0ATQBTAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgA1AC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMgApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA1AF8AXwAyAF8AVABvAHQAYQBsAE4AaQB0AHIAbwBnAGUAbgBWAG8AbABhAHQAaQBsAGkAcwBlAGQARgByAG8AbQBNAE0AUwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANQBfAF8AMgBfAFQAbwB0AGEAbABOAGkAdAByAG8AZwBlAG4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAEYAcgBvAG0ATQBNAFMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE0AUwBfAHsAQQBUAE0ATwBTAH0APQBcAFwAcwB1AG0AXwB7AGoAfQBcAFwAcwB1AG0AXwB7AG0AfQBcAFwAcwB1AG0AXwB7AFQAfQAoAE0ATgBfAHsAagBtAFQAfQBcAFwAdABpAG0AZQBzACAARgByAGEAYwBHAEEAUwBNAF8AewBtAFQAfQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA1AF8AXwAyAF8AVABvAHQAYQBsAE4AaQB0AHIAbwBnAGUAbgBWAG8AbABhAHQAaQBsAGkAcwBlAGQARgByAG8AbQBNAE0AUwBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE4AXwBqAG0AVABcACIALAAgAFwAIgBuAGkAdAByAG8AZwBlAG4AIABwAGUAcgAgAHMAdwBpAG4AZQAgAGMAbABhAHMAcwAsACAATQBNAFMAIABhAG4AZAAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlAFwAIgAsACAAXAAiAGsAZwAgAE4AXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAA0AC4ANQAuADEALgAzACAAKAAyACkAKAA2ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAcgBhAGMARwBBAFMATQBtAFQAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGkAbgAgAGUAYQBjAGgAIABNAE0AUwBcACIALAAgAFwAIgAoAGsAZwAgAE4ASAAzAC0ATgAgACsAIABOAE8AeAAtAE4AKQAvAGsAZwAgAE4AXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAE0ATQBTAF8AUwB3AGkAbgBlAF8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADQALgA1ADoAIABTAHcAaQBuAGUAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADQALgA1AC4AMQAuADcAIABNAGUAdABoAG8AZAAgADEAIAAtACAATQBhAG4AdQByAGUAIABMAGUAYQBjAGgAaQBuAGcAIABBAG4AZAAgAFIAdQBuAG8AZgBmACAATgAyAE8AIABTAHcAaQBuAGUAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA3AF8AXwAxAF8AQQBuAG4AdQBhAGwARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARgByAG8AbQBNAE0AUwBcAG4AQQBuAG4AdQBhAGwAIABlAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmACAAZgByAG8AbQAgAGUAYQBjAGgAIABNAE0AUwBcAG4ARQBfAE4AMgBPAGwAZQBhAGMAaABcAG4AdAAgAE4AMgBPAFwAbgBFAF8AewBOADIATwAsAGwAZQBhAGMAaAB9AD0ATQBOAEwAZQBhAGMAaABfAHsAagBtAD0ANQB9AFwAXAB0AGkAbQBlAHMAIABFAEYAXwB7AGwAZQBhAGMAaAB9AFwAXAB0AGkAbQBlAHMAIABDAF8AewBOADIATwB9AFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9AFwAbgBNAE4ATABlAGEAYwBoAF8AagBtADUAIAA9ACAAbQBhAHMAcwAgAG8AZgAgAE4AIABsAG8AcwB0ACAAdABoAHIAbwB1AGcAaAAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIABmAHIAbwBtACAAZAByAHkAbABvAHQAIABNAE0AUwAgACgAawBnACAATgApAFwAbgBFAEYAXwBsAGUAYQBjAGgAIAA9ACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQBcAG4AQwBfAE4AMgBPACAAPQAgAGYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFADoAIABEAHUAZQAgAHQAbwAgAHMAdAByAGkAYwB0ACAAZQBuAHYAaQByAG8AbgBtAGUAbgB0AGEAbAAgAGMAbwBuAHQAcgBvAGwAcwAsACAAZQBtAGkAcwBzAGkAbwBuAHMAIABhAHIAZQAgAGUAcwB0AGkAbQBhAHQAZQBkACAAbwBuAGwAeQAgAGYAbwByACAAZAByAHkAbABvAHQAIABNAE0AUwAgACgAbQA9ADUAKQAuAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADcAXwBfADEAXwBBAG4AbgB1AGEAbABFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBGAHIAbwBtAE0ATQBTAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0ATgBMAGUAYQBjAGgAXwBqAG0ANQAsACAARQBGAF8AbABlAGEAYwBoACwAIABDAF8ATgAyAE8ALABcAG4AIAAgACAAIABNAE4ATABlAGEAYwBoAF8AagBtADUAIAAqACAARQBGAF8AbABlAGEAYwBoACAAKgAgAEMAXwBOADIATwAgACoAIAAxADAAIABeACAALQAzAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANwBfAF8AMQBfAEEAbgBuAHUAYQBsAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEYAcgBvAG0ATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAbgBuAHUAYQBsACAAZQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgAgAGYAcgBvAG0AIABlAGEAYwBoACAATQBNAFMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADcAXwBfADEAXwBBAG4AbgB1AGEAbABFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBGAHIAbwBtAE0ATQBTAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8ATgAyAE8AbABlAGEAYwBoAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA3AF8AXwAxAF8AQQBuAG4AdQBhAGwARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARgByAG8AbQBNAE0AUwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABOADIATwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANwBfAF8AMQBfAEEAbgBuAHUAYQBsAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEYAcgBvAG0ATQBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADUALgAxAC4ANwAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAxACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADcAXwBfADEAXwBBAG4AbgB1AGEAbABFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBGAHIAbwBtAE0ATQBTAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA3AF8AXwAxAF8AQQBuAG4AdQBhAGwARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARgByAG8AbQBNAE0AUwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwB7AE4AMgBPACwAbABlAGEAYwBoAH0APQBNAE4ATABlAGEAYwBoAF8AewBqAG0APQA1AH0AXABcAHQAaQBtAGUAcwAgAEUARgBfAHsAbABlAGEAYwBoAH0AXABcAHQAaQBtAGUAcwAgAEMAXwB7AE4AMgBPAH0AXABcAHQAaQBtAGUAcwAgADEAMABeAHsALQAzAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADcAXwBfADEAXwBBAG4AbgB1AGEAbABFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBGAHIAbwBtAE0ATQBTAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0ATgBMAGUAYQBjAGgAXwBqAG0ANQBcACIALAAgAFwAIgBtAGEAcwBzACAAbwBmACAATgAgAGwAbwBzAHQAIAB0AGgAcgBvAHUAZwBoACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgAgAGYAcgBvAG0AIABkAHIAeQBsAG8AdAAgAE0ATQBTAFwAIgAsACAAXAAiAGsAZwAgAE4AXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAA0AC4ANQAuADEALgA3ACAAKAAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBfAGwAZQBhAGMAaABcACIALAAgAFwAIgBlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIALAAgAFwAIgBrAGcAIABOADIATwAtAE4ALwBrAGcAIABOAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBfAE4AMgBPAFwAIgAsACAAXAAiAGYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA3AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABvAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBGAHIAbwBtAEQAcgB5AGwAbwB0AE0ATQBTAFwAbgBNAGEAcwBzACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAbABvAHMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIABmAHIAbwBtACAAZAByAHkAbABvAHQAIABNAE0AUwBcAG4ATQBOAEwAZQBhAGMAaABfAGoAbQA1AFwAbgBrAGcAIABOAFwAbgBNAE4ATABlAGEAYwBoAF8AewBqAG0APQA1AH0APQBNAE4AXwB7AGoAbQA9ADUALABUAD0AMQB9AFwAXAB0AGkAbQBlAHMAIABGAHIAYQBjAFcARQBUAFwAXAB0AGkAbQBlAHMAIABGAHIAYQBjAEwARQBBAEMASABfAHsATQBTAH0AXABuAE0ATgBfAGoAbQA1AFQAMQAgAD0AIABuAGkAdAByAG8AZwBlAG4AIABpAG4AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADEAIABkAHIAeQBsAG8AdAAgAE0ATQBTACAAKABrAGcAIABOACkAXABuAEYAcgBhAGMAVwBFAFQAIAA9ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgBGAHIAYQBjAEwARQBBAEMASABfAE0AUwAgAD0AIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAbABvAHMAdAAgAHQAaAByAG8AdQBnAGgAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADcAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAG8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEYAcgBvAG0ARAByAHkAbABvAHQATQBNAFMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBOAF8AagBtADUAVAAxACwAIABGAHIAYQBjAFcARQBUACwAIABGAHIAYQBjAEwARQBBAEMASABfAE0AUwAsAFwAbgAgACAAIAAgAE0ATgBfAGoAbQA1AFQAMQAgACoAIABGAHIAYQBjAFcARQBUACAAKgAgAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANwBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAbwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARgByAG8AbQBEAHIAeQBsAG8AdABNAE0AUwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBhAHMAcwAgAG8AZgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAbwBzAHQAIAB0AG8AIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmACAAZgByAG8AbQAgAGQAcgB5AGwAbwB0ACAATQBNAFMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADcAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAG8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEYAcgBvAG0ARAByAHkAbABvAHQATQBNAFMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0ATgBMAGUAYQBjAGgAXwBqAG0ANQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANwBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAbwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARgByAG8AbQBEAHIAeQBsAG8AdABNAE0AUwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADcAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAG8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEYAcgBvAG0ARAByAHkAbABvAHQATQBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADUALgAxAC4ANwAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAyACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADcAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAG8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEYAcgBvAG0ARAByAHkAbABvAHQATQBNAFMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADcAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAG8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEYAcgBvAG0ARAByAHkAbABvAHQATQBNAFMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE4ATABlAGEAYwBoAF8AewBqAG0APQA1AH0APQBNAE4AXwB7AGoAbQA9ADUALABUAD0AMQB9AFwAXAB0AGkAbQBlAHMAIABGAHIAYQBjAFcARQBUAFwAXAB0AGkAbQBlAHMAIABGAHIAYQBjAEwARQBBAEMASABfAHsATQBTAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADcAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAG8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEYAcgBvAG0ARAByAHkAbABvAHQATQBNAFMAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBOAF8AagBtADUAVAAxAFwAIgAsACAAXAAiAG4AaQB0AHIAbwBnAGUAbgAgAGkAbgAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMQAgAGQAcgB5AGwAbwB0ACAATQBNAFMAXAAiACwAIABcACIAawBnACAATgBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADQALgA1AC4AMQAuADMAIAAoADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBXAEUAVABcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAGwAbwBzAHQAIAB0AGgAcgBvAHUAZwBoACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgB6AFwAIgAsACAAXAAiAGwAbwBjAGEAdABpAG8AbgAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBqAFwAIgAsACAAXAAiAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAGkAcgBcACIALAAgAFwAIgBpAHIAcgBpAGcAYQB0AGkAbwBuACAAbQBlAHQAaABvAGQAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBhAG4AdQByAGUAQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADQALgA1ADoAIABTAHcAaQBuAGUAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADQALgA1AC4AMQAuADkAIABNAGEAbgB1AHIAZQAgAEEAcABwAGwAaQBlAGQAIAB0AG8AIABTAG8AaQBsAHMAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA5AF8AXwAxAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMQBcAG4ATQBhAHMAcwAgAG8AZgAgAG4AaQB0AHIAbwBnAGUAbgAgAGEAcABwAGwAaQBlAGQAIAB0AG8AIABzAG8AaQBsAHMAIABmAG8AcgAgAHMAYwBvAHAAZQAgADEAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ATQBOAFMAbwBpAGwAXwBzAGMAbwBwAGUAMQBcAG4AawBnACAATgBcAG4ATQBOAFMAbwBpAGwAXwB7AHMAYwBvAHAAZQAxAH0APQBcAFwAcwB1AG0AXwB7AGoAfQBcAFwAcwB1AG0AXwB7AG0AfQAoAE0ATgBfAHsAagBtAFQAPQAyAH0AXABcAHQAaQBtAGUAcwAoADEALQBFAEYAXwB7AG0AVAA9ADIAfQAtAEYAcgBhAGMARwBBAFMATQBfAHsAbQBUAD0AMgB9ACkALQBNAE4ATABlAGEAYwBoAF8AewBqAG0APQA1AH0AKQBcAFwAdABpAG0AZQBzACAAUABGAFwAbgBNAE4AXwBqAG0AVAAyACAAPQAgAG0AYQBzAHMAIABvAGYAIABOACAAaQBuACAATQBNAFMAIABhAHQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADIAIAA6ACAAawBnACAATgBcAG4ARQBGAF8AbQBUADIAIAA9ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABlAGEAYwBoACAATQBNAFMAIABhAHQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADIAIAA6ACAAawBnACAATgAyAE8ALQBOAC8AawBnACAATgBcAG4ARgByAGEAYwBHAEEAUwBNAF8AbQBUADIAIAA9ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAYQBuAGkAbQBhAGwAIAB3AGEAcwB0AGUAIABOACAAdgBvAGwAYQB0AGkAbABpAHMAZQBkACAAaQBuACAAZQBhAGMAaAAgAE0ATQBTACAAYQB0ACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAAyACAAOgAgACgAawBnACAATgBIADMALQBOACAAKwAgAE4ATwB4AC0ATgApAC8AawBnACAATgBcAG4ATQBOAEwAZQBhAGMAaABfAGoAbQA1ACAAPQAgAG0AYQBzAHMAIABvAGYAIABOACAAbABvAHMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIABmAHIAbwBtACAAZAByAHkAbABvAHQAIABNAE0AUwAgADoAIABrAGcAIABOAFwAbgBQAEYAIAA9ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAbQBhAG4AdQByAGUAIABhAHAAcABsAGkAZQBkACAAdABvACAAcwBvAGkAbAAgAHcAaQB0AGgAaQBuACAAdABoAGUAIABwAGkAZwBnAGUAcgB5ACAAYgBvAHUAbgBkAGEAcgB5ACAAOgAgAGYAcgBhAGMAdABpAG8AbgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA5AF8AXwAxAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAE4AXwBqAG0AVAAyACwAIABFAEYAXwBtAFQAMgAsACAARgByAGEAYwBHAEEAUwBNAF8AbQBUADIALAAgAE0ATgBMAGUAYQBjAGgAXwBqAG0ANQAsACAAUABGACwAXABuACAAIAAgACAAKABNAE4AXwBqAG0AVAAyACAAKgAgACgAMQAgAC0AIABFAEYAXwBtAFQAMgAgAC0AIABGAHIAYQBjAEcAQQBTAE0AXwBtAFQAMgApACAALQAgAE0ATgBMAGUAYQBjAGgAXwBqAG0ANQApACAAKgAgAFAARgBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADkAXwBfADEAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAxAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAcwBzACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAYQBwAHAAbABpAGUAZAAgAHQAbwAgAHMAbwBpAGwAcwAgAGYAbwByACAAcwBjAG8AcABlACAAMQAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA5AF8AXwAxAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBOAFMAbwBpAGwAXwBzAGMAbwBwAGUAMQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AOQBfAF8AMQBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADEAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA5AF8AXwAxAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4ANQAuADEALgA5ACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADEAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AOQBfAF8AMQBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADEAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADkAXwBfADEAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAxAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBOAFMAbwBpAGwAXwB7AHMAYwBvAHAAZQAxAH0APQBcAFwAcwB1AG0AXwB7AGoAfQBcAFwAcwB1AG0AXwB7AG0AfQAoAE0ATgBfAHsAagBtAFQAPQAyAH0AXABcAHQAaQBtAGUAcwAoADEALQBFAEYAXwB7AG0AVAA9ADIAfQAtAEYAcgBhAGMARwBBAFMATQBfAHsAbQBUAD0AMgB9ACkALQBNAE4ATABlAGEAYwBoAF8AewBqAG0APQA1AH0AKQBcAFwAdABpAG0AZQBzACAAUABGAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA5AF8AXwAxAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE4AXwBqAG0AVAAyAFwAIgAsAFwAIgBtAGEAcwBzACAAbwBmACAATgAgAGkAbgAgAE0ATQBTACAAYQB0ACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAAyAFwAIgAsACAAXAAiAGsAZwAgAE4AXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAA0AC4ANQAuADEALgAzACAAKAA2ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBfAG0AVAAyAFwAIgAsAFwAIgBuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGUAYQBjAGgAIABNAE0AUwAgAGEAdAAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMgBcACIALAAgAFwAIgBrAGcAIABOADIATwAtAE4ALwBrAGcAIABOAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBHAEEAUwBNAF8AbQBUADIAXAAiACwAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAGEAbgBpAG0AYQBsACAAdwBhAHMAdABlACAATgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGkAbgAgAGUAYQBjAGgAIABNAE0AUwAgAGEAdAAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMgBcACIALAAgAFwAIgAoAGsAZwAgAE4ASAAzAC0ATgAgACsAIABOAE8AeAAtAE4AKQAvAGsAZwAgAE4AXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE4ATABlAGEAYwBoAF8AagBtADUAXAAiACwAXAAiAG0AYQBzAHMAIABvAGYAIABOACAAbABvAHMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIABmAHIAbwBtACAAZAByAHkAbABvAHQAIABNAE0AUwBcACIALAAgAFwAIgBrAGcAIABOAFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAANAAuADUALgAxAC4ANwAgACgAMgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEYAXAAiACwAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG0AYQBuAHUAcgBlACAAYQBwAHAAbABpAGUAZAAgAHQAbwAgAHMAbwBpAGwAIAB3AGkAdABoAGkAbgAgAHQAaABlACAAcABpAGcAZwBlAHIAeQAgAGIAbwB1AG4AZABhAHIAeQBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADkAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAzAFwAbgBNAGEAcwBzACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAYQBwAHAAbABpAGUAZAAgAHQAbwAgAHMAbwBpAGwAcwAgAGYAbwByACAAcwBjAG8AcABlACAAMwAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBNAE4AUwBvAGkAbABfAHMAYwBvAHAAZQAzAFwAbgBrAGcAIABOAFwAbgBNAE4AUwBvAGkAbABfAHsAcwBjAG8AcABlADMAfQA9AFwAXABzAHUAbQBfAHsAagB9AFwAXABzAHUAbQBfAHsAbQB9ACgATQBOAF8AewBqAG0AVAA9ADIAfQBcAFwAdABpAG0AZQBzACgAMQAtAEUARgBfAHsAbQBUAD0AMgB9AC0ARgByAGEAYwBHAEEAUwBNAF8AewBtAFQAPQAyAH0AKQAtAE0ATgBMAGUAYQBjAGgAXwB7AGoAbQA9ADUAfQApAFwAXAB0AGkAbQBlAHMAKAAxAC0AUABGACkAXABuAE0ATgBfAGoAbQBUADIAIAA9ACAAbQBhAHMAcwAgAG8AZgAgAE4AIABpAG4AIABNAE0AUwAgAGEAdAAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMgAgADoAIABrAGcAIABOAFwAbgBFAEYAXwBtAFQAMgAgAD0AIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGUAYQBjAGgAIABNAE0AUwAgAGEAdAAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMgAgADoAIABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOAFwAbgBGAHIAYQBjAEcAQQBTAE0AXwBtAFQAMgAgAD0AIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABhAG4AaQBtAGEAbAAgAHcAYQBzAHQAZQAgAE4AIAB2AG8AbABhAHQAaQBsAGkAcwBlAGQAIABpAG4AIABlAGEAYwBoACAATQBNAFMAIABhAHQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADIAIAA6ACAAKABrAGcAIABOAEgAMwAtAE4AIAArACAATgBPAHgALQBOACkALwBrAGcAIABOAFwAbgBNAE4ATABlAGEAYwBoAF8AagBtADUAIAA9ACAAbQBhAHMAcwAgAG8AZgAgAE4AIABsAG8AcwB0ACAAdABvACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgAgAGYAcgBvAG0AIABkAHIAeQBsAG8AdAAgAE0ATQBTACAAOgAgAGsAZwAgAE4AXABuAFAARgAgAD0AIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABtAGEAbgB1AHIAZQAgAGEAcABwAGwAaQBlAGQAIAB0AG8AIABzAG8AaQBsACAAdwBpAHQAaABpAG4AIAB0AGgAZQAgAHAAaQBnAGcAZQByAHkAIABiAG8AdQBuAGQAYQByAHkAIAA6ACAAZgByAGEAYwB0AGkAbwBuAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADkAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0ATgBfAGoAbQBUADIALAAgAEUARgBfAG0AVAAyACwAIABGAHIAYQBjAEcAQQBTAE0AXwBtAFQAMgAsACAATQBOAEwAZQBhAGMAaABfAGoAbQA1ACwAIABQAEYALABcAG4AIAAgACAAIAAoAE0ATgBfAGoAbQBUADIAIAAqACAAKAAxACAALQAgAEUARgBfAG0AVAAyACAALQAgAEYAcgBhAGMARwBBAFMATQBfAG0AVAAyACkAIAAtACAATQBOAEwAZQBhAGMAaABfAGoAbQA1ACkAIAAqACAAKAAxACAALQAgAFAARgApAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AOQBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AYQBzAHMAIABvAGYAIABuAGkAdAByAG8AZwBlAG4AIABhAHAAcABsAGkAZQBkACAAdABvACAAcwBvAGkAbABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADkAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE4AUwBvAGkAbABfAHMAYwBvAHAAZQAzAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA5AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADkAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgA1AC4AMQAuADkALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMgApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA5AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AOQBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE4AUwBvAGkAbABfAHsAcwBjAG8AcABlADMAfQA9AFwAXABzAHUAbQBfAHsAagB9AFwAXABzAHUAbQBfAHsAbQB9ACgATQBOAF8AewBqAG0AVAA9ADIAfQBcAFwAdABpAG0AZQBzACgAMQAtAEUARgBfAHsAbQBUAD0AMgB9AC0ARgByAGEAYwBHAEEAUwBNAF8AewBtAFQAPQAyAH0AKQAtAE0ATgBMAGUAYQBjAGgAXwB7AGoAbQA9ADUAfQApAFwAXAB0AGkAbQBlAHMAKAAxAC0AUABGACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADkAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAzAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0ATgBfAGoAbQBUADIAXAAiACwAXAAiAG0AYQBzAHMAIABvAGYAIABOACAAaQBuACAATQBNAFMAIABhAHQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADIAXAAiACwAIABcACIAawBnACAATgBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADQALgA1AC4AMQAuADMAIAAoADYAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAF8AbQBUADIAXAAiACwAXAAiAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAZQBhAGMAaAAgAE0ATQBTACAAYQB0ACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAAyAFwAIgAsACAAXAAiAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAHIAYQBjAEcAQQBTAE0AXwBtAFQAMgBcACIALABcACIAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAYQBuAGkAbQBhAGwAIAB3AGEAcwB0AGUAIABOACAAdgBvAGwAYQB0AGkAbABpAHMAZQBkACAAaQBuACAAZQBhAGMAaAAgAE0ATQBTACAAYQB0ACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAAyAFwAIgAsACAAXAAiACgAawBnACAATgBIADMALQBOACAAKwAgAE4ATwB4AC0ATgApAC8AawBnACAATgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0ATgBMAGUAYQBjAGgAXwBqAG0ANQBcACIALABcACIAbQBhAHMAcwAgAG8AZgAgAE4AIABsAG8AcwB0ACAAdABvACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgAgAGYAcgBvAG0AIABkAHIAeQBsAG8AdAAgAE0ATQBTAFwAIgAsACAAXAAiAGsAZwAgAE4AXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAA0AC4ANQAuADEALgA3ACAAKAAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAARgBcACIALABcACIAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAbQBhAG4AdQByAGUAIABhAHAAcABsAGkAZQBkACAAdABvACAAcwBvAGkAbAAgAHcAaQB0AGgAaQBuACAAdABoAGUAIABwAGkAZwBnAGUAcgB5ACAAYgBvAHUAbgBkAGEAcgB5AFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuACIAfQBdACwAIgBwAHIAbwBqAGUAYwB0AE4AYQBtAGUAcwAiADoAWwAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBWAGEAaQByAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAHIAYQB5AEkAbgBUAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAVAB3AG8AQwBvAGwAdQBtAG4AcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHAAbABpAHQAUwB0AHIAaQBuAGcASQBuAHQAbwBBAHIAcgBhAHkAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAEkAdABlAG0ARgByAG8AbQBNAGkAbgBNAGEAeAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAGcAdQBtAGUAbgB0AHMAXwAxAF8AMgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMwBfADQAIgAsACIAQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ARwBlAHQARgByAGEAYwBXAEUAVAAiACwAIgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBIAGEAcgB2AGUAcwB0AEkAbgBkAGUAeAAiACwAIgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBSAGUAcwBpAGQAdQBlAEMAcgBvAHAAUgBhAHQAaQBvACIALAAiAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEMAYQBsAGMAdQBsAGEAdABlAEYAcgBhAGMAdABpAG8AbgBSAGUAcwBpAGQAdQBlAFIAZQBtAG8AdgBlAGQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUALgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBGAGUAZQBkAEkAbgB0AGEAawBlAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUALgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ARgBlAGUAZABJAG4AdABhAGsAZQBfAFUAbgBpAHQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBGAGUAZQBkAEkAbgB0AGEAawBlAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBGAGUAZQBkAEkAbgB0AGEAawBlAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBGAGUAZQBkAEkAbgB0AGEAawBlAF8ARABhAHQAYQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE4AaQB0AHIAbwBnAGUAbgBJAG4AVwBhAHMAdABlAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUALgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATgBpAHQAcgBvAGcAZQBuAEkAbgBXAGEAcwB0AGUAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUALgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATgBpAHQAcgBvAGcAZQBuAEkAbgBXAGEAcwB0AGUAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE4AaQB0AHIAbwBnAGUAbgBJAG4AVwBhAHMAdABlAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBOAGkAdAByAG8AZwBlAG4ASQBuAFcAYQBzAHQAZQBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBGAHIAYQBjAHQAaQBvAG4ATgBWAG8AbABhAHQAaQBsAGkAcwBlAGQAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBGAHIAYQBjAHQAaQBvAG4ATgBWAG8AbABhAHQAaQBsAGkAcwBlAGQAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUALgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ARgByAGEAYwB0AGkAbwBuAE4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBGAHIAYQBjAHQAaQBvAG4ATgBWAG8AbABhAHQAaQBsAGkAcwBlAGQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAEYAcgBhAGMAdABpAG8AbgBOAFYAbwBsAGEAdABpAGwAaQBzAGUAZABfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUALgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUALgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUALgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUALgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATQBNAFMAXwBNAEMARgBzAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUALgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATQBNAFMAXwBNAEMARgBzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE0ATQBTAF8ATQBDAEYAcwBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUALgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATQBNAFMAXwBNAEMARgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBNAE0AUwBfAE0AQwBGAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUALgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8AQQB2AGUAcgBhAGcAZQBMAGkAdgBlAHcAZQBpAGcAaAB0AF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUALgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8AQQB2AGUAcgBhAGcAZQBMAGkAdgBlAHcAZQBpAGcAaAB0AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAEEAdgBlAHIAYQBnAGUATABpAHYAZQB3AGUAaQBnAGgAdABfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUALgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8AQQB2AGUAcgBhAGcAZQBMAGkAdgBlAHcAZQBpAGcAaAB0AF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBBAHYAZQByAGEAZwBlAEwAaQB2AGUAdwBlAGkAZwBoAHQAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUALgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8AUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBzAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUALgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8AUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AcwBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUALgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8AUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUALgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAHIAeQBsAG8AdABNAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARAByAHkAbABvAHQATQBNAFMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBGAHIAYQBjAEwARQBBAEMASABfAEQAcgB5AGwAbwB0AE0ATQBTAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARAByAHkAbABvAHQATQBNAFMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARAByAHkAbABvAHQATQBNAFMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARAByAHkAbABvAHQATQBNAFMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUALgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATQBlAGcAYQBqAG8AdQBsAGUAcwBQAGUAcgBLAGkAbABvAGcAcgBhAG0ATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE0AZQBnAGEAagBvAHUAbABlAHMAUABlAHIASwBpAGwAbwBnAHIAYQBtAE0AZQB0AGgAYQBuAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBNAGUAZwBhAGoAbwB1AGwAZQBzAFAAZQByAEsAaQBsAG8AZwByAGEAbQBNAGUAdABoAGEAbgBlAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE0AZQBnAGEAagBvAHUAbABlAHMAUABlAHIASwBpAGwAbwBnAHIAYQBtAE0AZQB0AGgAYQBuAGUAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE0AZQBnAGEAagBvAHUAbABlAHMAUABlAHIASwBpAGwAbwBnAHIAYQBtAE0AZQB0AGgAYQBuAGUAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE0AZQBnAGEAagBvAHUAbABlAHMAUABlAHIASwBpAGwAbwBnAHIAYQBtAE0AZQB0AGgAYQBuAGUAXwBEAGEAdABhACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAFMAdwBpAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADUAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBTAHcAaQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwA1AF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8AUwB3AGkAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8ANQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAFMAdwBpAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADUAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAFUAbgBpAHQAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8AUwB3AGkAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8ANQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8AUwB3AGkAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8ANQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8AUwB3AGkAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8ANQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBTAHcAaQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwA1AF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBTAHcAaQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwA1AF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8AUwB3AGkAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8ANQBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAFMAdwBpAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADUAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBTAHcAaQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwA1AF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAFMAdwBpAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADUAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAFMAdwBpAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADUAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAFMAdwBpAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADUAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8AUwB3AGkAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8ANQBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBUAGkAdABsAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBVAG4AaQB0ACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAF8AUwBvAHUAcgBjAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADIAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUABlAHIAQwBsAGEAcwBzACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMgBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAGUAcgBDAGwAYQBzAHMAVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAyAF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAZQByAEMAbABhAHMAcwBfAFQAaQB0AGwAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADIAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUABlAHIAQwBsAGEAcwBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMgBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAGUAcgBDAGwAYQBzAHMAXwBVAG4AaQB0ACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMgBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAGUAcgBDAGwAYQBzAHMAXwBTAG8AdQByAGMAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADIAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUABlAHIAQwBsAGEAcwBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAyAF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAZQByAEMAbABhAHMAcwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAyAF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAZQByAEMAbABhAHMAcwBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMgBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAGUAcgBDAGwAYQBzAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADMAXwBTAHQAYQBnAGUAMQBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAzAF8AUwB0AGEAZwBlADEATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADMAXwBTAHQAYQBnAGUAMQBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAzAF8AUwB0AGEAZwBlADEATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA0AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBQAHIAaQBtAGEAcgB5AFMAeQBzAHQAZQBtACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANABfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAUAByAGkAbQBhAHIAeQBTAHkAcwB0AGUAbQBfAFQAaQB0AGwAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADQAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFAAcgBpAG0AYQByAHkAUwB5AHMAdABlAG0AXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA0AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBQAHIAaQBtAGEAcgB5AFMAeQBzAHQAZQBtAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADQAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFAAcgBpAG0AYQByAHkAUwB5AHMAdABlAG0AXwBTAG8AdQByAGMAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADQAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFAAcgBpAG0AYQByAHkAUwB5AHMAdABlAG0AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADQAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFAAcgBpAG0AYQByAHkAUwB5AHMAdABlAG0AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANABfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAUAByAGkAbQBhAHIAeQBTAHkAcwB0AGUAbQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANABfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAUAByAGkAbQBhAHIAeQBTAHkAcwB0AGUAbQBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA1AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADUAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8AVABpAHQAbABlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA1AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAFUAbgBpAHQAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA1AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAFMAbwB1AHIAYwBlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADUAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADUAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADUAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA1AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANgBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADYAXwBTAHQAYQBnAGUAMgBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA2AF8AUwB0AGEAZwBlADIATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANgBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFUAbgBpAHQAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA2AF8AUwB0AGEAZwBlADIATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA2AF8AUwB0AGEAZwBlADIATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA2AF8AUwB0AGEAZwBlADIATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADYAXwBTAHQAYQBnAGUAMgBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADYAXwBTAHQAYQBnAGUAMgBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwBfAE0AZQB0AGgAbwBkADIAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA3AF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFQAcgBhAG4AcwBmAGUAcgByAGUAZABTAHQAYQBnAGUAMgAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADcAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVAByAGEAbgBzAGYAZQByAHIAZQBkAFMAdABhAGcAZQAyAF8AVABpAHQAbABlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANwBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBUAHIAYQBuAHMAZgBlAHIAcgBlAGQAUwB0AGEAZwBlADIAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA3AF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFQAcgBhAG4AcwBmAGUAcgByAGUAZABTAHQAYQBnAGUAMgBfAFUAbgBpAHQAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA3AF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFQAcgBhAG4AcwBmAGUAcgByAGUAZABTAHQAYQBnAGUAMgBfAFMAbwB1AHIAYwBlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANwBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBUAHIAYQBuAHMAZgBlAHIAcgBlAGQAUwB0AGEAZwBlADIAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADcAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVAByAGEAbgBzAGYAZQByAHIAZQBkAFMAdABhAGcAZQAyAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADcAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVAByAGEAbgBzAGYAZQByAHIAZQBkAFMAdABhAGcAZQAyAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABEAGkAcgBlAGMAdABOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAE0ATQBTACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwARABpAHIAZQBjAHQATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBNAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0ATQBNAFMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABEAGkAcgBlAGMAdABOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0ATQBNAFMAXwBTAG8AdQByAGMAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0ATQBNAFMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0ATQBNAFMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwARABpAHIAZQBjAHQATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBNAE0AUwBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADIAXwBTAHQAYQBnAGUAMQBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADIAXwBTAHQAYQBnAGUAMQBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAF8AVABpAHQAbABlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADIAXwBTAHQAYQBnAGUAMQBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADIAXwBTAHQAYQBnAGUAMQBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwAyAF8AUwB0AGEAZwBlADEATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADIAXwBTAHQAYQBnAGUAMQBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8AMgBfAFMAdABhAGcAZQAxAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADIAXwBTAHQAYQBnAGUAMQBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8AMwBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEkAbgBQAHIAaQBtAGEAcgB5AE0ATQBTACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADMAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBJAG4AUAByAGkAbQBhAHIAeQBNAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwAzAF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ASQBuAFAAcgBpAG0AYQByAHkATQBNAFMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8AMwBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEkAbgBQAHIAaQBtAGEAcgB5AE0ATQBTAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwAzAF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ASQBuAFAAcgBpAG0AYQByAHkATQBNAFMAXwBTAG8AdQByAGMAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwAzAF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ASQBuAFAAcgBpAG0AYQByAHkATQBNAFMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwAzAF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ASQBuAFAAcgBpAG0AYQByAHkATQBNAFMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADMAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBJAG4AUAByAGkAbQBhAHIAeQBNAE0AUwBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADQAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBJAG4AUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8ANABfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEkAbgBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA0AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ASQBuAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8AVABpAHQAbABlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADQAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBJAG4AUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8ANABfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEkAbgBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAFUAbgBpAHQAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8ANABfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEkAbgBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAFMAbwB1AHIAYwBlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADQAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBJAG4AUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA0AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ASQBuAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA0AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ASQBuAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA0AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ASQBuAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8ANABfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEkAbgBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADUAXwBBAG4AbgB1AGEAbABOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAaQBvAG4AIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8ANQBfAEEAbgBuAHUAYQBsAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBfAFQAaQB0AGwAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA1AF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADUAXwBBAG4AbgB1AGEAbABOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADUAXwBBAG4AbgB1AGEAbABOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA1AF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8ANQBfAEEAbgBuAHUAYQBsAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8ANQBfAEEAbgBuAHUAYQBsAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADYAXwBTAHQAYQBnAGUAMgBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADYAXwBTAHQAYQBnAGUAMgBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAF8AVABpAHQAbABlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADYAXwBTAHQAYQBnAGUAMgBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADYAXwBTAHQAYQBnAGUAMgBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA2AF8AUwB0AGEAZwBlADIATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADYAXwBTAHQAYQBnAGUAMgBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8ANgBfAFMAdABhAGcAZQAyAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADYAXwBTAHQAYQBnAGUAMgBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8ANwBfAE4AaQB0AHIAbwBnAGUAbgBUAHIAYQBuAHMAZgBlAHIAcgBlAGQAVABvAFMAdABhAGcAZQAyAE0ATQBTACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADcAXwBOAGkAdAByAG8AZwBlAG4AVAByAGEAbgBzAGYAZQByAHIAZQBkAFQAbwBTAHQAYQBnAGUAMgBNAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA3AF8ATgBpAHQAcgBvAGcAZQBuAFQAcgBhAG4AcwBmAGUAcgByAGUAZABUAG8AUwB0AGEAZwBlADIATQBNAFMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8ANwBfAE4AaQB0AHIAbwBnAGUAbgBUAHIAYQBuAHMAZgBlAHIAcgBlAGQAVABvAFMAdABhAGcAZQAyAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA3AF8ATgBpAHQAcgBvAGcAZQBuAFQAcgBhAG4AcwBmAGUAcgByAGUAZABUAG8AUwB0AGEAZwBlADIATQBNAFMAXwBTAG8AdQByAGMAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA3AF8ATgBpAHQAcgBvAGcAZQBuAFQAcgBhAG4AcwBmAGUAcgByAGUAZABUAG8AUwB0AGEAZwBlADIATQBNAFMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA3AF8ATgBpAHQAcgBvAGcAZQBuAFQAcgBhAG4AcwBmAGUAcgByAGUAZABUAG8AUwB0AGEAZwBlADIATQBNAFMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADcAXwBOAGkAdAByAG8AZwBlAG4AVAByAGEAbgBzAGYAZQByAHIAZQBkAFQAbwBTAHQAYQBnAGUAMgBNAE0AUwBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADUAXwBfADEAXwBBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAE0ATQBTACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADUAXwBfADEAXwBBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAE0ATQBTAF8AVABpAHQAbABlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADUAXwBfADEAXwBBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAE0ATQBTAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADUAXwBfADEAXwBBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA1AF8AXwAxAF8AQQBuAG4AdQBhAGwAQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBNAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADUAXwBfADEAXwBBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAE0ATQBTAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANQBfAF8AMQBfAEEAbgBuAHUAYQBsAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0ATQBNAFMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADUAXwBfADEAXwBBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAE0ATQBTAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANQBfAF8AMgBfAFQAbwB0AGEAbABOAGkAdAByAG8AZwBlAG4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAEYAcgBvAG0ATQBNAFMAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANQBfAF8AMgBfAFQAbwB0AGEAbABOAGkAdAByAG8AZwBlAG4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAEYAcgBvAG0ATQBNAFMAXwBUAGkAdABsAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANQBfAF8AMgBfAFQAbwB0AGEAbABOAGkAdAByAG8AZwBlAG4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAEYAcgBvAG0ATQBNAFMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANQBfAF8AMgBfAFQAbwB0AGEAbABOAGkAdAByAG8AZwBlAG4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAEYAcgBvAG0ATQBNAFMAXwBVAG4AaQB0ACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADUAXwBfADIAXwBUAG8AdABhAGwATgBpAHQAcgBvAGcAZQBuAFYAbwBsAGEAdABpAGwAaQBzAGUAZABGAHIAbwBtAE0ATQBTAF8AUwBvAHUAcgBjAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANQBfAF8AMgBfAFQAbwB0AGEAbABOAGkAdAByAG8AZwBlAG4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAEYAcgBvAG0ATQBNAFMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA1AF8AXwAyAF8AVABvAHQAYQBsAE4AaQB0AHIAbwBnAGUAbgBWAG8AbABhAHQAaQBsAGkAcwBlAGQARgByAG8AbQBNAE0AUwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANQBfAF8AMgBfAFQAbwB0AGEAbABOAGkAdAByAG8AZwBlAG4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAEYAcgBvAG0ATQBNAFMAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANwBfAF8AMQBfAEEAbgBuAHUAYQBsAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEYAcgBvAG0ATQBNAFMAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADcAXwBfADEAXwBBAG4AbgB1AGEAbABFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBGAHIAbwBtAE0ATQBTAF8AVABpAHQAbABlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA3AF8AXwAxAF8AQQBuAG4AdQBhAGwARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARgByAG8AbQBNAE0AUwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANwBfAF8AMQBfAEEAbgBuAHUAYQBsAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEYAcgBvAG0ATQBNAFMAXwBVAG4AaQB0ACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA3AF8AXwAxAF8AQQBuAG4AdQBhAGwARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARgByAG8AbQBNAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA3AF8AXwAxAF8AQQBuAG4AdQBhAGwARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARgByAG8AbQBNAE0AUwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA3AF8AXwAxAF8AQQBuAG4AdQBhAGwARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARgByAG8AbQBNAE0AUwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADcAXwBfADEAXwBBAG4AbgB1AGEAbABFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBGAHIAbwBtAE0ATQBTAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADcAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAG8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEYAcgBvAG0ARAByAHkAbABvAHQATQBNAFMAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADcAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAG8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEYAcgBvAG0ARAByAHkAbABvAHQATQBNAFMAXwBUAGkAdABsAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADcAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAG8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEYAcgBvAG0ARAByAHkAbABvAHQATQBNAFMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADcAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAG8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEYAcgBvAG0ARAByAHkAbABvAHQATQBNAFMAXwBVAG4AaQB0ACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA3AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABvAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBGAHIAbwBtAEQAcgB5AGwAbwB0AE0ATQBTAF8AUwBvAHUAcgBjAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADcAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAG8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEYAcgBvAG0ARAByAHkAbABvAHQATQBNAFMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANwBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAbwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARgByAG8AbQBEAHIAeQBsAG8AdABNAE0AUwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADcAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAG8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEYAcgBvAG0ARAByAHkAbABvAHQATQBNAFMAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AYQBuAHUAcgBlAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AOQBfAF8AMQBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADEAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGEAbgB1AHIAZQBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADkAXwBfADEAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAxAF8AVABpAHQAbABlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBhAG4AdQByAGUAQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA5AF8AXwAxAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AYQBuAHUAcgBlAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AOQBfAF8AMQBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADEAXwBVAG4AaQB0ACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBhAG4AdQByAGUAQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA5AF8AXwAxAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMQBfAFMAbwB1AHIAYwBlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBhAG4AdQByAGUAQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA5AF8AXwAxAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBhAG4AdQByAGUAQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA5AF8AXwAxAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGEAbgB1AHIAZQBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADkAXwBfADEAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAxAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGEAbgB1AHIAZQBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADkAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAzACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBhAG4AdQByAGUAQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA5AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMwBfAFQAaQB0AGwAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AYQBuAHUAcgBlAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AOQBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGEAbgB1AHIAZQBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADkAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAzAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AYQBuAHUAcgBlAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AOQBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADMAXwBTAG8AdQByAGMAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AYQBuAHUAcgBlAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AOQBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AYQBuAHUAcgBlAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AOQBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBhAG4AdQByAGUAQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA5AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMwBfAEEAcgBnAHUAbQBlAG4AdABzACIAXQAsACIAbABvAGMAYQBsAGUAIgA6AHsAIgBsAGkAcwB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAcgBvAHcAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBjAG8AbAB1AG0AbgBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUABvAHMAaQB0AGkAbwBuAHMAIgA6AFsAMwBdACwAIgBkAGUAYwBpAG0AYQBsAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiAC4AIgAsACIAZABhAHQAZQBPAHIAZABlAHIAIgA6ACIARABNAFkAIgAsACIAYwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsACIAOgAiACQAIgAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbABMAGUAYQBkACIAOgB0AHIAdQBlACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAZQBwAEIAeQBTAHAAYQBjAGUAIgA6AGYAYQBsAHMAZQAsACIAcgBvAHcATABlAHQAdABlAHIAIgA6ACIAUgAiACwAIgBjAG8AbAB1AG0AbgBMAGUAdAB0AGUAcgAiADoAIgBDACIALAAiAHIAYwBMAGUAZgB0AEIAcgBhAGMAawBlAHQAIgA6ACIAWwAiACwAIgByAGMAUgBpAGcAaAB0AEIAcgBhAGMAawBlAHQAIgA6ACIAXQAiACwAIgBzAHQAYQB0AGUAbQBlAG4AdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGwAbwBjAGEAbABlAE4AYQBtAGUAIgA6ACIAZQBuAC0AdQBzACIAfQB9AA==</AFEJSONBlob>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100ACB660BB23738846A00119B5826AC974" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3e3613359d4ae7f6bda6c57be713f101">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7291119c-fce9-4911-96ae-b800be5dccd8" xmlns:ns3="09eef6d6-daa8-4301-8f9f-b1ec38079286" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87491bfad7f11426ad96486e70428b3e" ns2:_="" ns3:_="">
     <xsd:import namespace="7291119c-fce9-4911-96ae-b800be5dccd8"/>
@@ -19284,34 +19260,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
-    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgAFwAdQAwADAAMgA3AEYAcgB5AFwAdQAwADAAMgA3ACAAdABvACAAXAB1ADAAMAAyADcARAByAHkAXAB1ADAAMAAyADcALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIAVwBlAHQAIABvAHIAIABEAHIAeQAgAFoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAGkAbgAgAE0AQQBUACAAdgBhAGwAdQBlACAAZgBvAHIAIAB3AGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABjAGgAYQBuAGcAZQBkACAAMQAwACAAdABvACAAMQAxAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAG0AaQBuACAAYQBuAGQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIABmAG8AcgAgAE0AQQBUACwAIABNAEEAUAAsACAAZgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgAsACAAZQBsAGUAdgBhAHQAaQBvAG4ALAAgAE0AQQBQADoAUABFAFQAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAcwAgAGYAcgBvAG0AIAByAGUAYQBsACAAYwBsAGkAbQBhAHQAZQAgAGQAYQB0AGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBBAEYAIABhAGMAYwBlAHAAdABzACAAcgBhAGkAbgBmAGEAbABsACAAYQBzACAAYQAgAHAAcgBvAHgAeQAgAGYAbwByACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUAFwAIgAsACAAXAAiAE0AQQBQAFwAIgAsACAAXAAiAEYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIAXAAiACwAIABcACIARQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAHQAZQBtAHAAXAAiACwAIABcACIATQBhAHgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AaQBuACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AYQB4ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AaQBuACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGEAeAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBpAG4AIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGEAeAAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADIAMAAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAG0AIAAtACAAZCIgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwAC4AMAAwADEALAAgADIAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0AGUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFQAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAUAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEUAVAAgAD0AIABwAG8AdABlAG4AdABpAGEAbAAgAGUAdgBhAHAAbwB0AHIAYQBuAHMAcABpAHIAYQB0AGkAbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAE0AQQBUACAAbQBpAG4AIABhAG4AZAAgAE0AQQBUACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AZQBkAGkAYQBuACAAQQBuAG4AdQBhAGwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAAoAE0AQQBUACkAXAAiACwAIABcACIATQBpAG4AIABNAEEAVABcACIALAAgAFwAIgBNAGEAeAAgAE0AQQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiIAAyADYAIABDAFwAIgAsACAAMgA2ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgAFwAIgAxADUAIAAtACAAMgA1ACAAQwBcACIALAAgADEANQAsACAAMgA1AC4AOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIiAAMQA0ACAAQwBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEANAAuADkAOQA5AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABaAG8AbgBlAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAXAB1ADAAMAAzAGUAIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAXAB1ADAAMAAzAGUAowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABkAG8AZQBzACAAbgBvAHQAIABvAGMAYwB1AHIAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAGQiowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBzACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAWQBlAHMAIAAtACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvACAALQAgAG4AbwB0ACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAZABhAHQAYQAgAHMAYwBvAHIAZQBzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFgAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAdABhACAAcwBvAHUAcgBjAGUAXAAiACwAIABcACIARABhAHQAYQAgAHMAYwBvAHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBuAHQAZQByAG4AYQB0AGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUAIABvAHIAIAByAGUAZwBpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGkAbgB0AGUAbgBzAGkAdAB5ACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIABhAHAAcAByAG8AdgBlAGQAIABtAGUAdABoAG8AZABcACIALAAgADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBlAHIAaQBmAGkAZQBkACAAYwByAGUAZABlAG4AdABpAGEAbAAgAG0AYQB0AGMAaABpAG4AZwAgAEkAUwBPADEANAAwADYANwBcACIALAAgADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAAoADMALgBEAC4AYgAuADIAKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBMAEUAQQBDAEgAXAAiACwAMAAuADIANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABFAHEAdQBhAHQAaQBvAG4AIAAzAC4ARAAuAEIAXwAxADAAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAGwAZQBhAGMAaABcACIALAAwAC4AMAAxADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcAG4ATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADQALAAgADUALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAGoAXAAiACwAXAAiAEUARgBOADIATwBcACIALAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5AFwAIgAsACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAA1ADkALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAXAAiACwAMAAuADAAMAA3ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABsAG8AdwAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAMgA5ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAOAAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAMAAuADAAMQA5ADkALAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsADAALgAwADAANQAzACwAIABcACIAQwBvAHQAdABvAG4AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAMAAuADAAMAA2ADQALAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABjAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnACkAXAAiACwAMAAuADAAMAAzACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBDAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABzAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnACkAXAAiACwAMAAuADAAMAA1ACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBTAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAMAAuADAAMAAyADYALAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABkAHUAcABsAGkAYwBhAHQAZQAgAFwAdQAwADAAMgA3AEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcAHUAMAAwADIANwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcAcAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcAHUAMAAwADIANwAsACAAXAB1ADAAMAAyADcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcAHUAMAAwADIANwAgAGEAbgBkACAAXAB1ADAAMAAyADcAaQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AG4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAdQAwADAAMgA3ACAAcgBvAHcAIAB3AGkAdABoACAAcwBhAG0AZQAgAEUARgAgAGYAbwByACAAbABvAHcAIABhAG4AZAAgAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXABuAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXABuAEkAUABDAEMAOgAgAE4AMgBPACAARQBNAEkAUwBTAEkATwBOAFMAIABGAFIATwBNACAATQBBAE4AQQBHAEUARAAgAFMATwBJAEwAUwAsACAAQQBOAEQAIABDAE8AMgAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAEwASQBNAEUAIABBAE4ARAAgAFUAUgBFAEEAIABBAFAAUABMAEkAQwBBAFQASQBPAE4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAFcARQBUACAAZgBvAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBkAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAQwBoAGEAcAB0AGUAcgAgADEALAAgAHMAZQBjAHQAaQBvAG4AIAAxAC4AOAAuADIAIABMAGUAYQBjAGgAaQBuAGcALAAgAGMAbABpAG0AYQB0AGUAIABhAG4AZAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEkAUABDAEMAIAAyADAAMQA5ACAAUgBlAGYAaQBuAGUAbQBlAG4AdAAgAFYAbwBsAHUAbQBlACAANAA6ACAAQwBoAGEAcAB0AGUAcgAgADEAMQA6ACAATgAyAE8AIABFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABNAGEAbgBhAGcAZQBkACAAUwBvAGkAbABzACwAIABhAG4AZAAgAEMATwAyACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATABpAG0AZQAgAGEAbgBkACAAVQByAGUAYQAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIAB0AHkAcABlACAAaQByAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAaQBwACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBwAHIAaQBuAGsAbABlAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAcgBmAGEAYwBlACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwB0AGgAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABUAGEAYgBsAGUAIABjAHIAZQBhAHQAZQBkACAAYgBhAHMAZQBkACAAbwBuACAAVgBFAEUAUgBHACAAdABlAHgAdAAgAFwAdQAwADAAMgA3AEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuAFwAdQAwADAAMgA3AFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAOgAgAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAFAAUgBQACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAFAAUgBQAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEMAaABhAG4AZwBlAGQAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAB1ADAAMAAyADcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAdQAwADAAMgA3ACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AbwBuAHQAaABzACAAdABvACAAUwBlAGEAcwBvAG4AcwAgAE0AYQBwAHAAaQBuAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAG8AbgB0AGgAXAAiACwAIABcACIAUwBlAGEAcwBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAYQBuAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAZQBiAHIAdQBhAHIAeQBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAHIAYwBoAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHAAcgBpAGwAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQB5AFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbgBlAFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbAB5AFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAZwB1AHMAdABcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAHAAdABlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AYwB0AG8AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB2AGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABlAGMAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAbgB1AHIAZQAgAE0AYQBuAGEAZwBlAG0AZQBuAHQAIAATICAATQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHAAZQByACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGkAbQApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgA4AC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAxACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAIAAoALoAQwApAFwAIgAsACAAXAAiAFUAbgBjAG8AdgBlAHIAZQBkACAAYQBuAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAUwBsAHUAcgByAHkAIAAoAHcAaQB0AGgAbwB1AHQAIABuAGEAdAB1AHIAYQBsACAAYwByAHUAcwB0ACkAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAGIAKQBcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABTAHQAbwByAGEAZwBlACAAXAB1ADAAMAAzAGMAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AFAAbwB1AGwAdAByAHkAIAB3AGkAdABoACAAYQBuAGQAIAB3AGkAdABoAG8AdQB0ACAAbABpAHQAdABlAHIAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHcAaQB0AGgAIABzAGUAcABhAHIAYQB0AGUAIABOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE0AQQBUACAAcgBhAHcAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAbABsAG8AdwAgAGwAbwBvAGsAdQBwACAAbwBmACAAbgB1AG0AYgBlAHIAcwAuAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBuAGQAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAcgBlAHQAdQByAG4AZQBkACAAdABvACAAdABoAGUAIABzAG8AaQBsAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYATgBpACAAXAB1ADAAMAAyADYAIABFAEYATgAyAE8AaQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADEALgA0AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBOAGkAIABcAHUAMAAwADIANgAgAEUARgBOADIATwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAE4AMgBPACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUATgAyAE8AOgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXABuAEcAVwBQAE4AMgBPADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBOADIATwAsACAARwBXAFAAXwBOADIATwAsAFwAbgAgACAAIAAgAEUAXwBOADIATwAgACoAIABHAFcAUABfAE4AMgBPAFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAE4AMgBPACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AE4AMgBPAH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AE4AMgBPAH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBOADIATwBcACIALABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAATgAyAE8AXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAEMASAA0ACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUAQwBIADQAOgAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXABuAEcAVwBQAEMASAA0ADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBDAEgANAAsACAARwBXAFAAXwBDAEgANAAsAFwAbgAgACAAIAAgAEUAXwBDAEgANAAgACoAIABHAFcAUABfAEMASAA0AFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEMASAA0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AEMASAA0AH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AEMASAA0AH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBDAEgANABcACIALABcACIATQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAAQwBIADQAXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQAgAGQAYQB0AGEAIAB0AGgAYQB0ACAAaQBzACAAYwBvAG0AbQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAbABpAHYAZQBzAHQAbwBjAGsAIAB0AHkAcABlAHMAXABuAEUAeABjAGUAbAAgAG0AbwBkAHUAbABlACAAbgBhAG0AZQA6ACAAUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlADoAIABOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcAG4ATgBJAFIAXwAyADAAMgAzAF8AVgBvAGwAMQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBcAG4ARgByAGEAYwBXAEUAVABNAE0AUwBpACAAPQAgAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4AKABUAGEAYgBsAGUAIABBADUALgA1AC4AMQAwAC4AMgAgAGkAcwAgAHIAZQBmAGUAcgBlAG4AYwBlAGQAIABpAG4AIABOAEkAUgAgAGIAdQB0ACAAMQAgAGkAcwAgAHUAcwBlAGQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAxACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXABuAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTACAAPQAgADAALgAwADIAIAAoAEcAZwAgAE4ALwBHAGcAIABhAHAAcABsAGkAZQBkACkAIAAoAEMAUwAgAEUARgAsACAAcwBvAHUAcgBjAGUAIABJAFAAQwBDACAAKAAyADAAMQA5ACkAKQAgAFwAbgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAbABvAHMAdAAgAHQAaAByAG8AdQBnAGgAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABsAG8AcwB0ACAAdABoAHIAbwB1AGcAaAAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA4ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAIAAwAC4AMAAwADUAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwAFwAIgAsACAAMAAuADAAMAA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAgADAALgAwADAAMQA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcABcACIALAAgADAALgAwADAANAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAIABjAGEAbgBlAFwAIgAsACAAMAAuADAAMQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsACAAMAAuADAAMAA1ADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBlAFwAIgAsACAAMAAuADAAMAA2ADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXABuAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVgBhAGkAcgBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE0AUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAAVABhAGIAbABlACAANQAuADEAMgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAOQAsACAAMwAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB5AG0AYgBvAGwAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgAgACgAbQA9ADEAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADIAXAAiACwAIABcACIATABpAHEAdQBpAGQAIABzAHkAcwB0AGUAbQBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwAgACgAbQA9ADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADMAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAG0APQAzACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGEAXAAiACwAIABcACIAUwB1AG0AcAAgAGEAbgBkACAAZABpAHMAcABlAHIAcwBhAGwAIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbAAgAHMAeQBzAHQAZQBtACAAKABtAD0AMwBhACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGIAXAAiACwAIABcACIARAByAGEAaQBuAHMAIAB0AG8AIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAEQAcgBhAGkAbgBzACAAdABvACAAcABhAGQAZABvAGMAawAgACgAbQA9ADMAYgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIANABcACIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAIAAoAG0APQA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA1AFwAIgAsACAAXAAiAEQAcgB5AGwAbwB0ACAAKABmAGUAZQBkACAAcABhAGQAKQBcACIALAAgAFwAIgBEAHIAeQBsAG8AdAAgACgAZgBlAGUAZAAgAHAAYQBkACkAIAAoAG0APQA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA2AFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQAgACgAbQA9ADYAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADcAXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEQAaQBnAGUAcwB0AGUAcgAgAC8AIABjAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AcwAgACgAbQA9ADcAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADgAXAAiACwAIABcACIARABlAGUAcAAgAGwAaQB0AHQAZQByAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgAgACgAbQA9ADgAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADkAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQAgACgAbQA9ADkAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMABcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwAgACgAbQA9ADEAMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnACAAKABtAD0AMQAxACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADEAYQBcACIALAAgAFwAIgBCAGUAbAB0ACAAbQBhAG4AdQByAGUAIAByAGUAbQBvAHYAYQBsAFwAIgAsACAAXAAiAEIAZQBsAHQAIABtAGEAbgB1AHIAZQAgAHIAZQBtAG8AdgBhAGwAIAAoAG0APQAxADEAYQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAGIAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABzAHQAbwByAGUAZAAgAGkAbgAgAGgAbwB1AHMAZQBcACIALAAgAFwAIgBNAGEAbgB1AHIAZQAgAHMAdABvAHIAZQBkACAAaQBuACAAaABvAHUAcwBlACAAKABtAD0AMQAxAGIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAKABtAD0AMQAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADMAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAAoAG0APQAxADMAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEANABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACAAcgBhAG4AZwBlACAAYQBuAGQAIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAIAAoAG0APQAxADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQgBlAGUAZgAgAGMAYQB0AHQAbABlACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBfAFYAYQBpAHIAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAaQBmAGUAYwB5AGMAbABlAHMALgAgACgAMgAwADIANgApAC4AIABHAHIAZQBlAG4AaABvAHUAcwBlACAARwBhAHMAIABFAG0AaQBzAHMAaQBvAG4AIABJAG4AdABlAG4AcwBpAHQAaQBlAHMAIABmAG8AcgAgAE0AYQB0AGUAcgBpAGEAbAAgAEkAbgBwAHUAdABzACAAdABvACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAEEAZwByAGkAYwB1AGwAdAB1AHIAZQAsACAARgBpAHMAaABlAHIAaQBlAHMAIABhAG4AZAAgAEYAbwByAGUAcwB0AHIAeQAuACAAVgBlAHIAcwBpAG8AbgAgADQAOAAuACAAZABvAGkAIAAxADAALgA1ADIAOAAxAC8AegBlAG4AbwBkAG8ALgAxADkANgA1ADYANQA4ADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAXAAiACwAIABcACIAUwBvAHUAcgBjAGUAIAByAGUAZwBpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAYQB0AHQAbABlACwAIABmAG8AcgAgAG0AYQBuAHUAZgBhAGMAdAB1AHIAaQBuAGcAIABiAGUAZQBmAFwAIgAsACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBhAHQAdABsAGUALAAgAGYAbwByACAAcAByAGkAbQBlACAAYgBlAGUAZgBcACIALAAgAFwAIgBOAFMAVwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAYQB0AHQAbABlACwAIAB3AGUAYQBuAGUAcgBzAFwAIgAsACAAXAAiAE4AVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFEATABEAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAVABBAFMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBWAEkAQwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFcAQQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBDAGgAaQBjAGsAZQBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEMAaABpAGMAawBlAG4AcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBoAGkAYwBrAGUAbgBzACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQwBoAGkAYwBrAGUAbgBzAF8AVgBhAGkAcgBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEMAaABpAGMAawBlAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQwBoAGkAYwBrAGUAbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAaQBmAGUAYwB5AGMAbABlAHMALgAgACgAMgAwADIANgApAC4AIABHAHIAZQBlAG4AaABvAHUAcwBlACAARwBhAHMAIABFAG0AaQBzAHMAaQBvAG4AIABJAG4AdABlAG4AcwBpAHQAaQBlAHMAIABmAG8AcgAgAE0AYQB0AGUAcgBpAGEAbAAgAEkAbgBwAHUAdABzACAAdABvACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAEEAZwByAGkAYwB1AGwAdAB1AHIAZQAsACAARgBpAHMAaABlAHIAaQBlAHMAIABhAG4AZAAgAEYAbwByAGUAcwB0AHIAeQAuACAAVgBlAHIAcwBpAG8AbgAgADQAOAAuACAAZABvAGkAIAAxADAALgA1ADIAOAAxAC8AegBlAG4AbwBkAG8ALgAxADkANgA1ADYANQA4ADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBDAGgAaQBjAGsAZQBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUAByAG8AZAB1AGMAdABcACIALAAgAFwAIgBTAG8AdQByAGMAZQAgAHIAZQBnAGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBoAGkAYwBrAGUAbgBzAFwAIgAsACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEQAYQBpAHIAeQBjAGEAdAB0AGwAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIABwAHIAbwBkAHUAYwB0AHMAIABmAG8AcgAgAHMAYwBvAHAAZQAgADMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXwBWAGEAaQByAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8ARABhAGkAcgB5AGMAYQB0AHQAbABlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATABpAGYAZQBjAHkAYwBsAGUAcwAuACAAKAAyADAAMgA2ACkALgAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABHAGEAcwAgAEUAbQBpAHMAcwBpAG8AbgAgAEkAbgB0AGUAbgBzAGkAdABpAGUAcwAgAGYAbwByACAATQBhAHQAZQByAGkAYQBsACAASQBuAHAAdQB0AHMAIAB0AG8AIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAQQBnAHIAaQBjAHUAbAB0AHUAcgBlACwAIABGAGkAcwBoAGUAcgBpAGUAcwAgAGEAbgBkACAARgBvAHIAZQBzAHQAcgB5AC4AIABWAGUAcgBzAGkAbwBuACAANAA4AC4AIABkAG8AaQAgADEAMAAuADUAMgA4ADEALwB6AGUAbgBvAGQAbwAuADEAOQA2ADUANgA1ADgAMABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEQAYQBpAHIAeQBjAGEAdAB0AGwAZQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AFwAIgAsACAAXAAiAFMAbwB1AHIAYwBlACAAcgBlAGcAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAaQByAHkAIABjAG8AdwBzAFwAIgAsACAAXAAiAFYASQBDAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBQAGkAZwBzACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUABpAGcAcwBfAFYAYQBpAHIAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAaQBmAGUAYwB5AGMAbABlAHMALgAgACgAMgAwADIANgApAC4AIABHAHIAZQBlAG4AaABvAHUAcwBlACAARwBhAHMAIABFAG0AaQBzAHMAaQBvAG4AIABJAG4AdABlAG4AcwBpAHQAaQBlAHMAIABmAG8AcgAgAE0AYQB0AGUAcgBpAGEAbAAgAEkAbgBwAHUAdABzACAAdABvACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAEEAZwByAGkAYwB1AGwAdAB1AHIAZQAsACAARgBpAHMAaABlAHIAaQBlAHMAIABhAG4AZAAgAEYAbwByAGUAcwB0AHIAeQAuACAAVgBlAHIAcwBpAG8AbgAgADQAOAAuACAAZABvAGkAIAAxADAALgA1ADIAOAAxAC8AegBlAG4AbwBkAG8ALgAxADkANgA1ADYANQA4ADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAXAAiACwAIABcACIAUwBvAHUAcgBjAGUAIAByAGUAZwBpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAaQBnAHMAXAAiACwAIABcACIAQQB1AHMAdAByAGEAbABpAGEAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUwBoAGUAZQBwAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBTAGgAZQBlAHAAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFMAaABlAGUAcAAgAHAAcgBvAGQAdQBjAHQAcwAgAGYAbwByACAAcwBjAG8AcABlACAAMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFMAaABlAGUAcABfAFYAYQBpAHIAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBTAGgAZQBlAHAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFMAaABlAGUAcABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBMAGkAZgBlAGMAeQBjAGwAZQBzAC4AIAAoADIAMAAyADYAKQAuACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAEcAYQBzACAARQBtAGkAcwBzAGkAbwBuACAASQBuAHQAZQBuAHMAaQB0AGkAZQBzACAAZgBvAHIAIABNAGEAdABlAHIAaQBhAGwAIABJAG4AcAB1AHQAcwAgAHQAbwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABBAGcAcgBpAGMAdQBsAHQAdQByAGUALAAgAEYAaQBzAGgAZQByAGkAZQBzACAAYQBuAGQAIABGAG8AcgBlAHMAdAByAHkALgAgAFYAZQByAHMAaQBvAG4AIAA0ADgALgAgAGQAbwBpACAAMQAwAC4ANQAyADgAMQAvAHoAZQBuAG8AZABvAC4AMQA5ADYANQA2ADUAOAAwAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUwBoAGUAZQBwAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAXAAiACwAIABcACIAUwBvAHUAcgBjAGUAIAByAGUAZwBpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAaABlAGUAcAAsACAAZgBvAHIAIABtAHUAdAB0AG8AbgBcACIALAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAaABlAGUAcAAsACAAZgBvAHIAIABwAHIAaQBtAGUAIABsAGEAbQBiAFwAIgAsACAAXAAiAE4AUwBXAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAUQBMAEQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBTAEEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFYASQBDAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAVwBBAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFIATwBXACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwAKQAgACsAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACAALQAgADEAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAVABhAGIAbABlAEgAZQBhAGQAZQByAEMAZQBsAGwALABcAG4AIAAgAEMATwBMAFUATQBOACgAVABhAGIAbABlAEgAZQBhAGQAZQByAEMAZQBsAGwAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAHIAYQB5AEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIABBAHIAcgBhAHkARABhAHQAYQAsACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkALAAgAFsAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQBdACwAXABuACAASQBGAEUAUgBSAE8AUgAoAFwAbgAgACAAIAAgACAASQBOAEQARQBYACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFUATgBJAFEAVQBFACgAQQByAHIAYQB5AEQAYQB0AGEAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIATwBXACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABDAE8ATABVAE0ATgAoACkALQBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5ACkALAAgADEALAAgAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALAAgAFwAIgBcACIAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABJAEYAKABJAFMATgBVAE0AQgBFAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkAXABuACAAIAAgACAAKQAsACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQAsACAAMAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAVAB3AG8AQwBvAGwAdQBtAG4AcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkARgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIAAoAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlADEAKQAqACgATABvAG8AawB1AHAAQQByAHIAYQB5ADIAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgApACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAVgBhAGwAdQBlAEkARgBGAGEAbABzAGUAKQAsACAAXAAiAFwAIgAsACAAVgBhAGwAdQBlAEkARgBGAGEAbABzAGUAKQApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATwBuAGUAQwBvAGwAdQBtAG4AQQBuAGQASABlAGEAZABlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABbAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlAF0ALABcAG4AIAAgACAAIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBmAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBmAEYAYQBsAHMAZQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHAAbABpAHQAUwB0AHIAaQBuAGcASQBuAHQAbwBBAHIAcgBhAHkAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABDAGUAbABsACwAIABEAGUAbABpAG0AaQB0AGUAcgAsACAAWwBDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQBdACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyAF0ALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSAFgATQBMACgAXABuACAAIAAgACAAIAAgACAAIABcACIAXAB1ADAAMAAzAGMAdABcAHUAMAAwADMAZQBcAHUAMAAwADMAYwBzAFwAdQAwADAAMwBlAFwAIgAgAFwAdQAwADAAMgA2AFwAbgAgACAAIAAgACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAUwBVAEIAUwBUAEkAVABVAFQARQAoAEMAZQBsAGwALABDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQAsAFwAIgBcACIAKQAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEQAZQBsAGkAbQBpAHQAZQByACwAXAAiAFwAdQAwADAAMwBjAC8AcwBcAHUAMAAwADMAZQBcAHUAMAAwADMAYwBzAFwAdQAwADAAMwBlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgACkAIABcAHUAMAAwADIANgBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcAHUAMAAwADMAYwAvAHMAXAB1ADAAMAAzAGUAXAB1ADAAMAAzAGMALwB0AFwAdQAwADAAMwBlAFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAC8ALwBzAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAYQB2AGcAVABlAG0AcAAsAGEAdgBnAFIAYQBpAG4ALABmAHIAbwBzAHQARABhAHkAcwAsAGUAbABlAHYALABtAGEAcABfAHAAZQB0ACwAXABuACAAIAAgACAAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkALABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQAsAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABtAGEAeABFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBQAEUAVABBAHIAcgBhAHkALABtAGEAeABQAEUAVABBAHIAcgBhAHkALABcAG4AIAAgACAAIABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AGEAdgBnAFQAZQBtAHAAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBhAHYAZwBSAGEAaQBuACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AZgByAG8AcwB0AEQAYQB5AHMAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABGAHIAbwBzAHQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AZQBsAGUAdgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AZQBsAGUAdgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAFAARQBUAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AbQBhAHAAXwBwAGUAdAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFAARQBUAEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AbQBhAHAAXwBwAGUAdAApACwAXABuACAAIAAgACAAIAAgACAAIABUAEEASwBFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgAYwBsAGkAbQBhAHQAZQBaAG8AbgBlAEEAcgByAGEAeQAsAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAMQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAEkAdABlAG0ARgByAG8AbQBNAGkAbgBNAGEAeABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATQBpAG4AQQByAHIAYQB5ACwAIABNAGEAeABBAHIAcgBhAHkALAAgAEkAdABlAG0AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBpAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGEAeABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACwAXABuACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgAoAEkAdABlAG0AQQByAHIAYQB5ACwAIABtAGEAcwBrACwAIABcACIATgBvACAAbQBhAHQAYwBoAFwAIgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABDAHIAaQB0AGUAcgBpAGEAMQAsACAAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkALAAgAFEAdQBhAG4AdABpAHQAeQAsACAAWwBNAHUAbAB0AGkAcABsAGkAZQByAF0ALAAgAFsAQwByAGkAdABlAHIAaQBhADIAXQAsAFsAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AF0ALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAbQB1AGwAdABpAHAAbABpAGUAcgAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABNAHUAbAB0AGkAcABsAGkAZQByACkALAAxACwATQB1AGwAdABpAHAAbABpAGUAcgApACwAXABuACAAIAAgACAAcQB1AGEAbgB0AGkAdAB5ACwAIABRAHUAYQBuAHQAaQB0AHkAKgBNAHUAbAB0AGkAcABsAGkAZQByACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAxACkALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMgAsAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwByAGkAdABlAHIAaQBhADIAKQAsADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMgApACkALABcAG4AIAAgACAAIABTAFUATQBQAFIATwBEAFUAQwBUACgAYwByAGkAdABlAHIAaQBhADEAKgBjAHIAaQB0AGUAcgBpAGEAMgAqAHEAdQBhAG4AdABpAHQAeQApAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAXAB1ADAAMAAzAGMAIABTACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAXAB1ADAAMAAzAGUAIABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAE0AQQBYACgAMAAsAGwAYQBzAHQAWQBlAGEAcgAtAGYAaQByAHMAdABZAGUAYQByACsAMQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBQAGUAcgBpAG8AZABzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAIAAvACoAaABlAGwAcABlAHIAOgAgAGUAbgBkACAAZABhAHQAZQAgAGYAbwByACAAYQAgAHIAZQBwAG8AcgB0AGkAbgBnACAAcABlAHIAaQBvAGQAIABzAHQAYQByAHQAaQBuAGcAIABhAHQAIABhACAAZwBpAHYAZQBuACAAZABhAHQAZQAqAC8AXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALAAgAC8AKgBvAG4AbAB5ACAAbgBlAGUAZAAgAHQAbwAgAGwAbwBvAGsAIABiAGEAYwBrACAAMwA2ADUAIABkAGEAeQBzACgAbQBhAHgAIABvAHYAZQByAGwAYQBwACAAdwBpAG4AZABvAHcAKQAqAC8AXABuACAAIAAgACAAIAAgACAAIABBACwAUwAtADMANgA1ACwAXABuACAAIAAgACAAIAAgACAAIAB5AGEALABZAEUAQQBSACgAQQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AGIALABZAEUAQQBSACgARQApACwAIAAvACoAaQBmACAAdABoAGUAIABhAG4AYwBoAG8AcgAgAGYAbwByACAAeQBhACAAZQBuAGQAcwAgAGIAZQBmAG8AcgBlACAAUwAsAGkAdAAgAGMAYQBuAFwAdQAwADAAMgA3AHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAbgBlAHgAdAAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQBcAHUAMAAwADMAYwBTACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGIAIABzAHQAYQByAHQAcwAgAGEAZgB0AGUAcgAgAEUALABpAHQAIABjAGEAbgBcAHUAMAAwADIANwB0ACAAbwB2AGUAcgBsAGEAcAA7ACAAbQBvAHYAZQAgAHQAbwAgAHAAcgBlAHYAaQBvAHUAcwAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQBcAHUAMAAwADMAZQBFACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4ALABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQByAHMALABTAEUAUQBVAEUATgBDAEUAKABuACwAMQAsAGYAaQByAHMAdABZAGUAYQByACwAMQApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwAsAEQAQQBUAEUAKAB5AHIAcwAsAG0ALABkACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMALABNAEEAUAAoAHMAdABhAHIAdABzACwAUABlAHIAaQBvAGQARQBuAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAdABhAGcALABJAEYAKABzAHQAYQByAHQAcwA9AFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcACIAIAAoAFQAaABpAHMAIAByAGUAcABvAHIAdABpAG4AZwAgAGMAeQBjAGwAZQApAFwAIgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMAVABlAHgAdAAsAFQARQBYAFQAKABzAHQAYQByAHQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMAVABlAHgAdAAsAFQARQBYAFQAKABlAG4AZABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAbgA9ADAALABcACIAXAAiACwASABTAFQAQQBDAEsAKABzAHQAYQByAHQAcwBUAGUAeAB0ACAAXAB1ADAAMAAyADYAIABcACIAIAB0AG8AIABcACIAIABcAHUAMAAwADIANgAgAGUAbgBkAHMAVABlAHgAdAAgAFwAdQAwADAAMgA2ACAAdABhAGcAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlAFwAbgA9AEwAQQBNAEIARABBACgARgB1AG4AYwB0AGkAbwBuACwAIABUAEUAWABUAEIARQBGAE8AUgBFACgARgBPAFIATQBVAEwAQQBUAEUAWABUACgARgB1AG4AYwB0AGkAbwBuACkALAAgAFwAIgAoAFwAIgApACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZABBAHIAcgBhAHkALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQAsAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABJAEYAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAD0AXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBBAG4AeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAIAA9ACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgAMQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBBAHIAcgBhAHkAPQBQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQA9AEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQA9AFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAgACsAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQAXAB1ADAAMAAzAGUAMAAsACAAMQAsACAAMAApAFwAbgAgACAAIAAgACkAKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBDAG8AbgB2AGUAcgB0AFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAFQAbwBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlACwAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAQQByAHIAYQB5ACwAIABTAHQAYQB0AGUAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlACwAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAFwAbgA9AEwAQQBNAEIARABBACgAVABhAHIAZwBlAHQAQwBlAGwAbAAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABzAGgALAAgAFQARQBYAFQAQQBGAFQARQBSACgAQwBFAEwATAAoAFwAIgBmAGkAbABlAG4AYQBtAGUAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALAAgAFwAIgBdAFwAIgApACwAXABuACAAIAAgACAAYQBkAGQAcgAsACAAQwBFAEwATAAoAFwAIgBhAGQAZAByAGUAcwBzAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAXABuACAAIAAgACAAXAAiACMAXAB1ADAAMAAyADcAXAAiACAAXAB1ADAAMAAyADYAIABzAGgAIABcAHUAMAAwADIANgAgAFwAIgBcAHUAMAAwADIANwAhAFwAIgAgAFwAdQAwADAAMgA2ACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawBEAGkAZgBmAGUAcgBlAG4AdABTAGgAZQBlAHQAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwBcACIAIABcAHUAMAAwADIANgAgAGEAZABkAHIAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADEAXwAyAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAXABuACAAIAAgACAAQwBIAE8ATwBTAEUAQwBPAEwAUwAoAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsACAAMQAsACAAMgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADMAXwA0AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAXABuACAAIAAgACAAQwBIAE8ATwBTAEUAQwBPAEwAUwAoAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsACAAMwAsACAANAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEcAZQB0AE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACwAIABNAE0AUwAsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAXABuACAAIAAgACAAIAAgACAAIABNAEUARABJAEEATgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAE8AVQBOAEQAKABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgADAAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAE0ASQBOACgAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBBAFgAKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATQBNAFMALAAgAE0ATQBTAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBSAGUAcwB1AGwAdABzAEkAdABlAG0ARgByAG8AbQBFAHEAdQBhAHQAaQBvAG4AVABpAHQAbABlAEEAbgBkAFMAbwB1AHIAYwBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABpAHQAbABlAEMAZQBsAGwALAAgAFMAbwB1AHIAYwBlAEMAZQBsAGwALABcAG4AIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgATABFAEYAVAAoAFMAbwB1AHIAYwBlAEMAZQBsAGwALAAgAEYASQBOAEQAKABcACIALABcACIALAAgAFMAbwB1AHIAYwBlAEMAZQBsAGwAKQAgAC0AMQApACwAIABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAXAAiACwAIABcACIAXAAiACkAIABcAHUAMAAwADIANgAgAFwAIgAgAFwAIgAgAFwAdQAwADAAMgA2ACAAVABpAHQAbABlAEMAZQBsAGwAXABuACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAgACsAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQAXAB1ADAAMAAzAGUAMAAsACAAMQAsACAAMAApAFwAbgAgACAAIAAgACkAKQA7AFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEMAYQBsAGMAdQBsAGEAdABlAEgAYQByAHYAZQBzAHQASQBuAGQAZQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQwByAG8AcABUAHkAcABlACwAIABDAHIAbwBwAFQAeQBwAGUAQQByAHIAYQB5ACwAIABSAGUAcwBpAGQAdQBlAEMAcgBvAHAAUgBhAHQAaQBvAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgADEALwAoADEAKwBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAEMAcgBvAHAAVAB5AHAAZQAsACAAQwByAG8AcABUAHkAcABlAEEAcgByAGEAeQAsACAAUgBlAHMAaQBkAHUAZQBDAHIAbwBwAFIAYQB0AGkAbwBBAHIAcgBhAHkAKQApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBSAGUAcwBpAGQAdQBlAEMAcgBvAHAAUgBhAHQAaQBvAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAASABhAHIAdgBlAHMAdABJAG4AZABlAHgALABcAG4AIAAgACAAIAAoADEALQBIAGEAcgB2AGUAcwB0AEkAbgBkAGUAeAApAC8ASABhAHIAdgBlAHMAdABJAG4AZABlAHgAXABuACkAOwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBGAHIAYQBjAHQAaQBvAG4AUgBlAHMAaQBkAHUAZQBSAGUAbQBvAHYAZQBkAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABvAHQAYQBsAFIAZQBzAGkAZAB1AGUALAAgAEEAbQBvAHUAbgB0AFIAZQBtAG8AdgBlAGQALABcAG4AIAAgACAAIAAoAEEAbQBvAHUAbgB0AFIAZQBtAG8AdgBlAGQAKgAxADAAXgAzACkALwAoAFQAbwB0AGEAbABSAGUAcwBpAGQAdQBlACoAMQAwAF4AMwApAFwAbgApACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAIABkAGEAdABhACAARgBvAHIAIABTAHcAaQBuAGUAXABuAEUAeABjAGUAbAAgAG0AbwBkAHUAbABlACAAbgBhAG0AZQA6ACAAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAXABuAFYAUwBqAFwAbgBrAGcALwBoAGUAYQBkAC8AZABhAHkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAUwB3AGkAbgBlACAALQAgAFYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZABzACAAKABWAFMAagApACAALQAgADIAMAAyADAAIAB0AG8AIAAyADAAMgA0AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnAC8AaABlAGEAZAAvAGQAYQB5AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4ANgAuADEAOgAgAFMAdwBpAG4AZQAgAC0AIABJAG4AdABhAGsAZQAgAGEAbgBkACAAbQBhAG4AdQByAGUAIABjAGgAYQByAGEAYwB0AGUAcgBpAHMAdABpAGMAcwAgAGQAZQByAGkAdgBlAGQAIABmAHIAbwBtACAAUABpAGcAQgBhAGwAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAE8AbgBsAHkAIAB1AHMAZQBzACAAZABhAHQAYQAgAGYAbwByACAAMgAwADIAMAAtADIAMAAyADQALgAgAFUAcwBlACAAXAB1ADAAMAAyADcAUwBsAGEAdQBnAGgAdABlAHIAIABwAGkAZwBzAFwAdQAwADAAMgA3ACAAZABhAHQAYQAgAGYAbwByACAAXAB1ADAAMAAyADcATwB0AGgAZQByACAAagA9ADQAXAB1ADAAMAAyADcAIABjAGwAYQBzAHMALgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAYQBzAHMAXAAiACwAIABcACIAVgBTAGoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAbwBhAHIAcwBcACIALAAgADAALgA0ADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHcAcwBcACIALAAgADAALgA0ADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBpAGwAdABzAFwAIgAsACAAMAAuADUANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAHQAaABlAHIAcwBcACIALAAgADAALgAzADkAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ARgBlAGUAZABJAG4AdABhAGsAZQBcAG4ASQBqAFwAbgBrAGcALwBoAGUAYQBkAC8AZABhAHkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAEYAZQBlAGQASQBuAHQAYQBrAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFMAdwBpAG4AZQAgAC0AIABGAGUAZQBkACAAaQBuAHQAYQBrAGUAIAAtACAAaQBuAGcAZQBzAHQAZQBkACAAYQBzACAAZgBlAGQAIAAgACgASQBqACkAIAAtACAAMgAwADIAMAAgAHQAbwAgADIAMAAyADQAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBGAGUAZQBkAEkAbgB0AGEAawBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnAC8AaABlAGEAZAAvAGQAYQB5AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ARgBlAGUAZABJAG4AdABhAGsAZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADYALgAxADoAIABTAHcAaQBuAGUAIAAtACAASQBuAHQAYQBrAGUAIABhAG4AZAAgAG0AYQBuAHUAcgBlACAAYwBoAGEAcgBhAGMAdABlAHIAaQBzAHQAaQBjAHMAIABkAGUAcgBpAHYAZQBkACAAZgByAG8AbQAgAFAAaQBnAEIAYQBsAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ARgBlAGUAZABJAG4AdABhAGsAZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAATwBuAGwAeQAgAHUAcwBlAHMAIABkAGEAdABhACAAZgBvAHIAIAAyADAAMgAwAC0AMgAwADIANAAuACAAVQBzAGUAIABcAHUAMAAwADIANwBTAGwAYQB1AGcAaAB0AGUAcgAgAHAAaQBnAHMAXAB1ADAAMAAyADcAIABkAGEAdABhACAAZgBvAHIAIABcAHUAMAAwADIANwBPAHQAaABlAHIAIABqAD0ANABcAHUAMAAwADIANwAgAGMAbABhAHMAcwAuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ARgBlAGUAZABJAG4AdABhAGsAZQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAYQBzAHMAXAAiACwAIABcACIASQBqAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBCAG8AYQByAHMAXAAiACwAIAAyAC4ANgAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAbwB3AHMAXAAiACwAMgAuADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAGkAbAB0AHMAXAAiACwAIAAyAC4ANQAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AdABoAGUAcgBzAFwAIgAsACAAMQAuADcAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE4AaQB0AHIAbwBnAGUAbgBJAG4AVwBhAHMAdABlAFwAbgBOAFcAagBcAG4AawBnAC8AaABlAGEAZAAvAGQAYQB5AFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBOAGkAdAByAG8AZwBlAG4ASQBuAFcAYQBzAHQAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAUwB3AGkAbgBlACAALQAgAE4AaQB0AHIAbwBnAGUAbgAgAGkAbgAgAHcAYQBzAHQAZQAgACgATgBXAGoAKQAgAC0AIAAyADAAMgAwACAAdABvACAAMgAwADIANABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE4AaQB0AHIAbwBnAGUAbgBJAG4AVwBhAHMAdABlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnAC8AaABlAGEAZAAvAGQAYQB5AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATgBpAHQAcgBvAGcAZQBuAEkAbgBXAGEAcwB0AGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgA2AC4AMQA6ACAAUwB3AGkAbgBlACAALQAgAEkAbgB0AGEAawBlACAAYQBuAGQAIABtAGEAbgB1AHIAZQAgAGMAaABhAHIAYQBjAHQAZQByAGkAcwB0AGkAYwBzACAAZABlAHIAaQB2AGUAZAAgAGYAcgBvAG0AIABQAGkAZwBCAGEAbABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE4AaQB0AHIAbwBnAGUAbgBJAG4AVwBhAHMAdABlAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBOACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABPAG4AbAB5ACAAdQBzAGUAcwAgAGQAYQB0AGEAIABmAG8AcgAgADIAMAAyADAALQAyADAAMgA0AC4AIABVAHMAZQAgAFwAdQAwADAAMgA3AFMAbABhAHUAZwBoAHQAZQByACAAcABpAGcAcwBcAHUAMAAwADIANwAgAGQAYQB0AGEAIABmAG8AcgAgAFwAdQAwADAAMgA3AE8AdABoAGUAcgAgAGoAPQA0AFwAdQAwADAAMgA3ACAAYwBsAGEAcwBzAC4AIABBAGQAZABlAGQAIABcAHUAMAAwADIANwBOAFcAagAgAGQAYQBpAGwAeQBcAHUAMAAwADIANwAgAGMAbwBsAHUAbQBuACAAdABvACAAcAByAG8AdgBpAGQAZQAgAGQAYQBpAGwAeQAgAHYAYQBsAHUAZQAgAGYAbwByACAATwB0AGgAZQByAHMAIABjAGwAYQBzAHMALgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AEMAbABhAHMAcwAgAG4AYQBtAGUAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE4AaQB0AHIAbwBnAGUAbgBJAG4AVwBhAHMAdABlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADQALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABhAHMAcwBcACIALAAgAFwAIgBOAFcAagBcACIALAAgAFwAIgBOAFcAagAgAGQAYQBpAGwAeQBcACIALAAgAFwAIgBDAGwAYQBzAHMAIABuAGEAbQBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBCAG8AYQByAHMAXAAiACwAIAAwAC4AMAA0ADYALAAgADAALgAwADQANgAsACAAXAAiAEIAbwBhAHIAcwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHcAcwBcACIALAAwAC4AMAA0ADkALAAgADAALgAwADQAOQAsACAAXAAiAFMAbwB3AHMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAaQBsAHQAcwBcACIALAAgADAALgAwADQANgAsACAAMAAuADAANAA2ACwAIABcACIARwBpAGwAdABzAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAHQAaABlAHIAcwAgACgAawBnAC8AaABlAGEAZAAvAHkAZQBhAHIAKQBcACIALAAgADEAMQAuADQALAAgADAALgAwADMAMQAyACwAIABcACIATwB0AGgAZQByAHMAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAEYAcgBhAGMAdABpAG8AbgBOAFYAbwBsAGEAdABpAGwAaQBzAGUAZABcAG4ARgByAGEAYwBHAEEAUwBNAG0AVABcAG4AKABrAGcAIABOAEgAMwAtAE4AIAArACAATgBPAHgALQBOACkALwBrAGcATgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ARgByAGEAYwB0AGkAbwBuAE4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBTAHcAaQBuAGUAIAAtACAARgByAGEAYwB0AGkAbwBuACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAdgBvAGwAYQB0AGkAbABpAHMAZQBkACAAKABGAHIAYQBjAEcAQQBTAE0AbQBUACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBGAHIAYQBjAHQAaQBvAG4ATgBWAG8AbABhAHQAaQBsAGkAcwBlAGQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4ASAAzAC0ATgAgACsAIABOAE8AeAAtAE4AKQAvAGsAZwBOAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ARgByAGEAYwB0AGkAbwBuAE4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4ANgAuADIAOgAgAFMAdwBpAG4AZQAgAC0AIABGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdgBvAGwAYQB0AGkAbABpAHMAZQBkACAAYgB5ACAATQBNAFMAIAAoACgAawBnACAATgBIADMALQBOACAAKwAgAE4ATwB4AC0ATgApAC8AawBnAE4AKQAgACgARgByAGEAYwBHAEEAUwBNAG0AVAApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ARgByAGEAYwB0AGkAbwBuAE4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBOACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABcAHUAMAAwADIANwBOAEkAUgAgAHIAZQBmAGUAcgBlAG4AYwBlACAAYwBvAGwAdQBtAG4AIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBGAHIAYQBjAHQAaQBvAG4ATgBWAG8AbABhAHQAaQBsAGkAcwBlAGQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANwAsACAAMwAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBNAFMAbQBcACIALAAgAFwAIgBGAHIAYQBjAEcAQQBTAE0AbQBUAFwAIgAsACAAXAAiAE4ASQBSACAAcgBlAGYAZQByAGUAbgBjAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AdQB0AGQAbwBvAHIAIAAoAEQAcgB5ACAAbABvAHQAKQBcACIALAAgADAALgAzACwAIABcACIARAByAHkAbABvAHQAIAAoAGYAZQBlAGQAIABwAGEAZAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGUAZQBwACAAbABpAHQAdABlAHIAXAAiACwAIAAwAC4AMQAyADUALAAgAFwAIgBEAGUAZQBwACAAbABpAHQAdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABvAGMAawBwAGkAbABlACAAKABTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlACkAXAAiACwAIAAwAC4AMgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAZgBmAGwAdQBlAG4AdAAgAHAAbwBuAGQAIAAoAFUAbgBjAG8AdgBlAHIAZQBkACAAYQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgApAFwAIgAsACAAMAAuADUANQAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAZABpAGcAZQBzAHQAZQByACAALwAgAEMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBcACIALAAgADAALAAgAFwAIgBEAGkAZwBlAHMAdABlAHIAIAAvACAAYwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAHMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAaABvAHIAdAAgAEgAUgBUACAAdABhAG4AawAgAHMAdABvAHIAYQBnAGUAIABcAHUAMAAwADMAYwAgADEAIABtAG8AbgB0AGgAIAAoAHAAaQB0ACAAcwB0AG8AcgBhAGcAZQApAFwAIgAsACAAMAAuADIANQAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXABuAEYAcgBhAGMARwBBAFMATQBtAFQAXABuAGsAZwBOADIATwAgAC0AIABOACAALwAgAGsAZwBOAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAUwB3AGkAbgBlACAALQAgAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABFAEYAcwAgAGIAeQAgAE0ATQBTACAAKABFAEYAbQBUACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwBOADIATwAgAC0AIABOACAALwAgAGsAZwBOAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgA2AC4AMwA6ACAAUwB3AGkAbgBlACAALQAgAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABFAEYAcwAgAGIAeQAgAE0ATQBTACAAKABrAGcATgAyAE8ALQBOAC8AawBnAE4AKQAgACgARQBGAG0AVAApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE4ASQBSACAAcgBlAGYAZQByAGUAbgBjAGUAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADcALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0ATQBTAG0AXAAiACwAIABcACIARQBGAG0AVABcACIALAAgAFwAIgBOAEkAUgAgAHIAZQBmAGUAcgBlAG4AYwBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAHUAdABkAG8AbwByACAAKABEAHIAeQAgAGwAbwB0ACkAXAAiACwAIAAwAC4AMAAyACwAIABcACIARAByAHkAbABvAHQAIAAoAGYAZQBlAGQAIABwAGEAZAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGUAZQBwACAAbABpAHQAdABlAHIAXAAiACwAIAAwAC4AMAAxACwAIABcACIARABlAGUAcAAgAGwAaQB0AHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAbwBjAGsAcABpAGwAZQAgACgAUwBvAGwAaQBkACAAcwB0AG8AcgBhAGcAZQApAFwAIgAsACAAMAAuADAAMAA1ACwAIABcACIAUwBvAGwAaQBkACAAcwB0AG8AcgBhAGcAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBmAGYAbAB1AGUAbgB0ACAAcABvAG4AZAAgACgAVQBuAGMAbwB2AGUAcgBlAGQAIABhAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuACkAXAAiACwAIAAwACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABkAGkAZwBlAHMAdABvAHIAIAAvACAAQwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAFwAIgAsACAAMAAsACAAXAAiAEQAaQBnAGUAcwB0AGUAcgAgAC8AIABjAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AcwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBoAG8AcgB0ACAASABSAFQAIAB0AGEAbgBrACAAcwB0AG8AcgBhAGcAZQAgAFwAdQAwADAAMwBjACAAMQAgAG0AbwBuAHQAaAAgACgAcABpAHQAIABzAHQAbwByAGEAZwBlACkAXAAiACwAIAAwAC4AMAAwADIALAAgAFwAIgBQAGkAdAAgAHMAdABvAHIAYQBnAGUAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAFwAbgBCADAAXABuAG0AMwAgAEMASAA0AC8AawBnACAAVgBTAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuAHMAIABwAG8AdABlAG4AdABpAGEAbAAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAIABwAGUAcgAgAGsAaQBsAG8AZwByAGEAbQAgAG8AZgAgAHYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZABzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEIAMABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAbQAzACAAQwBIADQAIAAvACAAawBnACAAVgBTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIASQBQAEMAQwAgACgAMgAwADEAOQApACwAIABDAGgAYQBwAHQAZQByACAAMQAwACAAWwA0AF0AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMQA5ACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATQBNAFMAXwBNAEMARgBzAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADYALgA0ADoAIABTAHcAaQBuAGUAIAAtACAATQBDAEYAcwAgACgATQBDAEYAaQBtACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE0ATQBTAF8ATQBDAEYAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQAgAGEAbgBkACAAbQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAcwB5AHMAdABlAG0ALgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE0ATQBTAF8ATQBDAEYAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATQBNAFMAXwBNAEMARgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4ANgAuADQAOgAgAFMAdwBpAG4AZQAgAC0AIABNAEMARgBzACAAKABNAEMARgBpAG0AKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE0ATQBTAF8ATQBDAEYAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQQBkAGQAZQBkACAAYwBvAGwAdQBtAG4AcwAgAGYAbwByACAAQQBDAFQALAAgAHMAcABsAGkAdAAgAFEATABEACAAYQBuAGQAIABOAFQALgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAGMAbwBsAHUAbQBuACAAdwBpAHQAaAAgAE0ATQBTACAAbgBhAG0AZQBzACAAdABoAGEAdAAgAG0AYQB0AGMAaAAgAE4ASQBSACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATQBNAFMAXwBNAEMARgBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADEAMAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBNAFMAXAAiACwAIABcACIATgBTAFcAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAUQBMAEQAXAAiACwAIABcACIATgBUAFwAIgAsACAAXAAiAFMAQQBcACIALAAgAFwAIgBUAEEAUwBcACIALAAgAFwAIgBWAEkAQwBcACIALAAgAFwAIgBXAEEAXAAiACwAIABcACIATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAHUAdABkAG8AbwByACAAKABEAHIAeQAgAGwAbwB0ACkAXAAiACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIAAwAC4AMAAzACwAIAAwAC4AMAAzACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIABcACIARAByAHkAbABvAHQAIAAoAGYAZQBlAGQAIABwAGEAZAApAFwAIgA7ACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgADAALgAwADQALAAgADAALgAwADQALAAgADAALgAwADQALAAgADAALgAwADQALAAgADAALgAwADQALAAgADAALgAwADQALAAgADAALgAwADQALAAgADAALgAwADQALAAgAFwAIgBEAGUAZQBwACAAbABpAHQAdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABvAGMAawBwAGkAbABlACAAKABTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlACkAXAAiACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIABcACIAUwBvAGwAaQBkACAAcwB0AG8AcgBhAGcAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBmAGYAbAB1AGUAbgB0ACAAcABvAG4AZAAgACgAVQBuAGMAbwB2AGUAcgBlAGQAIABhAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuACkAXAAiACwAIAAwAC4ANwA1ACwAIAAwAC4ANwA1ACwAIAAwAC4ANwA4ACwAIAAwAC4ANwA4ACwAIAAwAC4ANwA1ACwAIAAwAC4ANwAwACwAIAAwAC4ANwA0ACwAIAAwAC4ANwA2ACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABkAGkAZwBlAHMAdABlAHIAIAAvACAAQwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAFwAIgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMQAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMQAsACAAMAAuADEALAAgADAALgAxACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgA7ACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAaABvAHIAdAAgAEgAUgBUACAAdABhAG4AawAgAHMAdABvAHIAYQBnAGUAIABcAHUAMAAwADMAYwAgADEAIABtAG8AbgB0AGgAIAAoAHAAaQB0ACAAcwB0AG8AcgBhAGcAZQApAFwAIgAsACAAMAAuADAAMwAsACAAMAAuADAAMwAsACAAMAAuADAAMwAsACAAMAAuADAAMwAsACAAMAAuADAAMwAsACAAMAAuADAAMwAsACAAMAAuADAAMwAsACAAMAAuADAAMwAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQBcACIAOwAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGkAcgBlAGMAdAAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgAgAHQAbwAgAHMAbwBpAGwAXAAiACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAEEAdgBlAHIAYQBnAGUATABpAHYAZQB3AGUAaQBnAGgAdABcAG4AVwBjAG8AXABuAGsAZwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8AQQB2AGUAcgBhAGcAZQBMAGkAdgBlAHcAZQBpAGcAaAB0AF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBTAHcAaQBuAGUAIAAtACAAQQB2AGUAcgBhAGcAZQAgAGwAaQB2AGUAdwBlAGkAZwBoAHQAIAAoAGkAbgB2AGUAbgB0AG8AcgB5ACAAZABlAGYAYQB1AGwAdABzACkAIAAoAGsAZwApACAAKABXAGMAbwApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8AQQB2AGUAcgBhAGcAZQBMAGkAdgBlAHcAZQBpAGcAaAB0AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8AQQB2AGUAcgBhAGcAZQBMAGkAdgBlAHcAZQBpAGcAaAB0AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4ANgAuADUAOgAgAFMAdwBpAG4AZQAgAC0AIABBAHYAZQByAGEAZwBlACAAbABpAHYAZQB3AGUAaQBnAGgAdAAgACgAaQBuAHYAZQBuAHQAbwByAHkAIABkAGUAZgBhAHUAbAB0AHMAKQAgACgAawBnACkAIAAoAFcAYwBvACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBBAHYAZQByAGEAZwBlAEwAaQB2AGUAdwBlAGkAZwBoAHQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIALgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAEEAdgBlAHIAYQBnAGUATABpAHYAZQB3AGUAaQBnAGgAdABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGkAdgBlAHMAdABvAGMAawAgAFQAeQBwAGUAIABqAFwAIgAsACAAXAAiAEEAdgBlAHIAYQBnAGUAIABMAGkAdgBlAHcAZQBpAGcAaAB0ACAAKABrAGcAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHcAcwBcACIALAAgADEAOAA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAbwBhAHIAcwBcACIALAAgADIAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAaQBsAHQAcwBcACIALAAgADEAMgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAbABhAHUAZwBoAHQAZQByACAAcABpAGcAcwBcACIALAAgADMAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAGwAYQB1AGcAaAB0AGUAcgAgAHAAaQBnAHMAIABhAHQAIAB0AHUAcgBuAG8AZgBmAFwAIgAsACAAOQA3AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AcwBcAG4ANAAuADUAIABTAHcAaQBuAGUAIABGAGkAZwB1AHIAZQAgADQALgA4AFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFMAdwBpAG4AZQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQBzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8AUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADUAIABTAHcAaQBuAGUAIABGAGkAZwB1AHIAZQAgADQALgA4AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8AUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8AUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG4AdgBlAG4AdABpAG8AbgBhAGwAIABoAG8AdQBzAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGUAZQBwACAAbABpAHQAdABlAHIAIABoAG8AdQBzAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAHUAdABkAG8AbwByAC8AZgByAGUAZQAgAHIAYQBuAGcAZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAHIAeQBsAG8AdABNAE0AUwBcAG4ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXABuAGYAcgBhAGMAdABpAG8AbgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAHIAeQBsAG8AdABNAE0AUwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAbABvAHMAdAAgAHQAaAByAG8AdQBnAGgAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmACAAZgBvAHIAIABkAHIAeQBsAG8AdAAgAE0ATQBTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAHIAeQBsAG8AdABNAE0AUwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBGAHIAYQBjAEwARQBBAEMASABfAEQAcgB5AGwAbwB0AE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAHIAeQBsAG8AdABNAE0AUwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4ANQAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAHIAeQBsAG8AdABNAE0AUwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFADoAIABUAGUAeAB0ACAAcgBlAGYAZQByAHMAIAB0AG8AIABcAHUAMAAwADIANwBzAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAdQAwADAAMgA3ACAATQBNAFMALAAgAGIAdQB0ACAAZQBxAHUAYQB0AGkAbwBuACAAcgBlAGYAZQByAHMAIAB0AG8AIABcAHUAMAAwADIANwBkAHIAeQBsAG8AdABcAHUAMAAwADIANwAgAE0ATQBTAC4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBGAHIAYQBjAEwARQBBAEMASABfAEQAcgB5AGwAbwB0AE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMAAyACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATQBlAGcAYQBqAG8AdQBsAGUAcwBQAGUAcgBLAGkAbABvAGcAcgBhAG0ATQBlAHQAaABhAG4AZQBcAG4ARgBcAG4ATQBKAC8AawBnACAAQwBIADQAXABuAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBNAGUAZwBhAGoAbwB1AGwAZQBzAFAAZQByAEsAaQBsAG8AZwByAGEAbQBNAGUAdABoAGEAbgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGUAZwBhAGoAbwB1AGwAZQBzACAAcABlAHIAIABrAGkAbABvAGcAcgBhAG0AIABvAGYAIABtAGUAdABoAGEAbgBlAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATQBlAGcAYQBqAG8AdQBsAGUAcwBQAGUAcgBLAGkAbABvAGcAcgBhAG0ATQBlAHQAaABhAG4AZQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE0AZQBnAGEAagBvAHUAbABlAHMAUABlAHIASwBpAGwAbwBnAHIAYQBtAE0AZQB0AGgAYQBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAEoAIAAvACAAawBnACAAQwBIADQAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBNAGUAZwBhAGoAbwB1AGwAZQBzAFAAZQByAEsAaQBsAG8AZwByAGEAbQBNAGUAdABoAGEAbgBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADMALgA1AC4AMgAuADMAIABDAE8ATgBTAFQAQQBOAFQAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBNAGUAZwBhAGoAbwB1AGwAZQBzAFAAZQByAEsAaQBsAG8AZwByAGEAbQBNAGUAdABoAGEAbgBlAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATQBlAGcAYQBqAG8AdQBsAGUAcwBQAGUAcgBLAGkAbABvAGcAcgBhAG0ATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgANQA1AC4AMgAyACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAFMAdwBpAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAzAC4ANQA6ACAARQBuAHQAZQByAGkAYwAgAE0AZQB0AGgAYQBuAGUAIAAtACAAUwB3AGkAbgBlAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAzAC4ANQAuADEALgAxACAATQBlAHQAaABvAGQAIAAxACAALQAgAEUAbgB0AGUAcgBpAGMAIABTAHcAaQBuAGUAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwAzAF8ANQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAFwAbgBUAG8AdABhAGwAIABhAG4AbgB1AGEAbAAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgByAG8AbQAgAGUAbgB0AGUAcgBpAGMAIABmAGUAcgBtAGUAbgB0AGEAdABpAG8AbgAgAGkAbgAgAHMAdwBpAG4AZQBcAG4ARQBfAGUAbgB0AGUAcgBpAGMAXABuAHQAIABDAEgANABcAG4ARQBfAHsAZQBuAHQAZQByAGkAYwB9AD0AXABcAHMAdQBtAF8AewBqAH0AKABOAF8AagBcAFwAdABpAG0AZQBzACAATQBfAGoAXABcAHQAaQBtAGUAcwAgAEQAXwBqACkAXABcAHQAaQBtAGUAcwAgADEAMABeAHsALQAzAH0AXABuAE4AXwBqACAAPQAgAG4AdQBtAGIAZQByAHMAIABvAGYAIABzAHcAaQBuAGUAIABvAGYAIABlAGEAYwBoACAAYwBsAGEAcwBzACAAKABoAGUAYQBkACkAXABuAE0AXwBqACAAPQAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAKABrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQApAFwAbgBEAF8AagAgAD0AIAB0AGgAZQAgAGEAdgBlAHIAYQBnAGUAIABuAHUAbQBiAGUAcgAgAG8AZgAgAGQAYQB5AHMAIABvAG4AIABmAGEAcgBtACAAZgBvAHIAIABlAGEAYwBoACAAcwB3AGkAbgBlACAAYwBsAGEAcwBzACAAKABkAGEAeQBzACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADUAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABOAF8AagAsACAATQBfAGoALAAgAEQAXwBqACwAXABuACAAIAAgACAAKABOAF8AagAgACoAIABNAF8AagAgACoAIABEAF8AagApACAAKgAgADEAMAAgAF4AIAAtADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8ANQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAG8AdABhAGwAIABhAG4AbgB1AGEAbAAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgByAG8AbQAgAGUAbgB0AGUAcgBpAGMAIABmAGUAcgBtAGUAbgB0AGEAdABpAG8AbgAgAGkAbgAgAHMAdwBpAG4AZQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADUAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAGUAbgB0AGUAcgBpAGMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwA1AF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBIADQAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwA1AF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADUALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAxACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwA1AF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwA1AF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AewBlAG4AdABlAHIAaQBjAH0APQBcAFwAcwB1AG0AXABcAG4AbwBsAGkAbQBpAHQAcwBfAGoAKABOAF8AagBcAFwAdABpAG0AZQBzACAATQBfAGoAXABcAHQAaQBtAGUAcwAgAEQAXwBqACkAXABcAHQAaQBtAGUAcwAgADEAMABeAHsALQAzAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwA1AF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBfAGoAXAAiACwAIABcACIAbgB1AG0AYgBlAHIAcwAgAG8AZgAgAHMAdwBpAG4AZQAgAG8AZgAgAGUAYQBjAGgAIABjAGwAYQBzAHMAXAAiACwAIABcACIAaABlAGEAZABcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AXwBqAFwAIgAsACAAXAAiAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuAFwAIgAsACAAXAAiAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAAMwAuADUALgAxAC4AMQAsACAAKAAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAXwBqAFwAIgAsACAAXAAiAHQAaABlACAAYQB2AGUAcgBhAGcAZQAgAG4AdQBtAGIAZQByACAAbwBmACAAZABhAHkAcwAgAG8AbgAgAGYAYQByAG0AIABmAG8AcgAgAGUAYQBjAGgAIABzAHcAaQBuAGUAIABjAGwAYQBzAHMAXAAiACwAIABcACIAZABhAHkAcwBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMwBfADUAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBcAG4AVABvAHQAYQBsACAAZABhAGkAbAB5ACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAG8AZgAgAGUAbgB0AGUAcgBpAGMAIABtAGUAdABoAGEAbgBlACAAbwBmACAAcwB3AGkAbgBlAFwAbgBNAF8AagBcAG4AawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXABuAE0AXwBqAD0AXABcAGYAcgBhAGMAewBJAF8AagBcAFwAdABpAG0AZQBzACAAMQA4AC4ANgBcAFwAdABpAG0AZQBzACAAMAAuADAAMAA3AH0AewBGAH0AXABuAEkAXwBqACAAPQAgAGQAYQBpAGwAeQAgAGYAZQBlAGQAIABpAG4AZwBlAHMAdABlAGQAIABiAHkAIABlAGEAYwBoACAAcwB3AGkAbgBlACAAYwBsAGEAcwBzACAAKABrAGcALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ARgAgAD0AIABtAGUAZwBhAGoAbwB1AGwAZQBzACAAcABlAHIAIABrAGkAbABvAGcAcgBhAG0AIABvAGYAIABtAGUAdABoAGEAbgBlACAAKABNAEoALwBrAGcAIABDAEgANAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADMAXwA1AF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAASQBfAGoALAAgAEYALABcAG4AIAAgACAAIAAoAEkAXwBqACAAKgAgADEAOAAuADYAIAAqACAAMAAuADAAMAA3ACkAIAAvACAARgBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwA1AF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAbwB0AGEAbAAgAGQAYQBpAGwAeQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABvAGYAIABlAG4AdABlAHIAaQBjACAAbQBlAHQAaABhAG4AZQAgAG8AZgAgAHMAdwBpAG4AZQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADUAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBfAGoAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwA1AF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADUAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4ANQAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADIAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADUAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADUAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AXwBqAD0AXABcAGYAcgBhAGMAewBJAF8AagBcAFwAdABpAG0AZQBzACAAMQA4AC4ANgBcAFwAdABpAG0AZQBzACAAMAAuADAAMAA3AH0AewBGAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwA1AF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBfAGoAXAAiACwAIABcACIAZABhAGkAbAB5ACAAZgBlAGUAZAAgAGkAbgBnAGUAcwB0AGUAZAAgAGIAeQAgAGUAYQBjAGgAIABzAHcAaQBuAGUAIABjAGwAYQBzAHMAXAAiACwAIABcACIAawBnAC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAMQA4AC4ANgBcACIALAAgAFwAIgBnAHIAbwBzAHMAIABlAG4AZQByAGcAeQAgACgARwBFACkAIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAZgBlAGUAZABcACIALAAgAFwAIgBNAEoAIABHAEUALwBrAGcAIABmAGUAZQBkAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAMAAuADAAMAA3AFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAEcARQAgAGkAbgB0AGEAawBlACAAYwBvAG4AdgBlAHIAdABlAGQAIAB0AG8AIABtAGUAdABoAGEAbgBlACAAYgB5ACAAcwB3AGkAbgBlAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAXAAiACwAIABcACIAbQBlAGcAYQBqAG8AdQBsAGUAcwAgAHAAZQByACAAawBpAGwAbwBnAHIAYQBtACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIALAAgAFwAIgBNAEoALwBrAGcAIABDAEgANABcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ANAAuADUAOgAgAFMAdwBpAG4AZQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ANAAuADUALgAxAC4AMQAgAE0AZQB0AGgAbwBkACAAMQAgABQgIABNAGEAbgB1AHIAZQAgAE0AZQB0AGgAYQBuAGUAIABTAHcAaQBuAGUAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAXABuAFQAbwB0AGEAbAAgAGEAbgBuAHUAYQBsACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdABcAG4ARQBDAEgANABcAG4AdAAgAEMASAA0AFwAbgB7AEUAfQBfAHsAQwBIADQAfQA9AFwAXABzAHUAbQBfAHsAagB9ACgARABfAHsAagB9AFwAXAB0AGkAbQBlAHMAIABNAF8AewBtAGoAfQBcAFwAdABpAG0AZQBzACAATgBfAHsAagB9ACkAXABcAHQAaQBtAGUAcwAxADAAXgB7AC0AMwB9AFwAbgBEAGoAIAA9ACAAbABlAG4AZwB0AGgAIABvAGYAIABzAHQAYQB5ACAAbwBmACAAZQBhAGMAaAAgAGMAbABhAHMAcwAgAG8AZgAgAHMAdwBpAG4AZQAgADoAIABkAGEAeQBzAFwAbgBNAG0AagAgAD0AIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIABtAGEAbgB1AHIAZQAgAGkAbgAgAGUAYQBjAGgAIABzAHcAaQBuAGUAIABjAGwAYQBzAHMAIAA6ACAAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXABuAE4AagAgAD0AIABuAHUAbQBiAGUAcgBzACAAbwBmACAAcwB3AGkAbgBlACAAaQBuACAAZQBhAGMAaAAgAGMAbABhAHMAcwAgADoAIABoAGUAYQBkAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABEAGoALAAgAE0AbQBqACwAIABOAGoALABcAG4AIAAgACAAIABEAGoAIAAqACAATQBtAGoAIAAqACAATgBqACAAKgAgADEAMAAgAF4AIAAtADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAbwB0AGEAbAAgAGEAbgBuAHUAYQBsACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEMASAA0AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBIADQAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4ANQAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADEAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB7AEUAfQBfAHsAQwBIADQAfQA9AFwAXABzAHUAbQBfAHsAagB9ACgARABfAHsAagB9AFwAXAB0AGkAbQBlAHMAIABNAF8AewBtAGoAfQBcAFwAdABpAG0AZQBzACAATgBfAHsAagB9ACkAXABcAHQAaQBtAGUAcwAxADAAXgB7AC0AMwB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABqAFwAIgAsAFwAIgBsAGUAbgBnAHQAaAAgAG8AZgAgAHMAdABhAHkAIABvAGYAIABlAGEAYwBoACAAYwBsAGEAcwBzACAAbwBmACAAcwB3AGkAbgBlAFwAIgAsACAAXAAiAGQAYQB5AHMAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAG0AagBcACIALABcACIAbQBlAHQAaABhAG4AZQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAHIAbwBtACAAbQBhAG4AdQByAGUAIABpAG4AIABlAGEAYwBoACAAcwB3AGkAbgBlACAAYwBsAGEAcwBzAFwAIgAsACAAXAAiAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAANAAuADUALgAxAC4AMQAgACgAMgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAGoAXAAiACwAXAAiAG4AdQBtAGIAZQByAHMAIABvAGYAIABzAHcAaQBuAGUAIABpAG4AIABlAGEAYwBoACAAYwBsAGEAcwBzAFwAIgAsACAAXAAiAGgAZQBhAGQAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADIAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUABlAHIAQwBsAGEAcwBzAFwAbgBNAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIAB0AGgAZQAgAG0AYQBuAHUAcgBlACAAbwBmACAAZQBhAGMAaAAgAGMAbABhAHMAcwAgAG8AZgAgAHMAdwBpAG4AZQBcAG4ATQBtAGoAXABuAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5AFwAbgBNAF8AewBtAGoAfQA9AFwAXABzAHUAbQBfAHsAbQB9AFwAXABzAHUAbQBfAHsAVAB9AE0AXwB7AGoAbQBUAH0AXABuAE0AagBtAFQAIAA9ACAAbQBlAHQAaABhAG4AZQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAHIAbwBtACAAbQBhAG4AdQByAGUAIABwAGUAcgAgAGMAbABhAHMAcwAsACAATQBNAFMALAAgAGEAbgBkACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAA6ACAAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMgBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAGUAcgBDAGwAYQBzAHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBqAG0AVAAsAFwAbgAgACAAIAAgAFMAVQBNACgATQBqAG0AVAApAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMgBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAGUAcgBDAGwAYQBzAHMAVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBqAG0AVAAxACwAIABNAGoAbQBUADIALABcAG4AIAAgACAAIAAgAFMAVQBNACgATQBqAG0AVAAxACwAIABNAGoAbQBUADIAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADIAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUABlAHIAQwBsAGEAcwBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIAB0AGgAZQAgAG0AYQBuAHUAcgBlACAAbwBmACAAZQBhAGMAaAAgAGMAbABhAHMAcwAgAG8AZgAgAHMAdwBpAG4AZQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMgBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAGUAcgBDAGwAYQBzAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AbQBqAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAyAF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAZQByAEMAbABhAHMAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAyAF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAZQByAEMAbABhAHMAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4ANQAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADIAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMgBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAGUAcgBDAGwAYQBzAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADIAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUABlAHIAQwBsAGEAcwBzAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBfAHsAbQBqAH0APQBcAFwAcwB1AG0AXwB7AG0AfQBcAFwAcwB1AG0AXwB7AFQAfQBNAF8AewBqAG0AVAB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAyAF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAZQByAEMAbABhAHMAcwBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGoAbQBUAFwAIgAsAFwAIgBtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIABtAGEAbgB1AHIAZQAgAHAAZQByACAAYwBsAGEAcwBzACwAIABNAE0AUwAsACAAYQBuAGQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQBcACIALAAgAFwAIgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADQALgA1AC4AMQAuADEAIAAoADMAKQAgAGEAbgBkACAAKAA2ACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAyAF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAZQByAEMAbABhAHMAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFADoAIABTAHAAbABpAHQAIAB2AGEAcgBpAGEAYgBsAGUAIABNAGoAbQAgAGkAbgB0AG8AIABNAGoAbQBUADEAIABhAG4AZAAgAE0AagBtAFQAMgAgAGYAbwByACAAcwB0AGEAZwBlACAAMQAgAGEAbgBkACAAMgAgAE0ATQBTAC4AXAAiACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAzAF8AUwB0AGEAZwBlADEATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFwAbgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAbwBmACAAbQBlAHQAaABhAG4AZQAgAGkAbgAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMQAgAE0ATQBTAFwAbgBNAGkAagBtAFQAMQBcAG4AawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXABuAE0AXwB7AGkAagBtACwAVAA9ADEAfQA9AFYAUwBfAHsAagB9AFwAXAB0AGkAbQBlAHMAIABGAFYAUwBfAHsAagBtACwAVAA9ADEAfQBcAFwAdABpAG0AZQBzACAATQBDAEYAXwB7AGkAbQB9AFwAXAB0AGkAbQBlAHMAIABCAE8AXABcAHQAaQBtAGUAcwAgAFwAXAByAGgAbwBcAG4AVgBTAGoAIAA9ACAAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIABzAHcAaQBuAGUAIABpAG4AIABlAGEAYwBoACAAYwBsAGEAcwBzACAAOgAgAGsAZwAvAGgAZQBhAGQALwBkAGEAeQBcAG4ARgBWAFMAagBtAFQAMQAgAD0AIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIAB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgAGkAbgAgAGUAYQBjAGgAIABwAHIAaQBtAGEAcgB5ACAAcwB5AHMAdABlAG0AIAA6ACAAZgByAGEAYwB0AGkAbwBuAFwAbgBNAEMARgBpAG0AIAA9ACAAbQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdABlAG0AcABlAHIAYQB0AGUAIAB6AG8AbgBlACAAYQBuAGQAIABzAHkAcwB0AGUAbQAgADoAIABmAHIAYQBjAHQAaQBvAG4AXABuAEIATwAgAD0AIABlAG0AaQBzAHMAaQBvAG4AcwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAOgAgAG0AMwAgAEMASAA0AC8AawBnACAAVgBTAFwAbgByAGgAbwAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgADoAIABrAGcALwBtADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABWAFMAagAsACAARgBWAFMAagBtAFQAMQAsACAATQBDAEYAaQBtACwAIABCAE8ALAAgAHIAaABvACwAXABuACAAIAAgACAAVgBTAGoAIAAqACAARgBWAFMAagBtAFQAMQAgACoAIABNAEMARgBpAG0AIAAqACAAQgBPACAAKgAgAHIAaABvAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAUAByAG8AZAB1AGMAdABpAG8AbgAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAIABpAG4AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADEAIABNAE0AUwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBpAGoAbQBUADEAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADMAXwBTAHQAYQBnAGUAMQBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4ANQAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADMAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AXwB7AGkAagBtACwAVAA9ADEAfQA9AFYAUwBfAHsAagB9AFwAXAB0AGkAbQBlAHMAIABGAFYAUwBfAHsAagBtACwAVAA9ADEAfQBcAFwAdABpAG0AZQBzACAATQBDAEYAXwB7AGkAbQB9AFwAXAB0AGkAbQBlAHMAIABCAE8AXABcAHQAaQBtAGUAcwAgAFwAXAByAGgAbwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAFMAagBcACIALABcACIAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIABzAHcAaQBuAGUAIABpAG4AIABlAGEAYwBoACAAYwBsAGEAcwBzAFwAIgAsACAAXAAiAGsAZwAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAVgBTAGoAbQBUADEAXAAiACwAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAHYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZABzACAAaQBuACAAZQBhAGMAaAAgAHAAcgBpAG0AYQByAHkAIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAA0AC4ANQAuADEALgAxACAAKAA0ACkAKAA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQwBGAGkAbQBcACIALABcACIAbQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAdABlAG0AcABlAHIAYQB0AGUAIAB6AG8AbgBlACAAYQBuAGQAIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBCAE8AXAAiACwAXAAiAGUAbQBpAHMAcwBpAG8AbgBzACAAcABvAHQAZQBuAHQAaQBhAGwAXAAiACwAIABcACIAbQAzACAAQwBIADQALwBrAGcAIABWAFMAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgByAGgAbwBcACIALABcACIAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAXAAiACwAIABcACIAawBnAC8AbQAzAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA0AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBQAHIAaQBtAGEAcgB5AFMAeQBzAHQAZQBtAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIAB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgAGkAbgAgAGUAYQBjAGgAIABwAHIAaQBtAGEAcgB5ACAAcwB5AHMAdABlAG0AIABvAHQAaABlAHIAIAB0AGgAYQBuACAAcwBvAGwAaQBkACAAcwB0AG8AcgBhAGcAZQBcAG4ARgBWAFMAagBtAFQAMQBcAG4AZgByAGEAYwB0AGkAbwBuAFwAbgBGAFYAUwBfAHsAagBtACwAVAA9ADEAfQA9AE0ATQBTAF8AewBqAG0ALABUAD0AMQB9AFwAXAB0AGkAbQBlAHMAKAAxAC0AUwBTAF8AewBtAH0AKQBcAG4ATQBNAFMAagBtAFQAMQAgAD0AIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABtAGEAbgB1AHIAZQAgAHQAbwAgAGUAYQBjAGgAIABwAHIAaQBtAGEAcgB5ACAATQBNAFMAIABmAG8AcgAgAGUAYQBjAGgAIABjAGwAYQBzAHMAIABwAHIAaQBvAHIAIAB0AG8AIABzAG8AbABpAGQAIABzAGUAcABhAHIAYQB0AGkAbwBuACAAOgAgAGYAcgBhAGMAdABpAG8AbgBcAG4AUwBTAG0AIAA9ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkAHMAIABzAGUAcABhAHIAYQB0AGUAZAAgAHQAbwAgAHMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAIABmAG8AcgAgAGUAYQBjAGgAIABNAE0AUwAgADoAIABmAHIAYQBjAHQAaQBvAG4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANABfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAUAByAGkAbQBhAHIAeQBTAHkAcwB0AGUAbQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAE0AUwBqAG0AVAAxACwAIABTAFMAbQAsAFwAbgAgACAAIAAgAE0ATQBTAGoAbQBUADEAIAAqACAAKAAxACAALQAgAFMAUwBtACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA0AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBQAHIAaQBtAGEAcgB5AFMAeQBzAHQAZQBtAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIAB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgAGkAbgAgAGUAYQBjAGgAIABwAHIAaQBtAGEAcgB5ACAAcwB5AHMAdABlAG0AIABvAHQAaABlAHIAIAB0AGgAYQBuACAAcwBvAGwAaQBkACAAcwB0AG8AcgBhAGcAZQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANABfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAUAByAGkAbQBhAHIAeQBTAHkAcwB0AGUAbQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBWAFMAagBtAFQAMQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANABfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAUAByAGkAbQBhAHIAeQBTAHkAcwB0AGUAbQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANABfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAUAByAGkAbQBhAHIAeQBTAHkAcwB0AGUAbQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4ANQAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADQAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANABfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAUAByAGkAbQBhAHIAeQBTAHkAcwB0AGUAbQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANABfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAUAByAGkAbQBhAHIAeQBTAHkAcwB0AGUAbQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAVgBTAF8AewBqAG0ALABUAD0AMQB9AD0ATQBNAFMAXwB7AGoAbQAsAFQAPQAxAH0AXABcAHQAaQBtAGUAcwAoADEALQBTAFMAXwB7AG0AfQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA0AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBQAHIAaQBtAGEAcgB5AFMAeQBzAHQAZQBtAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0ATQBTAGoAbQBUADEAXAAiACwAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG0AYQBuAHUAcgBlACAAdABvACAAZQBhAGMAaAAgAHAAcgBpAG0AYQByAHkAIABNAE0AUwAgAGYAbwByACAAZQBhAGMAaAAgAGMAbABhAHMAcwAgAHAAcgBpAG8AcgAgAHQAbwAgAHMAbwBsAGkAZAAgAHMAZQBwAGEAcgBhAHQAaQBvAG4AXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBTAG0AXAAiACwAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAHYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZABzACAAcwBlAHAAYQByAGEAdABlAGQAIAB0AG8AIABzAG8AbABpAGQAIABzAHQAbwByAGEAZwBlACAAZgBvAHIAIABlAGEAYwBoACAATQBNAFMAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADQAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFAAcgBpAG0AYQByAHkAUwB5AHMAdABlAG0AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA1AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkAHMAIABpAG4AIABzAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAbgBGAFYAUwBqAG0ANABUADEAXABuAGYAcgBhAGMAdABpAG8AbgBcAG4ARgBWAFMAXwB7AGoALABtAD0ANAAsAFQAPQAxAH0APQBNAE0AUwBfAHsAagAsAG0APQA0ACwAVAA9ADEAfQArACgATQBNAFMAXwB7AGoALABtAD0AMQAsADcALAA5ACwAVAA9ADEAfQBcAFwAdABpAG0AZQBzACAAUwBTAF8AewBtAH0AKQBcAG4ATQBNAFMAagBtADQAVAAxACAAPQAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG0AYQBuAHUAcgBlACAAaQBuACAAcwBvAGwAaQBkACAAcwB0AG8AcgBhAGcAZQAgAHAAcgBpAG0AYQByAHkAIABzAHkAcwB0AGUAbQAgADoAIABmAHIAYQBjAHQAaQBvAG4AXABuAE0ATQBTAGoAbQAxADcAOQBUADEAIAA9ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAbQBhAG4AdQByAGUAIABpAG4AIABNAE0AUwAgADEALAAgADcALAAgAGEAbgBkACAAOQAgAGkAbgAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMQAgADoAIABmAHIAYQBjAHQAaQBvAG4AXABuAFMAUwBtACAAPQAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAHYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZABzACAAcwBlAHAAYQByAGEAdABlAGQAIAB0AG8AIABzAG8AbABpAGQAIABzAHQAbwByAGEAZwBlACAAZgBvAHIAIABlAGEAYwBoACAATQBNAFMAIAA6ACAAZgByAGEAYwB0AGkAbwBuAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADUAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0ATQBTAGoAbQA0AFQAMQAsACAATQBNAFMAagBtADEANwA5AFQAMQAsACAAUwBTAG0ALABcAG4AIAAgACAAIABNAE0AUwBqAG0ANABUADEAIAArACAAKABNAE0AUwBqAG0AMQA3ADkAVAAxACAAKgAgAFMAUwBtACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA1AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAE0AUwBqAG0ANABUADEALABcAG4AIAAgACAAIABNAE0AUwBqAG0AVAAxAF8AMQAsACAATQBNAFMAagBtAFQAMQBfADIALAAgAE0ATQBTAGoAbQBUADEAXwAzACwAIABNAE0AUwBqAG0AVAAxAF8ANAAsACAATQBNAFMAagBtAFQAMQBfADUALABcAG4AIAAgACAAIABTAFMAagBtAFQAMQBfADEALAAgAFMAUwBqAG0AVAAxAF8AMgAsACAAUwBTAGoAbQBUADEAXwAzACwAIABTAFMAagBtAFQAMQBfADQALAAgAFMAUwBqAG0AVAAxAF8ANQAsAFwAbgAgACAAIAAgACAAIABNAE0AUwBqAG0ANABUADEAIAArACAAXABuACAAIAAgACAAIAAgACgATQBNAFMAagBtAFQAMQBfADEAIAAqACAAUwBTAGoAbQBUADEAXwAxACkAIAArACAAXABuACAAIAAgACAAIAAgACgATQBNAFMAagBtAFQAMQBfADIAIAAqACAAUwBTAGoAbQBUADEAXwAyACkAIAArACAAXABuACAAIAAgACAAIAAgACgATQBNAFMAagBtAFQAMQBfADMAIAAqACAAUwBTAGoAbQBUADEAXwAzACkAIAArAFwAbgAgACAAIAAgACAAIAAoAE0ATQBTAGoAbQBUADEAXwA0ACAAKgAgAFMAUwBqAG0AVAAxAF8ANAApACAAKwBcAG4AIAAgACAAIAAgACAAKABNAE0AUwBqAG0AVAAxAF8ANQAgACoAIABTAFMAagBtAFQAMQBfADUAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADUAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIAB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgAGkAbgAgAHMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADUAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAFYAUwBqAG0ANABUADEAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADUAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA1AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4ANQAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADUAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADUAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBWAFMAXwB7AGoALABtAD0ANAAsAFQAPQAxAH0APQBNAE0AUwBfAHsAagAsAG0APQA0ACwAVAA9ADEAfQArACgATQBNAFMAXwB7AGoALABtAD0AMQAsADcALAA5ACwAVAA9ADEAfQBcAFwAdABpAG0AZQBzACAAUwBTAF8AewBtAH0AKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAFYAUwBfAHsAagAsAG0APQA0ACwAVAA9ADEAfQA9AE0ATQBTAF8AewBqACwAbQA9ADQALABUAD0AMQB9ACsAKABNAE0AUwBfAHsAagAsAG0APQAxACwAVAA9ADEAfQBcAFwAdABpAG0AZQBzACAAUwBTAF8AewBtAD0AMQAsAFQAPQAxAH0AKQArACgATQBNAFMAXwB7AGoALABtAD0ANwAsAFQAPQAxAH0AXABcAHQAaQBtAGUAcwAgAFMAUwBfAHsAbQA9ADcALABUAD0AMQB9ACkAKwAoAE0ATQBTAF8AewBqACwAbQA9ADkALABUAD0AMQB9AFwAXAB0AGkAbQBlAHMAIABTAFMAXwB7AG0APQA5ACwAVAA9ADEAfQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA1AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE0AUwBqAG0ANABUADEAXAAiACwAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG0AYQBuAHUAcgBlACAAaQBuACAAcwBvAGwAaQBkACAAcwB0AG8AcgBhAGcAZQAgAHAAcgBpAG0AYQByAHkAIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE0AUwBqAG0AMQA3ADkAVAAxAFwAIgAsAFwAIgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABtAGEAbgB1AHIAZQAgAGkAbgAgAE0ATQBTACAAMQAsACAANwAsACAAYQBuAGQAIAA5ACAAaQBuACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAAxAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAUwBtAFwAIgAsAFwAIgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIAB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgAHMAZQBwAGEAcgBhAHQAZQBkACAAdABvACAAcwBvAGwAaQBkACAAcwB0AG8AcgBhAGcAZQAgAGYAbwByACAAZQBhAGMAaAAgAE0ATQBTAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA1AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFADoAIABTAHAAbABpAHQAIABlAHEAdQBhAHQAaQBvAG4AIABmAG8AcgAgAE0ATQBTAG0APQAxACwANwAsADkAIABpAG4AdABvACAAcwBlAHAAYQByAGEAdABlACAAaQB0AGUAbQBzACAAdABvACAAYQBsAGwAbwB3ACAAZgBvAHIAIABjAGEAbABjAHUAbABhAHQAaQBvAG4AXAAiACkAOwBcAG4AIAAgAFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADYAXwBTAHQAYQBnAGUAMgBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXABuAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABvAGYAIABtAGUAdABoAGEAbgBlACAAaQBuACAAZQBhAGMAaAAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMgAgAE0ATQBTAFwAbgBNAGkAagBtAFQAMgBcAG4AawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXABuAE0AXwB7AGkAagBtACwAVAA9ADIAfQA9AFYAUwBUAF8AewBqAG0ALABUAD0AMgB9AFwAXAB0AGkAbQBlAHMAIABCAE8AXABcAHQAaQBtAGUAcwAgAE0ATQBTAF8AewBqAG0ALABUAD0AMgB9AFwAXAB0AGkAbQBlAHMAIABNAEMARgBfAHsAaQBtAH0AXABcAHQAaQBtAGUAcwAgAFwAXAByAGgAbwBcAG4AVgBTAFQAagBtAFQAMgAgAD0AIAB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgAHQAcgBhAG4AcwBmAGUAcgByAGUAZAAgAHQAbwAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMgAgAE0ATQBTACAAOgAgAGsAZwAvAGgAZQBhAGQALwBkAGEAeQBcAG4AQgBPACAAPQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAcABvAHQAZQBuAHQAaQBhAGwAIAA6ACAAbQAzACAAQwBIADQALwBrAGcAIABWAFMAXABuAE0ATQBTAGoAbQBUADIAIAA9ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAbQBhAG4AdQByAGUAIABpAG4AIABlAGEAYwBoACAAcwBlAGMAbwBuAGQAYQByAHkAIABzAHkAcwB0AGUAbQAgADoAIABmAHIAYQBjAHQAaQBvAG4AXABuAE0AQwBGAGkAbQAgAD0AIABtAGUAdABoAGEAbgBlACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAHoAbwBuAGUAIABhAG4AZAAgAHMAeQBzAHQAZQBtACAAOgAgAGYAcgBhAGMAdABpAG8AbgBcAG4AcgBoAG8AIAA9ACAAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAIAA6ACAAawBnAC8AbQAzAFwAbgBpACAAPQAgAHMAdABhAHQAZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA2AF8AUwB0AGEAZwBlADIATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFYAUwBUAGoAbQBUADIALAAgAEIATwAsACAATQBNAFMAagBtAFQAMgAsACAATQBDAEYAaQBtACwAIAByAGgAbwAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgAFYAUwBUAGoAbQBUADIALAAgAEkARgAoAEkAUwBOAFUATQBCAEUAUgAoAFYAUwBUAGoAbQBUADIAKQAsACAAVgBTAFQAagBtAFQAMgAsACAAMAApACwAXABuACAAIAAgACAAIAAgAE0ATQBTAGoAbQBUADIALAAgAEkARgAoAEkAUwBOAFUATQBCAEUAUgAoAE0ATQBTAGoAbQBUADIAKQAsACAATQBNAFMAagBtAFQAMgAsACAAMAApACwAXABuACAAIAAgACAAIAAgAFYAUwBUAGoAbQBUADIAIAAqACAAQgBPACAAKgAgAE0ATQBTAGoAbQBUADIAIAAqACAATQBDAEYAaQBtACAAKgAgAHIAaABvAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA2AF8AUwB0AGEAZwBlADIATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAbwBmACAAbQBlAHQAaABhAG4AZQAgAGkAbgAgAGUAYQBjAGgAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADIAIABNAE0AUwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANgBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBpAGoAbQBUADIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADYAXwBTAHQAYQBnAGUAMgBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANgBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4ANQAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADYAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANgBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANgBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AXwB7AGkAagBtACwAVAA9ADIAfQA9AFYAUwBUAF8AewBqAG0ALABUAD0AMgB9AFwAXAB0AGkAbQBlAHMAIABCAE8AXABcAHQAaQBtAGUAcwAgAE0ATQBTAF8AewBqAG0ALABUAD0AMgB9AFwAXAB0AGkAbQBlAHMAIABNAEMARgBfAHsAaQBtAH0AXABcAHQAaQBtAGUAcwAgAFwAXAByAGgAbwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANgBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAFMAVABqAG0AVAAyAFwAIgAsAFwAIgB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgAHQAcgBhAG4AcwBmAGUAcgByAGUAZAAgAHQAbwAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMgAgAE0ATQBTAFwAIgAsACAAXAAiAGsAZwAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADQALgA1AC4AMQAuADEAIAAoADcAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgBPAFwAIgAsAFwAIgBlAG0AaQBzAHMAaQBvAG4AcwAgAHAAbwB0AGUAbgB0AGkAYQBsAFwAIgAsACAAXAAiAG0AMwAgAEMASAA0AC8AawBnACAAVgBTAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBNAFMAagBtAFQAMgBcACIALABcACIAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAbQBhAG4AdQByAGUAIABpAG4AIABlAGEAYwBoACAAcwBlAGMAbwBuAGQAYQByAHkAIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEMARgBpAG0AXAAiACwAXAAiAG0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHQAZQBtAHAAZQByAGEAdABlACAAegBvAG4AZQAgAGEAbgBkACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAcgBoAG8AXAAiACwAXAAiAGQAZQBuAHMAaQB0AHkAIABvAGYAIABtAGUAdABoAGEAbgBlAFwAIgAsACAAXAAiAGsAZwAvAG0AMwBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAGkAXAAiACwAXAAiAHMAdABhAHQAZQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA2AF8AUwB0AGEAZwBlADIATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AQQByAGcAdQBtAGUAbgB0AHMAXwBNAGUAdABoAG8AZAAyAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAFMAVABqAG0AVAAyAFwAIgAsAFwAIgB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgAHQAcgBhAG4AcwBmAGUAcgByAGUAZAAgAHQAbwAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMgAgAE0ATQBTAFwAIgAsACAAXAAiAGsAZwAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADQALgA1AC4AMQAuADEAIAAoADcAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgBPAFwAIgAsAFwAIgBlAG0AaQBzAHMAaQBvAG4AcwAgAHAAbwB0AGUAbgB0AGkAYQBsAFwAIgAsACAAXAAiAG0AMwAgAEMASAA0AC8AawBnACAAVgBTAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBNAFMAagBtAFQAMgBcACIALABcACIAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAbQBhAG4AdQByAGUAIABpAG4AIABlAGEAYwBoACAAcwBlAGMAbwBuAGQAYQByAHkAIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEMARgBpAG0AXAAiACwAXAAiAG0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHQAZQBtAHAAZQByAGEAdABlACAAegBvAG4AZQAgAGEAbgBkACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAcgBoAG8AXAAiACwAXAAiAGQAZQBuAHMAaQB0AHkAIABvAGYAIABtAGUAdABoAGEAbgBlAFwAIgAsACAAXAAiAGsAZwAvAG0AMwBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQQBUAFwAIgAsAFwAIgBNAGUAYQBuACAAYQBuAG4AdQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAXAAiACwAIABcACIAsABDAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANwBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBUAHIAYQBuAHMAZgBlAHIAcgBlAGQAUwB0AGEAZwBlADIAXABuAFYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZABzACAAdAByAGEAbgBzAGYAZQByAHIAZQBkACAAdABvACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAAyACAATQBNAFMAXABuAFYAUwBUAGkAagBtAFQAMgBcAG4AawBnACAAVgBTAFwAbgBWAFMAVABfAHsAaQBqAG0ALABUAD0AMgB9AD0AVgBTAF8AewBqAH0AXABcAHQAaQBtAGUAcwAgAEYAVgBTAF8AewBqAG0ALABUAD0AMQB9AFwAXAB0AGkAbQBlAHMAKAAxAC0AVgBTAEwAXwB7AG0ALABUAD0AMQB9ACkAXABuAFYAUwBqACAAPQAgAHYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZAAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAHIAbwBtACAAcwB3AGkAbgBlACAAaQBuACAAZQBhAGMAaAAgAGMAbABhAHMAcwAgADoAIABrAGcALwBoAGUAYQBkAC8AZABhAHkAXABuAEYAVgBTAGoAbQBUADEAIAA9ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkAHMAIABpAG4AIABlAGEAYwBoACAAcAByAGkAbQBhAHIAeQAgAHMAeQBzAHQAZQBtACAAOgAgAGYAcgBhAGMAdABpAG8AbgBcAG4AVgBTAEwAbQBUADEAIAA9ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkAHMAIABsAG8AcwB0ACAAZAB1AHIAaQBuAGcAIABzAHQAbwByAGEAZwBlACAAaQBuACAAdABoAGUAIABwAHIAaQBtAGEAcgB5ACAAcwB5AHMAdABlAG0AIAA6ACAAZgByAGEAYwB0AGkAbwBuAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADcAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVAByAGEAbgBzAGYAZQByAHIAZQBkAFMAdABhAGcAZQAyAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFYAUwBqACwAIABGAFYAUwBqAG0AVAAxACwAIABWAFMATABtAFQAMQAsAFwAbgAgACAAIAAgAFYAUwBqACAAKgAgAEYAVgBTAGoAbQBUADEAIAAqACAAKAAxACAALQAgAFYAUwBMAG0AVAAxACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA3AF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFQAcgBhAG4AcwBmAGUAcgByAGUAZABTAHQAYQBnAGUAMgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkAHMAIAB0AHIAYQBuAHMAZgBlAHIAcgBlAGQAIAB0AG8AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADIAIABNAE0AUwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANwBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBUAHIAYQBuAHMAZgBlAHIAcgBlAGQAUwB0AGEAZwBlADIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAUwBUAGkAagBtAFQAMgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANwBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBUAHIAYQBuAHMAZgBlAHIAcgBlAGQAUwB0AGEAZwBlADIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABWAFMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADcAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVAByAGEAbgBzAGYAZQByAHIAZQBkAFMAdABhAGcAZQAyAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgA1AC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgANwApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA3AF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFQAcgBhAG4AcwBmAGUAcgByAGUAZABTAHQAYQBnAGUAMgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANwBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBUAHIAYQBuAHMAZgBlAHIAcgBlAGQAUwB0AGEAZwBlADIAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAFMAVABfAHsAaQBqAG0ALABUAD0AMgB9AD0AVgBTAF8AewBqAH0AXABcAHQAaQBtAGUAcwAgAEYAVgBTAF8AewBqAG0ALABUAD0AMQB9AFwAXAB0AGkAbQBlAHMAKAAxAC0AVgBTAEwAXwB7AG0ALABUAD0AMQB9ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADcAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVAByAGEAbgBzAGYAZQByAHIAZQBkAFMAdABhAGcAZQAyAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAUwBqAFwAIgAsAFwAIgB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgByAG8AbQAgAHMAdwBpAG4AZQAgAGkAbgAgAGUAYQBjAGgAIABjAGwAYQBzAHMAXAAiACwAIABcACIAawBnAC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBWAFMAagBtAFQAMQBcACIALABcACIAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkAHMAIABpAG4AIABlAGEAYwBoACAAcAByAGkAbQBhAHIAeQAgAHMAeQBzAHQAZQBtAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADQALgA1AC4AMQAuADEAIAAoADQAKQAoADUAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBTAEwAbQBUADEAXAAiACwAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAHYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZABzACAAbABvAHMAdAAgAGQAdQByAGkAbgBnACAAcwB0AG8AcgBhAGcAZQAgAGkAbgAgAHQAaABlACAAcAByAGkAbQBhAHIAeQAgAHMAeQBzAHQAZQBtAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBMAG8AbwBrAHUAcABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ANAAuADUAOgAgAFMAdwBpAG4AZQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ANAAuADUALgAxAC4AMwAgAE0AZQB0AGgAbwBkACAAMQAgAC0AIABNAGEAbgB1AHIAZQAgAEQAaQByAGUAYwB0ACAATgAyAE8AIABTAHcAaQBuAGUAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0ATQBNAFMAXABuAFQAbwB0AGEAbAAgAGEAbgBuAHUAYQBsACAAZABpAHIAZQBjAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAAbQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAcwB5AHMAdABlAG0AcwBcAG4ARQBfAE4AMgBPAGQAaQByAFwAbgB0ACAATgAyAE8AXABuAEUAXwB7AE4AMgBPACwAZABpAHIAfQA9AFwAXABzAHUAbQBfAHsAagB9AFwAXABzAHUAbQBfAHsAbQB9AFwAXABzAHUAbQBfAHsAVAB9ACgATQBOAF8AewBqAG0AVAB9AFwAXAB0AGkAbQBlAHMAIABFAEYAXwB7AGoAbQB9AFwAXAB0AGkAbQBlAHMAIABDAF8AewBOADIATwB9ACkAXABcAHQAaQBtAGUAcwAxADAAXgB7AC0AMwB9AFwAbgBNAE4AXwBqAG0AVAAgAD0AIABuAGkAdAByAG8AZwBlAG4AIABwAGUAcgAgAHMAdwBpAG4AZQAgAGMAbABhAHMAcwAsACAATQBNAFMAIABhAG4AZAAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAKABrAGcAIABOACkAXABuAEUARgBfAGoAbQAgAD0AIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAE0ATQBTACAAKABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACkAXABuAEMAXwBOADIATwAgAD0AIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwARABpAHIAZQBjAHQATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBNAE0AUwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAE4AXwBqAG0AVAAsACAARQBGAF8AagBtACwAIABDAF8ATgAyAE8ALABcAG4AIAAgACAAIABNAE4AXwBqAG0AVAAgACoAIABFAEYAXwBqAG0AIAAqACAAQwBfAE4AMgBPACAAKgAgADEAMAAgAF4AIAAtADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0ATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAbwB0AGEAbAAgAGEAbgBuAHUAYQBsACAAZABpAHIAZQBjAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAAbQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAcwB5AHMAdABlAG0AcwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABEAGkAcgBlAGMAdABOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAE0ATQBTAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8ATgAyAE8AZABpAHIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwARABpAHIAZQBjAHQATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBNAE0AUwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABOADIATwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABEAGkAcgBlAGMAdABOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAE0ATQBTAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgA1AC4AMQAuADMALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0ATQBNAFMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwARABpAHIAZQBjAHQATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBNAE0AUwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwB7AE4AMgBPACwAZABpAHIAfQA9AFwAXABzAHUAbQBfAHsAagB9AFwAXABzAHUAbQBfAHsAbQB9AFwAXABzAHUAbQBfAHsAVAB9ACgATQBOAF8AewBqAG0AVAB9AFwAXAB0AGkAbQBlAHMAIABFAEYAXwB7AGoAbQB9AFwAXAB0AGkAbQBlAHMAIABDAF8AewBOADIATwB9ACkAXABcAHQAaQBtAGUAcwAxADAAXgB7AC0AMwB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0ATQBNAFMAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBOAF8AagBtAFQAXAAiACwAIABcACIAbgBpAHQAcgBvAGcAZQBuACAAcABlAHIAIABzAHcAaQBuAGUAIABjAGwAYQBzAHMALAAgAE0ATQBTACAAYQBuAGQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQBcACIALAAgAFwAIgBrAGcAIABOAFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAANAAuADUALgAxAC4AMwAgACgAMgApACgANgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEYAXwBqAG0AXAAiACwAIABcACIAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABNAE0AUwBcACIALAAgAFwAIgBrAGcAIABOADIATwAtAE4ALwBrAGcAIABOAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBfAE4AMgBPAFwAIgAsACAAXAAiAGYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXAAiACwAIABcACIAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADIAXwBTAHQAYQBnAGUAMQBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAFwAbgBOAGkAdAByAG8AZwBlAG4AIABpAG4AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADEAIABNAE0AUwBcAG4ATQBOAF8AagBtAFQAMQBcAG4AawBnACAATgBcAG4ATQBOAF8AewBqAG0ALABUAD0AMQB9AD0AQQBFAF8AewBqAH0AXABcAHQAaQBtAGUAcwAgAEYATgBfAHsAagBtACwAVAA9ADEAfQBcAG4AQQBFAF8AagAgAD0AIAB0AG8AdABhAGwAIABuAGkAdAByAG8AZwBlAG4AIABlAHgAYwByAGUAdABlAGQAIABiAHkAIABlAGEAYwBoACAAcwB3AGkAbgBlACAAYwBsAGEAcwBzACAAKABrAGcAIABOACkAXABuAEYATgBfAGoAbQBUADEAIAA9ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAaQBuACAAZQBhAGMAaAAgAHAAcgBpAG0AYQByAHkAIABNAE0AUwAgAHMAeQBzAHQAZQBtAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADIAXwBTAHQAYQBnAGUAMQBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEEARQBfAGoALAAgAEYATgBfAGoAbQBUADEALABcAG4AIAAgACAAIABBAEUAXwBqACAAKgAgAEYATgBfAGoAbQBUADEAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwAyAF8AUwB0AGEAZwBlADEATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBpAHQAcgBvAGcAZQBuACAAaQBuACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAAxACAATQBNAFMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADIAXwBTAHQAYQBnAGUAMQBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE4AXwBqAG0AVAAxAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwAyAF8AUwB0AGEAZwBlADEATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADIAXwBTAHQAYQBnAGUAMQBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgA1AC4AMQAuADMALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMgApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwAyAF8AUwB0AGEAZwBlADEATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8AMgBfAFMAdABhAGcAZQAxAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE4AXwB7AGoAbQAsAFQAPQAxAH0APQBBAEUAXwB7AGoAfQBcAFwAdABpAG0AZQBzACAARgBOAF8AewBqAG0ALABUAD0AMQB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwAyAF8AUwB0AGEAZwBlADEATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAEUAXwBqAFwAIgAsACAAXAAiAHQAbwB0AGEAbAAgAG4AaQB0AHIAbwBnAGUAbgAgAGUAeABjAHIAZQB0AGUAZAAgAGIAeQAgAGUAYQBjAGgAIABzAHcAaQBuAGUAIABjAGwAYQBzAHMAXAAiACwAIABcACIAawBnACAATgBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADQALgA1AC4AMQAuADMAIAAoADUAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBOAF8AagBtAFQAMQBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABuAGkAdAByAG8AZwBlAG4AIABpAG4AIABlAGEAYwBoACAAcAByAGkAbQBhAHIAeQAgAE0ATQBTACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAANAAuADUALgAxAC4AMwAgACgAMwApACgANAApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADMAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBJAG4AUAByAGkAbQBhAHIAeQBNAE0AUwBcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAaQBuACAAZQBhAGMAaAAgAHAAcgBpAG0AYQByAHkAIABNAE0AUwAgACgAZQB4AGMAbAB1AGQAaQBuAGcAIABzAG8AbABpAGQAIABzAHQAbwByAGEAZwBlACkAXABuAEYATgBfAGoAbQBUADEAXABuAGYAcgBhAGMAdABpAG8AbgBcAG4ARgBOAF8AewBqAG0ALABUAD0AMQB9AD0ATQBNAFMAXwB7AGoAbQAsAFQAPQAxAH0AXABcAHQAaQBtAGUAcwAoADEALQBTAE4AXwB7AG0AfQApAFwAbgBNAE0AUwBfAGoAbQBUADEAIAA9ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAbQBhAG4AdQByAGUAIABpAG4AIABwAHIAaQBtAGEAcgB5ACAATQBNAFMAXABuAFMATgBfAG0AIAA9ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAcwBlAHAAYQByAGEAdABlAGQAIAB0AG8AIABzAG8AbABpAGQAIABzAHQAbwByAGEAZwBlACAAZgBvAHIAIABlAGEAYwBoACAATQBNAFMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8AMwBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEkAbgBQAHIAaQBtAGEAcgB5AE0ATQBTAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0ATQBTAF8AagBtAFQAMQAsACAAUwBOAF8AbQAsAFwAbgAgACAAIAAgAE0ATQBTAF8AagBtAFQAMQAgACoAIAAoADEAIAAtACAAUwBOAF8AbQApAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8AMwBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEkAbgBQAHIAaQBtAGEAcgB5AE0ATQBTAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABuAGkAdAByAG8AZwBlAG4AIABpAG4AIABlAGEAYwBoACAAcAByAGkAbQBhAHIAeQAgAE0ATQBTACAAKABlAHgAYwBsAHUAZABpAG4AZwAgAHMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8AMwBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEkAbgBQAHIAaQBtAGEAcgB5AE0ATQBTAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAE4AXwBqAG0AVAAxAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwAzAF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ASQBuAFAAcgBpAG0AYQByAHkATQBNAFMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADMAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBJAG4AUAByAGkAbQBhAHIAeQBNAE0AUwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4ANQAuADEALgAzACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADMAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8AMwBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEkAbgBQAHIAaQBtAGEAcgB5AE0ATQBTAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwAzAF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ASQBuAFAAcgBpAG0AYQByAHkATQBNAFMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAE4AXwB7AGoAbQAsAFQAPQAxAH0APQBNAE0AUwBfAHsAagBtACwAVAA9ADEAfQBcAFwAdABpAG0AZQBzACgAMQAtAFMATgBfAHsAbQB9ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADMAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBJAG4AUAByAGkAbQBhAHIAeQBNAE0AUwBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE0AUwBfAGoAbQBUADEAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAbQBhAG4AdQByAGUAIABpAG4AIABwAHIAaQBtAGEAcgB5ACAATQBNAFMAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBOAF8AbQBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABuAGkAdAByAG8AZwBlAG4AIABzAGUAcABhAHIAYQB0AGUAZAAgAHQAbwAgAHMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAIABmAG8AcgAgAGUAYQBjAGgAIABNAE0AUwBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADQAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBJAG4AUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG4AaQB0AHIAbwBnAGUAbgAgAGkAbgAgAHMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXABuAEYATgBfAGoAbQA0AFQAMQBcAG4AZgByAGEAYwB0AGkAbwBuAFwAbgBGAE4AXwB7AGoAbQA9ADQALABUAD0AMQB9AD0ATQBNAFMAXwB7AGoAbQA9ADQALABUAD0AMQB9ACsAKABNAE0AUwBfAHsAagBtAD0AMQAsADcALAA5ACwAVAA9ADEAfQBcAFwAdABpAG0AZQBzACAAUwBOAF8AewBtAH0AKQBcAG4ATQBNAFMAXwBqAG0ANABUADEAIAA9ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAbQBhAG4AdQByAGUAIABpAG4AIABzAG8AbABpAGQAIABzAHQAbwByAGEAZwBlACAATQBNAFMAXABuAE0ATQBTAF8AagBtADEANwA5AFQAMQAgAD0AIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABtAGEAbgB1AHIAZQAgAGkAbgAgAHAAcgBpAG0AYQByAHkAIABsAGkAcQB1AGkAZAAgAHMAeQBzAHQAZQBtAHMAIAAoAG0APQAxACwANwAsADkAKQBcAG4AUwBOAF8AbQAgAD0AIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABuAGkAdAByAG8AZwBlAG4AIABzAGUAcABhAHIAYQB0AGUAZAAgAHQAbwAgAHMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAIABmAG8AcgAgAGUAYQBjAGgAIABNAE0AUwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA0AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ASQBuAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0ATQBTAF8AagBtADQAVAAxACwAIABNAE0AUwBfAGoAbQAxADcAOQBUADEALAAgAFMATgBfAG0ALABcAG4AIAAgACAAIABNAE0AUwBfAGoAbQA0AFQAMQAgACsAIAAoAE0ATQBTAF8AagBtADEANwA5AFQAMQAgACoAIABTAE4AXwBtACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA0AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ASQBuAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0ATQBTAF8AagBtADQAVAAxACwAXABuACAAIAAgACAATQBNAFMAagBtAFQAMQBfADEALAAgAE0ATQBTAGoAbQBUADEAXwAyACwAIABNAE0AUwBqAG0AVAAxAF8AMwAsACAATQBNAFMAagBtAFQAMQBfADQALAAgAE0ATQBTAGoAbQBUADEAXwA1ACwAXABuACAAIAAgACAAUwBTAGoAbQBUADEAXwAxACwAIABTAFMAagBtAFQAMQBfADIALAAgAFMAUwBqAG0AVAAxAF8AMwAsACAAUwBTAGoAbQBUADEAXwA0ACwAIABTAFMAagBtAFQAMQBfADUALABcAG4AIAAgACAAIABNAE0AUwBfAGoAbQA0AFQAMQAgACsAIAAoAE0ATQBTAGoAbQBUADEAXwAxACAAKgAgAFMAUwBqAG0AVAAxAF8AMQApACAAKwAgACgATQBNAFMAagBtAFQAMQBfADIAIAAqACAAUwBTAGoAbQBUADEAXwAyACkAIAArACAAKABNAE0AUwBqAG0AVAAxAF8AMwAgACoAIABTAFMAagBtAFQAMQBfADMAKQAgACsAIAAoAE0ATQBTAGoAbQBUADEAXwA0ACAAKgAgAFMAUwBqAG0AVAAxAF8ANAApACAAKwAgACgATQBNAFMAagBtAFQAMQBfADUAIAAqACAAUwBTAGoAbQBUADEAXwA1ACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA0AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ASQBuAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABuAGkAdAByAG8AZwBlAG4AIABpAG4AIABzAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA0AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ASQBuAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAE4AXwBqAG0ANABUADEAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADQAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBJAG4AUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADQAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBJAG4AUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADUALgAxAC4AMwAsACAARQBxAHUAYQB0AGkAbwBuACAAKAA0ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADQAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBJAG4AUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADQAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBJAG4AUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAE4AXwB7AGoAbQA9ADQALABUAD0AMQB9AD0ATQBNAFMAXwB7AGoAbQA9ADQALABUAD0AMQB9ACsAKABNAE0AUwBfAHsAagBtAD0AMQAsADcALAA5ACwAVAA9ADEAfQBcAFwAdABpAG0AZQBzACAAUwBOAF8AewBtAH0AKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8ANABfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEkAbgBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYATgBfAHsAagBtAD0ANAAsAFQAPQAxAH0APQBNAE0AUwBfAHsAagBtAD0ANAAsAFQAPQAxAH0AKwAoAE0ATQBTAF8AewBqACwAbQA9ADEALABUAD0AMQB9AFwAXAB0AGkAbQBlAHMAIABTAFMAXwB7AG0APQAxACwAVAA9ADEAfQApACsAKABNAE0AUwBfAHsAagAsAG0APQA3ACwAVAA9ADEAfQBcAFwAdABpAG0AZQBzACAAUwBTAF8AewBtAD0ANwAsAFQAPQAxAH0AKQArACgATQBNAFMAXwB7AGoALABtAD0AOQAsAFQAPQAxAH0AXABcAHQAaQBtAGUAcwAgAFMAUwBfAHsAbQA9ADkALABUAD0AMQB9ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADQAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBJAG4AUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBNAFMAXwBqAG0ANABUADEAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAbQBhAG4AdQByAGUAIABpAG4AIABzAG8AbABpAGQAIABzAHQAbwByAGEAZwBlACAATQBNAFMAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBNAFMAXwBqAG0AMQA3ADkAVAAxAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG0AYQBuAHUAcgBlACAAaQBuACAAcAByAGkAbQBhAHIAeQAgAGwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwAgACgAbQA9ADEALAA3ACwAOQApAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMATgBfAG0AXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAcwBlAHAAYQByAGEAdABlAGQAIAB0AG8AIABzAG8AbABpAGQAIABzAHQAbwByAGEAZwBlACAAZgBvAHIAIABlAGEAYwBoACAATQBNAFMAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADQAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBJAG4AUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6ACAAUwBwAGwAaQB0ACAAZQBxAHUAYQB0AGkAbwBuACAAZgBvAHIAIABNAE0AUwBtAD0AMQAsADcALAA5ACAAaQBuAHQAbwAgAHMAZQBwAGEAcgBhAHQAZQAgAGkAdABlAG0AcwAgAHQAbwAgAGEAbABsAG8AdwAgAGYAbwByACAAYwBhAGwAYwB1AGwAYQB0AGkAbwBuAFwAIgApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8ANQBfAEEAbgBuAHUAYQBsAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBcAG4AQQBuAG4AdQBhAGwAIABuAGkAdAByAG8AZwBlAG4AIABlAHgAYwByAGUAdABpAG8AbgAgAGYAcgBvAG0AIABlAGEAYwBoACAAcwB3AGkAbgBlACAAZwByAG8AdQBwAFwAbgBBAEUAXwBqAFwAbgBrAGcAIABOAFwAbgBBAEUAXwB7AGoAfQA9AE4AXwB7AGoAfQBcAFwAdABpAG0AZQBzACAATgBXAF8AewBqAH0AXABcAHQAaQBtAGUAcwAgAEQAXwB7AGoAfQBcAG4ATgBfAGoAIAA9ACAAbgB1AG0AYgBlAHIAIABvAGYAIABzAHcAaQBuAGUAIABpAG4AIABlAGEAYwBoACAAZwByAG8AdQBwACAAKABoAGUAYQBkACkAXABuAE4AVwBfAGoAIAA9ACAAbgBpAHQAcgBvAGcAZQBuACAAcAByAG8AZAB1AGMAZQBkACAAaQBuACAAcwB3AGkAbgBlACAAbQBhAG4AdQByAGUAIABhAG4AZAAgAHcAYQBzAHQAZQAgAGYAZQBlAGQAIABpAG4AIABlAGEAYwBoACAAYwBsAGEAcwBzACAAKABrAGcAIABOAC8AaABlAGEAZAAvAGQAYQB5ACkAXABuAEQAXwBqACAAPQAgAGQAdQByAGEAdABpAG8AbgAgAG8AZgAgAHMAdABhAHkAIABvAGYAIABzAHcAaQBuAGUAIABnAHIAbwB1AHAAIAAoAGQAYQB5AHMAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA1AF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE4AXwBqACwAIABOAFcAXwBqACwAIABEAF8AagAsAFwAbgAgACAAIAAgAE4AXwBqACAAKgAgAE4AVwBfAGoAIAAqACAARABfAGoAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA1AF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAG4AbgB1AGEAbAAgAG4AaQB0AHIAbwBnAGUAbgAgAGUAeABjAHIAZQB0AGkAbwBuACAAZgByAG8AbQAgAGUAYQBjAGgAIABzAHcAaQBuAGUAIABnAHIAbwB1AHAAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADUAXwBBAG4AbgB1AGEAbABOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAaQBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEARQBfAGoAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADUAXwBBAG4AbgB1AGEAbABOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA1AF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgA1AC4AMQAuADMALAAgAEUAcQB1AGEAdABpAG8AbgAgACgANQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA1AF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA1AF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBFAF8AewBqAH0APQBOAF8AewBqAH0AXABcAHQAaQBtAGUAcwAgAE4AVwBfAHsAagB9AFwAXAB0AGkAbQBlAHMAIABEAF8AewBqAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADUAXwBBAG4AbgB1AGEAbABOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBfAGoAXAAiACwAIABcACIAbgB1AG0AYgBlAHIAIABvAGYAIABzAHcAaQBuAGUAIABpAG4AIABlAGEAYwBoACAAZwByAG8AdQBwAFwAIgAsACAAXAAiAGgAZQBhAGQAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAFcAXwBqAFwAIgAsACAAXAAiAG4AaQB0AHIAbwBnAGUAbgAgAHAAcgBvAGQAdQBjAGUAZAAgAGkAbgAgAHMAdwBpAG4AZQAgAG0AYQBuAHUAcgBlACAAYQBuAGQAIAB3AGEAcwB0AGUAIABmAGUAZQBkACAAaQBuACAAZQBhAGMAaAAgAGMAbABhAHMAcwBcACIALAAgAFwAIgBrAGcAIABOAC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABfAGoAXAAiACwAIABcACIAZAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAG8AZgAgAHMAdwBpAG4AZQAgAGcAcgBvAHUAcABcACIALAAgAFwAIgBkAGEAeQBzAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA2AF8AUwB0AGEAZwBlADIATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBcAG4ATgBpAHQAcgBvAGcAZQBuACAAaQBuACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAAyACAATQBNAFMAXABuAE0ATgBfAGoAbQBUADIAXABuAGsAZwAgAE4AXABuAE0ATgBfAHsAagBtACwAVAA9ADIAfQA9AE4AVABfAHsAagBtACwAVAA9ADIAfQBcAFwAdABpAG0AZQBzACAATQBNAFMAXwB7AGoAbQAsAFQAPQAyAH0AXABuAE4AVABfAGoAbQBUADIAIAA9ACAAbgBpAHQAcgBvAGcAZQBuACAAdAByAGEAbgBzAGYAZQByAHIAZQBkACAAdABvACAAcwBlAGMAbwBuAGQAYQByAHkAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAE0ATQBTACAAKABrAGcAIABOACkAXABuAE0ATQBTAF8AagBtAFQAMgAgAD0AIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABtAGEAbgB1AHIAZQAgAGkAbgAgAGUAYQBjAGgAIABzAGUAYwBvAG4AZABhAHIAeQAgAHMAeQBzAHQAZQBtAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADYAXwBTAHQAYQBnAGUAMgBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE4AVABfAGoAbQBUADIALAAgAE0ATQBTAF8AagBtAFQAMgAsAFwAbgAgACAAIAAgAE4AVABfAGoAbQBUADIAIAAqACAATQBNAFMAXwBqAG0AVAAyAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8ANgBfAFMAdABhAGcAZQAyAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwBnAGUAbgAgAGkAbgAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMgAgAE0ATQBTAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA2AF8AUwB0AGEAZwBlADIATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBOAF8AagBtAFQAMgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8ANgBfAFMAdABhAGcAZQAyAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA2AF8AUwB0AGEAZwBlADIATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4ANQAuADEALgAzACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADYAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8ANgBfAFMAdABhAGcAZQAyAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADYAXwBTAHQAYQBnAGUAMgBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBOAF8AewBqAG0ALABUAD0AMgB9AD0ATgBUAF8AewBqAG0ALABUAD0AMgB9AFwAXAB0AGkAbQBlAHMAIABNAE0AUwBfAHsAagBtACwAVAA9ADIAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8ANgBfAFMAdABhAGcAZQAyAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBUAF8AagBtAFQAMgBcACIALAAgAFwAIgBuAGkAdAByAG8AZwBlAG4AIAB0AHIAYQBuAHMAZgBlAHIAcgBlAGQAIAB0AG8AIABzAGUAYwBvAG4AZABhAHIAeQAgAHQAcgBlAGEAdABtAGUAbgB0ACAATQBNAFMAXAAiACwAIABcACIAawBnACAATgBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADQALgA1AC4AMQAuADMAIAAoADcAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBNAFMAXwBqAG0AVAAyAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG0AYQBuAHUAcgBlACAAaQBuACAAZQBhAGMAaAAgAHMAZQBjAG8AbgBkAGEAcgB5ACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA3AF8ATgBpAHQAcgBvAGcAZQBuAFQAcgBhAG4AcwBmAGUAcgByAGUAZABUAG8AUwB0AGEAZwBlADIATQBNAFMAXABuAE4AaQB0AHIAbwBnAGUAbgAgAHQAcgBhAG4AcwBmAGUAcgByAGUAZAAgAHQAbwAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMgAgAE0ATQBTAFwAbgBOAFQAXwBqAG0AVAAyAFwAbgBrAGcAIABOAFwAbgBOAFQAXwB7AGoAbQAsAFQAPQAyAH0APQBNAE4AXwB7AGoAbQAsAFQAPQAxAH0AXABcAHQAaQBtAGUAcwAoADEALQBGAHIAYQBjAEcAQQBTAE0AXwB7AG0ALABUAD0AMQB9AC0ARQBGAF8AewBtACwAVAA9ADEAfQApAFwAbgBNAE4AXwBqAG0AVAAxACAAPQAgAG4AaQB0AHIAbwBnAGUAbgAgAHAAZQByACAAcwB3AGkAbgBlACAAYwBsAGEAcwBzACAAaQBuACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAAxACAATQBNAFMAIAAoAGsAZwAgAE4AKQBcAG4ARgByAGEAYwBHAEEAUwBNAG0AVAAxACAAPQAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB2AG8AbABhAHQAaQBsAGkAcwBlAGQAIABmAHIAbwBtACAATQBNAFMAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGEAdAAgAHMAdABhAGcAZQAgADEAXABuAEUARgBfAG0AVAAxACAAPQAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAATQBNAFMAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGEAdAAgAHMAdABhAGcAZQAgADEAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8ANwBfAE4AaQB0AHIAbwBnAGUAbgBUAHIAYQBuAHMAZgBlAHIAcgBlAGQAVABvAFMAdABhAGcAZQAyAE0ATQBTAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0ATgBfAGoAbQBUADEALAAgAEYAcgBhAGMARwBBAFMATQBtAFQAMQAsACAARQBGAF8AbQBUADEALABcAG4AIAAgACAAIABNAE4AXwBqAG0AVAAxACAAKgAgACgAMQAgAC0AIABGAHIAYQBjAEcAQQBTAE0AbQBUADEAIAAtACAARQBGAF8AbQBUADEAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADcAXwBOAGkAdAByAG8AZwBlAG4AVAByAGEAbgBzAGYAZQByAHIAZQBkAFQAbwBTAHQAYQBnAGUAMgBNAE0AUwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBpAHQAcgBvAGcAZQBuACAAdAByAGEAbgBzAGYAZQByAHIAZQBkACAAdABvACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAAyACAATQBNAFMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADcAXwBOAGkAdAByAG8AZwBlAG4AVAByAGEAbgBzAGYAZQByAHIAZQBkAFQAbwBTAHQAYQBnAGUAMgBNAE0AUwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBUAF8AagBtAFQAMgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8ANwBfAE4AaQB0AHIAbwBnAGUAbgBUAHIAYQBuAHMAZgBlAHIAcgBlAGQAVABvAFMAdABhAGcAZQAyAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8ANwBfAE4AaQB0AHIAbwBnAGUAbgBUAHIAYQBuAHMAZgBlAHIAcgBlAGQAVABvAFMAdABhAGcAZQAyAE0ATQBTAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgA1AC4AMQAuADMALAAgAEUAcQB1AGEAdABpAG8AbgAgACgANwApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA3AF8ATgBpAHQAcgBvAGcAZQBuAFQAcgBhAG4AcwBmAGUAcgByAGUAZABUAG8AUwB0AGEAZwBlADIATQBNAFMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADcAXwBOAGkAdAByAG8AZwBlAG4AVAByAGEAbgBzAGYAZQByAHIAZQBkAFQAbwBTAHQAYQBnAGUAMgBNAE0AUwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AVABfAHsAagBtACwAVAA9ADIAfQA9AE0ATgBfAHsAagBtACwAVAA9ADEAfQBcAFwAdABpAG0AZQBzACgAMQAtAEYAcgBhAGMARwBBAFMATQBfAHsAbQAsAFQAPQAxAH0ALQBFAEYAXwB7AG0ALABUAD0AMQB9ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADcAXwBOAGkAdAByAG8AZwBlAG4AVAByAGEAbgBzAGYAZQByAHIAZQBkAFQAbwBTAHQAYQBnAGUAMgBNAE0AUwBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE4AXwBqAG0AVAAxAFwAIgAsACAAXAAiAG4AaQB0AHIAbwBnAGUAbgAgAHAAZQByACAAcwB3AGkAbgBlACAAYwBsAGEAcwBzACAAaQBuACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAAxACAATQBNAFMAXAAiACwAIABcACIAawBnACAATgBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADQALgA1AC4AMQAuADMAIAAoADIAKQAoADYAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBHAEEAUwBNAG0AVAAxAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB2AG8AbABhAHQAaQBsAGkAcwBlAGQAIABmAHIAbwBtACAATQBNAFMAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAGEAdAAgAHMAdABhAGcAZQAgADEAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEwAbwBvAGsAdQBwAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEYAXwBtAFQAMQBcACIALAAgAFwAIgBuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAE0ATQBTACAAdAByAGUAYQB0AG0AZQBuAHQAIABhAHQAIABzAHQAYQBnAGUAIAAxAFwAIgAsACAAXAAiAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AXAAiACwAIABcACIATABvAG8AawB1AHAAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8ATQBNAFMAXwBTAHcAaQBuAGUAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA0AC4ANQA6ACAAUwB3AGkAbgBlAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA0AC4ANQAuADEALgA1ACAATQBlAHQAaABvAGQAIAAxACAALQAgAE0AYQBuAHUAcgBlACAAQQB0AG0AbwBzAHAAaABlAHIAaQBjACAARABlAHAAbwBzAGkAdABpAG8AbgAgAFMAdwBpAG4AZQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADUAXwBfADEAXwBBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAE0ATQBTAFwAbgBBAG4AbgB1AGEAbAAgAGEAdABtAG8AcwBwAGgAZQByAGkAYwAgAGQAZQBwAG8AcwBpAHQAaQBvAG4AIABlAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABNAE0AUwBcAG4ARQBfAE4AMgBPAE0ATQBTAGEAZABcAG4AdAAgAE4AMgBPAFwAbgBFAF8AewBOADIATwAsAGEAZAB9AD0ATQBNAFMAXwB7AEEAVABNAE8AUwB9AFwAXAB0AGkAbQBlAHMAIABFAEYAXwB7AE4AMgBPAH0AXABcAHQAaQBtAGUAcwAgAEMAXwB7AE4AMgBPAH0AXABcAHQAaQBtAGUAcwAgADEAMABeAHsALQAzAH0AXABuAE0ATQBTAF8AQQBUAE0ATwBTACAAPQAgAG0AYQBzAHMAIABvAGYAIABOACAAdgBvAGwAYQB0AGkAbABpAHMAZQBkACAAZgByAG8AbQAgAE0ATQBTACAAKABrAGcAIABOACkAXABuAEUARgBfAE4AMgBPACAAPQAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAYQB0AG0AbwBzAHAAaABlAHIAaQBjACAAZABlAHAAbwBzAGkAdABpAG8AbgAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApAFwAbgBDAF8ATgAyAE8AIAA9ACAAZgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAATgAyAE8AIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANQBfAF8AMQBfAEEAbgBuAHUAYQBsAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0ATQBNAFMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBNAFMAXwBBAFQATQBPAFMALAAgAEUARgBfAE4AMgBPACwAIABDAF8ATgAyAE8ALABcAG4AIAAgACAAIABNAE0AUwBfAEEAVABNAE8AUwAgACoAIABFAEYAXwBOADIATwAgACoAIABDAF8ATgAyAE8AIAAqACAAMQAwACAAXgAgAC0AMwBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADUAXwBfADEAXwBBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAE0ATQBTAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAG4AbgB1AGEAbAAgAGEAdABtAG8AcwBwAGgAZQByAGkAYwAgAGQAZQBwAG8AcwBpAHQAaQBvAG4AIABlAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABNAE0AUwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANQBfAF8AMQBfAEEAbgBuAHUAYQBsAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0ATQBNAFMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwBOADIATwBNAE0AUwBhAGQAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADUAXwBfADEAXwBBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAE4AMgBPAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA1AF8AXwAxAF8AQQBuAG4AdQBhAGwAQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBNAE0AUwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4ANQAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADEAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANQBfAF8AMQBfAEEAbgBuAHUAYQBsAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0ATQBNAFMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADUAXwBfADEAXwBBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAE0ATQBTAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAHsATgAyAE8ALABhAGQAfQA9AE0ATQBTAF8AewBBAFQATQBPAFMAfQBcAFwAdABpAG0AZQBzACAARQBGAF8AewBOADIATwB9AFwAXAB0AGkAbQBlAHMAIABDAF8AewBOADIATwB9AFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA1AF8AXwAxAF8AQQBuAG4AdQBhAGwAQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBNAE0AUwBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE0AUwBfAEEAVABNAE8AUwBcACIALAAgAFwAIgBtAGEAcwBzACAAbwBmACAATgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGYAcgBvAG0AIABNAE0AUwBcACIALAAgAFwAIgBrAGcAIABOAFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAANAAuADUALgAxAC4ANQAgACgAMgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEYAXwBOADIATwBcACIALAAgAFwAIgBuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGEAdABtAG8AcwBwAGgAZQByAGkAYwAgAGQAZQBwAG8AcwBpAHQAaQBvAG4AXAAiACwAIABcACIAawBnACAATgAyAE8ALQBOAC8AawBnACAATgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAXwBOADIATwBcACIALAAgAFwAIgBmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIALAAgAFwAIgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAGoAXAAiACwAIABcACIAcAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAaQByAFwAIgAsACAAXAAiAGkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAHIAXAAiACwAIABcACIAcgBhAGkAbgBmAGEAbABsACAAcgBlAGcAaQBvAG4AXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADUAXwBfADIAXwBUAG8AdABhAGwATgBpAHQAcgBvAGcAZQBuAFYAbwBsAGEAdABpAGwAaQBzAGUAZABGAHIAbwBtAE0ATQBTAFwAbgBUAG8AdABhAGwAIABuAGkAdAByAG8AZwBlAG4AIAB2AG8AbABhAHQAaQBsAGkAcwBlAGQAIABmAHIAbwBtACAATQBNAFMAXABuAE0ATQBTAF8AQQBUAE0ATwBTAFwAbgBrAGcAIABOAFwAbgBNAE0AUwBfAHsAQQBUAE0ATwBTAH0APQBcAFwAcwB1AG0AXwB7AGoAfQBcAFwAcwB1AG0AXwB7AG0AfQBcAFwAcwB1AG0AXwB7AFQAfQAoAE0ATgBfAHsAagBtAFQAfQBcAFwAdABpAG0AZQBzACAARgByAGEAYwBHAEEAUwBNAF8AewBtAFQAfQApAFwAbgBNAE4AXwBqAG0AVAAgAD0AIABuAGkAdAByAG8AZwBlAG4AIABwAGUAcgAgAHMAdwBpAG4AZQAgAGMAbABhAHMAcwAsACAATQBNAFMAIABhAG4AZAAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAKABrAGcAIABOACkAXABuAEYAcgBhAGMARwBBAFMATQBtAFQAIAA9ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGkAbgAgAGUAYQBjAGgAIABNAE0AUwAgACgAKABrAGcAIABOAEgAMwAtAE4AIAArACAATgBPAHgALQBOACkALwBrAGcAIABOACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANQBfAF8AMgBfAFQAbwB0AGEAbABOAGkAdAByAG8AZwBlAG4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAEYAcgBvAG0ATQBNAFMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBOAF8AagBtAFQALAAgAEYAcgBhAGMARwBBAFMATQBtAFQALABcAG4AIAAgACAAIABNAE4AXwBqAG0AVAAgACoAIABGAHIAYQBjAEcAQQBTAE0AbQBUAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANQBfAF8AMgBfAFQAbwB0AGEAbABOAGkAdAByAG8AZwBlAG4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAEYAcgBvAG0ATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAbwB0AGEAbAAgAG4AaQB0AHIAbwBnAGUAbgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGYAcgBvAG0AIABNAE0AUwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANQBfAF8AMgBfAFQAbwB0AGEAbABOAGkAdAByAG8AZwBlAG4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAEYAcgBvAG0ATQBNAFMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0ATQBTAF8AQQBUAE0ATwBTAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA1AF8AXwAyAF8AVABvAHQAYQBsAE4AaQB0AHIAbwBnAGUAbgBWAG8AbABhAHQAaQBsAGkAcwBlAGQARgByAG8AbQBNAE0AUwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADUAXwBfADIAXwBUAG8AdABhAGwATgBpAHQAcgBvAGcAZQBuAFYAbwBsAGEAdABpAGwAaQBzAGUAZABGAHIAbwBtAE0ATQBTAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgA1AC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMgApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA1AF8AXwAyAF8AVABvAHQAYQBsAE4AaQB0AHIAbwBnAGUAbgBWAG8AbABhAHQAaQBsAGkAcwBlAGQARgByAG8AbQBNAE0AUwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANQBfAF8AMgBfAFQAbwB0AGEAbABOAGkAdAByAG8AZwBlAG4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAEYAcgBvAG0ATQBNAFMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE0AUwBfAHsAQQBUAE0ATwBTAH0APQBcAFwAcwB1AG0AXwB7AGoAfQBcAFwAcwB1AG0AXwB7AG0AfQBcAFwAcwB1AG0AXwB7AFQAfQAoAE0ATgBfAHsAagBtAFQAfQBcAFwAdABpAG0AZQBzACAARgByAGEAYwBHAEEAUwBNAF8AewBtAFQAfQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA1AF8AXwAyAF8AVABvAHQAYQBsAE4AaQB0AHIAbwBnAGUAbgBWAG8AbABhAHQAaQBsAGkAcwBlAGQARgByAG8AbQBNAE0AUwBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE4AXwBqAG0AVABcACIALAAgAFwAIgBuAGkAdAByAG8AZwBlAG4AIABwAGUAcgAgAHMAdwBpAG4AZQAgAGMAbABhAHMAcwAsACAATQBNAFMAIABhAG4AZAAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlAFwAIgAsACAAXAAiAGsAZwAgAE4AXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAA0AC4ANQAuADEALgAzACAAKAAyACkAKAA2ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAcgBhAGMARwBBAFMATQBtAFQAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGkAbgAgAGUAYQBjAGgAIABNAE0AUwBcACIALAAgAFwAIgAoAGsAZwAgAE4ASAAzAC0ATgAgACsAIABOAE8AeAAtAE4AKQAvAGsAZwAgAE4AXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAE0ATQBTAF8AUwB3AGkAbgBlAF8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADQALgA1ADoAIABTAHcAaQBuAGUAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADQALgA1AC4AMQAuADcAIABNAGUAdABoAG8AZAAgADEAIAAtACAATQBhAG4AdQByAGUAIABMAGUAYQBjAGgAaQBuAGcAIABBAG4AZAAgAFIAdQBuAG8AZgBmACAATgAyAE8AIABTAHcAaQBuAGUAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA3AF8AXwAxAF8AQQBuAG4AdQBhAGwARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARgByAG8AbQBNAE0AUwBcAG4AQQBuAG4AdQBhAGwAIABlAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmACAAZgByAG8AbQAgAGUAYQBjAGgAIABNAE0AUwBcAG4ARQBfAE4AMgBPAGwAZQBhAGMAaABcAG4AdAAgAE4AMgBPAFwAbgBFAF8AewBOADIATwAsAGwAZQBhAGMAaAB9AD0ATQBOAEwAZQBhAGMAaABfAHsAagBtAD0ANQB9AFwAXAB0AGkAbQBlAHMAIABFAEYAXwB7AGwAZQBhAGMAaAB9AFwAXAB0AGkAbQBlAHMAIABDAF8AewBOADIATwB9AFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9AFwAbgBNAE4ATABlAGEAYwBoAF8AagBtADUAIAA9ACAAbQBhAHMAcwAgAG8AZgAgAE4AIABsAG8AcwB0ACAAdABoAHIAbwB1AGcAaAAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIABmAHIAbwBtACAAZAByAHkAbABvAHQAIABNAE0AUwAgACgAawBnACAATgApAFwAbgBFAEYAXwBsAGUAYQBjAGgAIAA9ACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQBcAG4AQwBfAE4AMgBPACAAPQAgAGYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFADoAIABEAHUAZQAgAHQAbwAgAHMAdAByAGkAYwB0ACAAZQBuAHYAaQByAG8AbgBtAGUAbgB0AGEAbAAgAGMAbwBuAHQAcgBvAGwAcwAsACAAZQBtAGkAcwBzAGkAbwBuAHMAIABhAHIAZQAgAGUAcwB0AGkAbQBhAHQAZQBkACAAbwBuAGwAeQAgAGYAbwByACAAZAByAHkAbABvAHQAIABNAE0AUwAgACgAbQA9ADUAKQAuAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADcAXwBfADEAXwBBAG4AbgB1AGEAbABFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBGAHIAbwBtAE0ATQBTAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0ATgBMAGUAYQBjAGgAXwBqAG0ANQAsACAARQBGAF8AbABlAGEAYwBoACwAIABDAF8ATgAyAE8ALABcAG4AIAAgACAAIABNAE4ATABlAGEAYwBoAF8AagBtADUAIAAqACAARQBGAF8AbABlAGEAYwBoACAAKgAgAEMAXwBOADIATwAgACoAIAAxADAAIABeACAALQAzAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANwBfAF8AMQBfAEEAbgBuAHUAYQBsAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEYAcgBvAG0ATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAbgBuAHUAYQBsACAAZQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgAgAGYAcgBvAG0AIABlAGEAYwBoACAATQBNAFMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADcAXwBfADEAXwBBAG4AbgB1AGEAbABFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBGAHIAbwBtAE0ATQBTAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8ATgAyAE8AbABlAGEAYwBoAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA3AF8AXwAxAF8AQQBuAG4AdQBhAGwARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARgByAG8AbQBNAE0AUwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABOADIATwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANwBfAF8AMQBfAEEAbgBuAHUAYQBsAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEYAcgBvAG0ATQBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADUALgAxAC4ANwAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAxACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADcAXwBfADEAXwBBAG4AbgB1AGEAbABFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBGAHIAbwBtAE0ATQBTAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA3AF8AXwAxAF8AQQBuAG4AdQBhAGwARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARgByAG8AbQBNAE0AUwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwB7AE4AMgBPACwAbABlAGEAYwBoAH0APQBNAE4ATABlAGEAYwBoAF8AewBqAG0APQA1AH0AXABcAHQAaQBtAGUAcwAgAEUARgBfAHsAbABlAGEAYwBoAH0AXABcAHQAaQBtAGUAcwAgAEMAXwB7AE4AMgBPAH0AXABcAHQAaQBtAGUAcwAgADEAMABeAHsALQAzAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADcAXwBfADEAXwBBAG4AbgB1AGEAbABFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBGAHIAbwBtAE0ATQBTAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0ATgBMAGUAYQBjAGgAXwBqAG0ANQBcACIALAAgAFwAIgBtAGEAcwBzACAAbwBmACAATgAgAGwAbwBzAHQAIAB0AGgAcgBvAHUAZwBoACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgAgAGYAcgBvAG0AIABkAHIAeQBsAG8AdAAgAE0ATQBTAFwAIgAsACAAXAAiAGsAZwAgAE4AXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAA0AC4ANQAuADEALgA3ACAAKAAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBfAGwAZQBhAGMAaABcACIALAAgAFwAIgBlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIALAAgAFwAIgBrAGcAIABOADIATwAtAE4ALwBrAGcAIABOAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBfAE4AMgBPAFwAIgAsACAAXAAiAGYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA3AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABvAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBGAHIAbwBtAEQAcgB5AGwAbwB0AE0ATQBTAFwAbgBNAGEAcwBzACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAbABvAHMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIABmAHIAbwBtACAAZAByAHkAbABvAHQAIABNAE0AUwBcAG4ATQBOAEwAZQBhAGMAaABfAGoAbQA1AFwAbgBrAGcAIABOAFwAbgBNAE4ATABlAGEAYwBoAF8AewBqAG0APQA1AH0APQBNAE4AXwB7AGoAbQA9ADUALABUAD0AMQB9AFwAXAB0AGkAbQBlAHMAIABGAHIAYQBjAFcARQBUAFwAXAB0AGkAbQBlAHMAIABGAHIAYQBjAEwARQBBAEMASABfAHsATQBTAH0AXABuAE0ATgBfAGoAbQA1AFQAMQAgAD0AIABuAGkAdAByAG8AZwBlAG4AIABpAG4AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADEAIABkAHIAeQBsAG8AdAAgAE0ATQBTACAAKABrAGcAIABOACkAXABuAEYAcgBhAGMAVwBFAFQAIAA9ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgBGAHIAYQBjAEwARQBBAEMASABfAE0AUwAgAD0AIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAbABvAHMAdAAgAHQAaAByAG8AdQBnAGgAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADcAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAG8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEYAcgBvAG0ARAByAHkAbABvAHQATQBNAFMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBOAF8AagBtADUAVAAxACwAIABGAHIAYQBjAFcARQBUACwAIABGAHIAYQBjAEwARQBBAEMASABfAE0AUwAsAFwAbgAgACAAIAAgAE0ATgBfAGoAbQA1AFQAMQAgACoAIABGAHIAYQBjAFcARQBUACAAKgAgAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANwBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAbwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARgByAG8AbQBEAHIAeQBsAG8AdABNAE0AUwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBhAHMAcwAgAG8AZgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAbwBzAHQAIAB0AG8AIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmACAAZgByAG8AbQAgAGQAcgB5AGwAbwB0ACAATQBNAFMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADcAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAG8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEYAcgBvAG0ARAByAHkAbABvAHQATQBNAFMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0ATgBMAGUAYQBjAGgAXwBqAG0ANQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANwBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAbwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARgByAG8AbQBEAHIAeQBsAG8AdABNAE0AUwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADcAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAG8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEYAcgBvAG0ARAByAHkAbABvAHQATQBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADUALgAxAC4ANwAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAyACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADcAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAG8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEYAcgBvAG0ARAByAHkAbABvAHQATQBNAFMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADcAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAG8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEYAcgBvAG0ARAByAHkAbABvAHQATQBNAFMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE4ATABlAGEAYwBoAF8AewBqAG0APQA1AH0APQBNAE4AXwB7AGoAbQA9ADUALABUAD0AMQB9AFwAXAB0AGkAbQBlAHMAIABGAHIAYQBjAFcARQBUAFwAXAB0AGkAbQBlAHMAIABGAHIAYQBjAEwARQBBAEMASABfAHsATQBTAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADcAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAG8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEYAcgBvAG0ARAByAHkAbABvAHQATQBNAFMAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBOAF8AagBtADUAVAAxAFwAIgAsACAAXAAiAG4AaQB0AHIAbwBnAGUAbgAgAGkAbgAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMQAgAGQAcgB5AGwAbwB0ACAATQBNAFMAXAAiACwAIABcACIAawBnACAATgBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADQALgA1AC4AMQAuADMAIAAoADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBXAEUAVABcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAGwAbwBzAHQAIAB0AGgAcgBvAHUAZwBoACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgB6AFwAIgAsACAAXAAiAGwAbwBjAGEAdABpAG8AbgAgAGkAbgAgAGwAZQBhAGMAaABpAG4AZwAgAHoAbwBuAGUAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBqAFwAIgAsACAAXAAiAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAGkAcgBcACIALAAgAFwAIgBpAHIAcgBpAGcAYQB0AGkAbwBuACAAbQBlAHQAaABvAGQAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBhAG4AdQByAGUAQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADQALgA1ADoAIABTAHcAaQBuAGUAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADQALgA1AC4AMQAuADkAIABNAGEAbgB1AHIAZQAgAEEAcABwAGwAaQBlAGQAIAB0AG8AIABTAG8AaQBsAHMAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA5AF8AXwAxAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMQBcAG4ATQBhAHMAcwAgAG8AZgAgAG4AaQB0AHIAbwBnAGUAbgAgAGEAcABwAGwAaQBlAGQAIAB0AG8AIABzAG8AaQBsAHMAIABmAG8AcgAgAHMAYwBvAHAAZQAgADEAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ATQBOAFMAbwBpAGwAXwBzAGMAbwBwAGUAMQBcAG4AawBnACAATgBcAG4ATQBOAFMAbwBpAGwAXwB7AHMAYwBvAHAAZQAxAH0APQBcAFwAcwB1AG0AXwB7AGoAfQBcAFwAcwB1AG0AXwB7AG0AfQAoAE0ATgBfAHsAagBtAFQAPQAyAH0AXABcAHQAaQBtAGUAcwAoADEALQBFAEYAXwB7AG0AVAA9ADIAfQAtAEYAcgBhAGMARwBBAFMATQBfAHsAbQBUAD0AMgB9ACkALQBNAE4ATABlAGEAYwBoAF8AewBqAG0APQA1AH0AKQBcAFwAdABpAG0AZQBzACAAUABGAFwAbgBNAE4AXwBqAG0AVAAyACAAPQAgAG0AYQBzAHMAIABvAGYAIABOACAAaQBuACAATQBNAFMAIABhAHQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADIAIAA6ACAAawBnACAATgBcAG4ARQBGAF8AbQBUADIAIAA9ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABlAGEAYwBoACAATQBNAFMAIABhAHQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADIAIAA6ACAAawBnACAATgAyAE8ALQBOAC8AawBnACAATgBcAG4ARgByAGEAYwBHAEEAUwBNAF8AbQBUADIAIAA9ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAYQBuAGkAbQBhAGwAIAB3AGEAcwB0AGUAIABOACAAdgBvAGwAYQB0AGkAbABpAHMAZQBkACAAaQBuACAAZQBhAGMAaAAgAE0ATQBTACAAYQB0ACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAAyACAAOgAgACgAawBnACAATgBIADMALQBOACAAKwAgAE4ATwB4AC0ATgApAC8AawBnACAATgBcAG4ATQBOAEwAZQBhAGMAaABfAGoAbQA1ACAAPQAgAG0AYQBzAHMAIABvAGYAIABOACAAbABvAHMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIABmAHIAbwBtACAAZAByAHkAbABvAHQAIABNAE0AUwAgADoAIABrAGcAIABOAFwAbgBQAEYAIAA9ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAbQBhAG4AdQByAGUAIABhAHAAcABsAGkAZQBkACAAdABvACAAcwBvAGkAbAAgAHcAaQB0AGgAaQBuACAAdABoAGUAIABwAGkAZwBnAGUAcgB5ACAAYgBvAHUAbgBkAGEAcgB5ACAAOgAgAGYAcgBhAGMAdABpAG8AbgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA5AF8AXwAxAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAE4AXwBqAG0AVAAyACwAIABFAEYAXwBtAFQAMgAsACAARgByAGEAYwBHAEEAUwBNAF8AbQBUADIALAAgAE0ATgBMAGUAYQBjAGgAXwBqAG0ANQAsACAAUABGACwAXABuACAAIAAgACAAKABNAE4AXwBqAG0AVAAyACAAKgAgACgAMQAgAC0AIABFAEYAXwBtAFQAMgAgAC0AIABGAHIAYQBjAEcAQQBTAE0AXwBtAFQAMgApACAALQAgAE0ATgBMAGUAYQBjAGgAXwBqAG0ANQApACAAKgAgAFAARgBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADkAXwBfADEAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAxAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAcwBzACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAYQBwAHAAbABpAGUAZAAgAHQAbwAgAHMAbwBpAGwAcwAgAGYAbwByACAAcwBjAG8AcABlACAAMQAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA5AF8AXwAxAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMQBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBOAFMAbwBpAGwAXwBzAGMAbwBwAGUAMQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AOQBfAF8AMQBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADEAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA5AF8AXwAxAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4ANQAuADEALgA5ACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADEAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AOQBfAF8AMQBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADEAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADkAXwBfADEAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAxAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBOAFMAbwBpAGwAXwB7AHMAYwBvAHAAZQAxAH0APQBcAFwAcwB1AG0AXwB7AGoAfQBcAFwAcwB1AG0AXwB7AG0AfQAoAE0ATgBfAHsAagBtAFQAPQAyAH0AXABcAHQAaQBtAGUAcwAoADEALQBFAEYAXwB7AG0AVAA9ADIAfQAtAEYAcgBhAGMARwBBAFMATQBfAHsAbQBUAD0AMgB9ACkALQBNAE4ATABlAGEAYwBoAF8AewBqAG0APQA1AH0AKQBcAFwAdABpAG0AZQBzACAAUABGAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA5AF8AXwAxAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE4AXwBqAG0AVAAyAFwAIgAsAFwAIgBtAGEAcwBzACAAbwBmACAATgAgAGkAbgAgAE0ATQBTACAAYQB0ACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAAyAFwAIgAsACAAXAAiAGsAZwAgAE4AXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAA0AC4ANQAuADEALgAzACAAKAA2ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBfAG0AVAAyAFwAIgAsAFwAIgBuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGUAYQBjAGgAIABNAE0AUwAgAGEAdAAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMgBcACIALAAgAFwAIgBrAGcAIABOADIATwAtAE4ALwBrAGcAIABOAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBHAEEAUwBNAF8AbQBUADIAXAAiACwAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAGEAbgBpAG0AYQBsACAAdwBhAHMAdABlACAATgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGkAbgAgAGUAYQBjAGgAIABNAE0AUwAgAGEAdAAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMgBcACIALAAgAFwAIgAoAGsAZwAgAE4ASAAzAC0ATgAgACsAIABOAE8AeAAtAE4AKQAvAGsAZwAgAE4AXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE4ATABlAGEAYwBoAF8AagBtADUAXAAiACwAXAAiAG0AYQBzAHMAIABvAGYAIABOACAAbABvAHMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIABmAHIAbwBtACAAZAByAHkAbABvAHQAIABNAE0AUwBcACIALAAgAFwAIgBrAGcAIABOAFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAANAAuADUALgAxAC4ANwAgACgAMgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEYAXAAiACwAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG0AYQBuAHUAcgBlACAAYQBwAHAAbABpAGUAZAAgAHQAbwAgAHMAbwBpAGwAIAB3AGkAdABoAGkAbgAgAHQAaABlACAAcABpAGcAZwBlAHIAeQAgAGIAbwB1AG4AZABhAHIAeQBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADkAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAzAFwAbgBNAGEAcwBzACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAYQBwAHAAbABpAGUAZAAgAHQAbwAgAHMAbwBpAGwAcwAgAGYAbwByACAAcwBjAG8AcABlACAAMwAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBNAE4AUwBvAGkAbABfAHMAYwBvAHAAZQAzAFwAbgBrAGcAIABOAFwAbgBNAE4AUwBvAGkAbABfAHsAcwBjAG8AcABlADMAfQA9AFwAXABzAHUAbQBfAHsAagB9AFwAXABzAHUAbQBfAHsAbQB9ACgATQBOAF8AewBqAG0AVAA9ADIAfQBcAFwAdABpAG0AZQBzACgAMQAtAEUARgBfAHsAbQBUAD0AMgB9AC0ARgByAGEAYwBHAEEAUwBNAF8AewBtAFQAPQAyAH0AKQAtAE0ATgBMAGUAYQBjAGgAXwB7AGoAbQA9ADUAfQApAFwAXAB0AGkAbQBlAHMAKAAxAC0AUABGACkAXABuAE0ATgBfAGoAbQBUADIAIAA9ACAAbQBhAHMAcwAgAG8AZgAgAE4AIABpAG4AIABNAE0AUwAgAGEAdAAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMgAgADoAIABrAGcAIABOAFwAbgBFAEYAXwBtAFQAMgAgAD0AIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGUAYQBjAGgAIABNAE0AUwAgAGEAdAAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMgAgADoAIABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOAFwAbgBGAHIAYQBjAEcAQQBTAE0AXwBtAFQAMgAgAD0AIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABhAG4AaQBtAGEAbAAgAHcAYQBzAHQAZQAgAE4AIAB2AG8AbABhAHQAaQBsAGkAcwBlAGQAIABpAG4AIABlAGEAYwBoACAATQBNAFMAIABhAHQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADIAIAA6ACAAKABrAGcAIABOAEgAMwAtAE4AIAArACAATgBPAHgALQBOACkALwBrAGcAIABOAFwAbgBNAE4ATABlAGEAYwBoAF8AagBtADUAIAA9ACAAbQBhAHMAcwAgAG8AZgAgAE4AIABsAG8AcwB0ACAAdABvACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgAgAGYAcgBvAG0AIABkAHIAeQBsAG8AdAAgAE0ATQBTACAAOgAgAGsAZwAgAE4AXABuAFAARgAgAD0AIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABtAGEAbgB1AHIAZQAgAGEAcABwAGwAaQBlAGQAIAB0AG8AIABzAG8AaQBsACAAdwBpAHQAaABpAG4AIAB0AGgAZQAgAHAAaQBnAGcAZQByAHkAIABiAG8AdQBuAGQAYQByAHkAIAA6ACAAZgByAGEAYwB0AGkAbwBuAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADkAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0ATgBfAGoAbQBUADIALAAgAEUARgBfAG0AVAAyACwAIABGAHIAYQBjAEcAQQBTAE0AXwBtAFQAMgAsACAATQBOAEwAZQBhAGMAaABfAGoAbQA1ACwAIABQAEYALABcAG4AIAAgACAAIAAoAE0ATgBfAGoAbQBUADIAIAAqACAAKAAxACAALQAgAEUARgBfAG0AVAAyACAALQAgAEYAcgBhAGMARwBBAFMATQBfAG0AVAAyACkAIAAtACAATQBOAEwAZQBhAGMAaABfAGoAbQA1ACkAIAAqACAAKAAxACAALQAgAFAARgApAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AOQBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AYQBzAHMAIABvAGYAIABuAGkAdAByAG8AZwBlAG4AIABhAHAAcABsAGkAZQBkACAAdABvACAAcwBvAGkAbABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADkAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE4AUwBvAGkAbABfAHMAYwBvAHAAZQAzAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA5AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADkAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgA1AC4AMQAuADkALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMgApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA5AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AOQBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE4AUwBvAGkAbABfAHsAcwBjAG8AcABlADMAfQA9AFwAXABzAHUAbQBfAHsAagB9AFwAXABzAHUAbQBfAHsAbQB9ACgATQBOAF8AewBqAG0AVAA9ADIAfQBcAFwAdABpAG0AZQBzACgAMQAtAEUARgBfAHsAbQBUAD0AMgB9AC0ARgByAGEAYwBHAEEAUwBNAF8AewBtAFQAPQAyAH0AKQAtAE0ATgBMAGUAYQBjAGgAXwB7AGoAbQA9ADUAfQApAFwAXAB0AGkAbQBlAHMAKAAxAC0AUABGACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADkAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAzAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA1ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0ATgBfAGoAbQBUADIAXAAiACwAXAAiAG0AYQBzAHMAIABvAGYAIABOACAAaQBuACAATQBNAFMAIABhAHQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADIAXAAiACwAIABcACIAawBnACAATgBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADQALgA1AC4AMQAuADMAIAAoADYAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAF8AbQBUADIAXAAiACwAXAAiAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAZQBhAGMAaAAgAE0ATQBTACAAYQB0ACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAAyAFwAIgAsACAAXAAiAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAHIAYQBjAEcAQQBTAE0AXwBtAFQAMgBcACIALABcACIAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAYQBuAGkAbQBhAGwAIAB3AGEAcwB0AGUAIABOACAAdgBvAGwAYQB0AGkAbABpAHMAZQBkACAAaQBuACAAZQBhAGMAaAAgAE0ATQBTACAAYQB0ACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAAyAFwAIgAsACAAXAAiACgAawBnACAATgBIADMALQBOACAAKwAgAE4ATwB4AC0ATgApAC8AawBnACAATgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0ATgBMAGUAYQBjAGgAXwBqAG0ANQBcACIALABcACIAbQBhAHMAcwAgAG8AZgAgAE4AIABsAG8AcwB0ACAAdABvACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgAgAGYAcgBvAG0AIABkAHIAeQBsAG8AdAAgAE0ATQBTAFwAIgAsACAAXAAiAGsAZwAgAE4AXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAA0AC4ANQAuADEALgA3ACAAKAAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAARgBcACIALABcACIAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAbQBhAG4AdQByAGUAIABhAHAAcABsAGkAZQBkACAAdABvACAAcwBvAGkAbAAgAHcAaQB0AGgAaQBuACAAdABoAGUAIABwAGkAZwBnAGUAcgB5ACAAYgBvAHUAbgBkAGEAcgB5AFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuACIAfQBdACwAIgBwAHIAbwBqAGUAYwB0AE4AYQBtAGUAcwAiADoAWwAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBWAGEAaQByAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAUgBvAHcAUwB0AGEAcgB0AE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAHIAYQB5AEkAbgBUAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAVAB3AG8AQwBvAGwAdQBtAG4AcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBPAG4AZQBDAG8AbAB1AG0AbgBBAG4AZABIAGUAYQBkAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHAAbABpAHQAUwB0AHIAaQBuAGcASQBuAHQAbwBBAHIAcgBhAHkAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAEkAdABlAG0ARgByAG8AbQBNAGkAbgBNAGEAeAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAHUAbQBRAHUAYQBuAHQAaQB0AHkARgByAG8AbQBDAHIAaQB0AGUAcgBpAGEAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAE4AMgBPAEUARgBGAHIAbwBtAFAAcgBvAGQASQByAHIAaQBnAGEAdABpAG8AbgBSAGEAaQBuAGYAYQBsAGwAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAGcAdQBtAGUAbgB0AHMAXwAxAF8AMgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMwBfADQAIgAsACIAQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ARwBlAHQARgByAGEAYwBXAEUAVAAiACwAIgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBIAGEAcgB2AGUAcwB0AEkAbgBkAGUAeAAiACwAIgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBSAGUAcwBpAGQAdQBlAEMAcgBvAHAAUgBhAHQAaQBvACIALAAiAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEMAYQBsAGMAdQBsAGEAdABlAEYAcgBhAGMAdABpAG8AbgBSAGUAcwBpAGQAdQBlAFIAZQBtAG8AdgBlAGQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUALgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBGAGUAZQBkAEkAbgB0AGEAawBlAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUALgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ARgBlAGUAZABJAG4AdABhAGsAZQBfAFUAbgBpAHQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBGAGUAZQBkAEkAbgB0AGEAawBlAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBGAGUAZQBkAEkAbgB0AGEAawBlAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBGAGUAZQBkAEkAbgB0AGEAawBlAF8ARABhAHQAYQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE4AaQB0AHIAbwBnAGUAbgBJAG4AVwBhAHMAdABlAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUALgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATgBpAHQAcgBvAGcAZQBuAEkAbgBXAGEAcwB0AGUAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUALgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATgBpAHQAcgBvAGcAZQBuAEkAbgBXAGEAcwB0AGUAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE4AaQB0AHIAbwBnAGUAbgBJAG4AVwBhAHMAdABlAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBOAGkAdAByAG8AZwBlAG4ASQBuAFcAYQBzAHQAZQBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBGAHIAYQBjAHQAaQBvAG4ATgBWAG8AbABhAHQAaQBsAGkAcwBlAGQAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBGAHIAYQBjAHQAaQBvAG4ATgBWAG8AbABhAHQAaQBsAGkAcwBlAGQAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUALgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ARgByAGEAYwB0AGkAbwBuAE4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBGAHIAYQBjAHQAaQBvAG4ATgBWAG8AbABhAHQAaQBsAGkAcwBlAGQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAEYAcgBhAGMAdABpAG8AbgBOAFYAbwBsAGEAdABpAGwAaQBzAGUAZABfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUALgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUALgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUALgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUALgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATQBNAFMAXwBNAEMARgBzAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUALgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATQBNAFMAXwBNAEMARgBzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE0ATQBTAF8ATQBDAEYAcwBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUALgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATQBNAFMAXwBNAEMARgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBNAE0AUwBfAE0AQwBGAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUALgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8AQQB2AGUAcgBhAGcAZQBMAGkAdgBlAHcAZQBpAGcAaAB0AF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUALgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8AQQB2AGUAcgBhAGcAZQBMAGkAdgBlAHcAZQBpAGcAaAB0AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAEEAdgBlAHIAYQBnAGUATABpAHYAZQB3AGUAaQBnAGgAdABfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUALgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8AQQB2AGUAcgBhAGcAZQBMAGkAdgBlAHcAZQBpAGcAaAB0AF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBBAHYAZQByAGEAZwBlAEwAaQB2AGUAdwBlAGkAZwBoAHQAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUALgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8AUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBzAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUALgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8AUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0AcwBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUALgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8AUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUALgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAHIAeQBsAG8AdABNAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARAByAHkAbABvAHQATQBNAFMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBGAHIAYQBjAEwARQBBAEMASABfAEQAcgB5AGwAbwB0AE0ATQBTAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARAByAHkAbABvAHQATQBNAFMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARAByAHkAbABvAHQATQBNAFMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARAByAHkAbABvAHQATQBNAFMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUALgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAF8ATQBlAGcAYQBqAG8AdQBsAGUAcwBQAGUAcgBLAGkAbABvAGcAcgBhAG0ATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE0AZQBnAGEAagBvAHUAbABlAHMAUABlAHIASwBpAGwAbwBnAHIAYQBtAE0AZQB0AGgAYQBuAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBTAHcAaQBuAGUAXwBNAGUAZwBhAGoAbwB1AGwAZQBzAFAAZQByAEsAaQBsAG8AZwByAGEAbQBNAGUAdABoAGEAbgBlAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE0AZQBnAGEAagBvAHUAbABlAHMAUABlAHIASwBpAGwAbwBnAHIAYQBtAE0AZQB0AGgAYQBuAGUAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE0AZQBnAGEAagBvAHUAbABlAHMAUABlAHIASwBpAGwAbwBnAHIAYQBtAE0AZQB0AGgAYQBuAGUAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8AUwB3AGkAbgBlAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAFMAdwBpAG4AZQBfAE0AZQBnAGEAagBvAHUAbABlAHMAUABlAHIASwBpAGwAbwBnAHIAYQBtAE0AZQB0AGgAYQBuAGUAXwBEAGEAdABhACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAFMAdwBpAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADUAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBTAHcAaQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwA1AF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8AUwB3AGkAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8ANQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAFMAdwBpAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADUAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAFUAbgBpAHQAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8AUwB3AGkAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8ANQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8AUwB3AGkAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8ANQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8AUwB3AGkAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8ANQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBTAHcAaQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwA1AF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBTAHcAaQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwA1AF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8AUwB3AGkAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8ANQBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAFMAdwBpAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADUAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBTAHcAaQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwA1AF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAFMAdwBpAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADUAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAFMAdwBpAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADUAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAFMAdwBpAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADUAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8AUwB3AGkAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8ANQBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBUAGkAdABsAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBVAG4AaQB0ACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAF8AUwBvAHUAcgBjAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADIAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUABlAHIAQwBsAGEAcwBzACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMgBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAGUAcgBDAGwAYQBzAHMAVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAyAF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAZQByAEMAbABhAHMAcwBfAFQAaQB0AGwAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADIAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUABlAHIAQwBsAGEAcwBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMgBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAGUAcgBDAGwAYQBzAHMAXwBVAG4AaQB0ACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMgBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAGUAcgBDAGwAYQBzAHMAXwBTAG8AdQByAGMAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADIAXwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AUABlAHIAQwBsAGEAcwBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAyAF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAZQByAEMAbABhAHMAcwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAyAF8ATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFAAZQByAEMAbABhAHMAcwBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMgBfAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBQAGUAcgBDAGwAYQBzAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADMAXwBTAHQAYQBnAGUAMQBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAzAF8AUwB0AGEAZwBlADEATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADMAXwBTAHQAYQBnAGUAMQBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwAzAF8AUwB0AGEAZwBlADEATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA0AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBQAHIAaQBtAGEAcgB5AFMAeQBzAHQAZQBtACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANABfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAUAByAGkAbQBhAHIAeQBTAHkAcwB0AGUAbQBfAFQAaQB0AGwAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADQAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFAAcgBpAG0AYQByAHkAUwB5AHMAdABlAG0AXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA0AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBQAHIAaQBtAGEAcgB5AFMAeQBzAHQAZQBtAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADQAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFAAcgBpAG0AYQByAHkAUwB5AHMAdABlAG0AXwBTAG8AdQByAGMAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADQAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFAAcgBpAG0AYQByAHkAUwB5AHMAdABlAG0AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADQAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFAAcgBpAG0AYQByAHkAUwB5AHMAdABlAG0AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANABfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAUAByAGkAbQBhAHIAeQBTAHkAcwB0AGUAbQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANABfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAUAByAGkAbQBhAHIAeQBTAHkAcwB0AGUAbQBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA1AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADUAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8AVABpAHQAbABlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA1AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAFUAbgBpAHQAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA1AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAFMAbwB1AHIAYwBlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANQBfAEYAcgBhAGMAdABpAG8AbgBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADUAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADUAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADUAXwBGAHIAYQBjAHQAaQBvAG4AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA1AF8ARgByAGEAYwB0AGkAbwBuAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANgBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADYAXwBTAHQAYQBnAGUAMgBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA2AF8AUwB0AGEAZwBlADIATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANgBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFUAbgBpAHQAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA2AF8AUwB0AGEAZwBlADIATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA2AF8AUwB0AGEAZwBlADIATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA2AF8AUwB0AGEAZwBlADIATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADYAXwBTAHQAYQBnAGUAMgBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADYAXwBTAHQAYQBnAGUAMgBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwBfAE0AZQB0AGgAbwBkADIAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA3AF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFQAcgBhAG4AcwBmAGUAcgByAGUAZABTAHQAYQBnAGUAMgAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADcAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVAByAGEAbgBzAGYAZQByAHIAZQBkAFMAdABhAGcAZQAyAF8AVABpAHQAbABlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANwBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBUAHIAYQBuAHMAZgBlAHIAcgBlAGQAUwB0AGEAZwBlADIAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA3AF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFQAcgBhAG4AcwBmAGUAcgByAGUAZABTAHQAYQBnAGUAMgBfAFUAbgBpAHQAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAxAF8AXwA3AF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFQAcgBhAG4AcwBmAGUAcgByAGUAZABTAHQAYQBnAGUAMgBfAFMAbwB1AHIAYwBlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMQBfAF8ANwBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBUAHIAYQBuAHMAZgBlAHIAcgBlAGQAUwB0AGEAZwBlADIAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADcAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVAByAGEAbgBzAGYAZQByAHIAZQBkAFMAdABhAGcAZQAyAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADEAXwBfADcAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAVAByAGEAbgBzAGYAZQByAHIAZQBkAFMAdABhAGcAZQAyAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABEAGkAcgBlAGMAdABOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAE0ATQBTACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwARABpAHIAZQBjAHQATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBNAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0ATQBNAFMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABEAGkAcgBlAGMAdABOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0ATQBNAFMAXwBTAG8AdQByAGMAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0ATQBNAFMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0ATQBNAFMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwARABpAHIAZQBjAHQATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBNAE0AUwBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADIAXwBTAHQAYQBnAGUAMQBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADIAXwBTAHQAYQBnAGUAMQBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAF8AVABpAHQAbABlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADIAXwBTAHQAYQBnAGUAMQBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADIAXwBTAHQAYQBnAGUAMQBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwAyAF8AUwB0AGEAZwBlADEATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADIAXwBTAHQAYQBnAGUAMQBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8AMgBfAFMAdABhAGcAZQAxAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADIAXwBTAHQAYQBnAGUAMQBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8AMwBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEkAbgBQAHIAaQBtAGEAcgB5AE0ATQBTACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADMAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBJAG4AUAByAGkAbQBhAHIAeQBNAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwAzAF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ASQBuAFAAcgBpAG0AYQByAHkATQBNAFMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8AMwBfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEkAbgBQAHIAaQBtAGEAcgB5AE0ATQBTAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwAzAF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ASQBuAFAAcgBpAG0AYQByAHkATQBNAFMAXwBTAG8AdQByAGMAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwAzAF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ASQBuAFAAcgBpAG0AYQByAHkATQBNAFMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwAzAF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ASQBuAFAAcgBpAG0AYQByAHkATQBNAFMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADMAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBJAG4AUAByAGkAbQBhAHIAeQBNAE0AUwBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADQAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBJAG4AUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8ANABfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEkAbgBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA0AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ASQBuAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8AVABpAHQAbABlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADQAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBJAG4AUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8ANABfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEkAbgBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAFUAbgBpAHQAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8ANABfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEkAbgBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAFMAbwB1AHIAYwBlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADQAXwBGAHIAYQBjAHQAaQBvAG4ATwBmAE4AaQB0AHIAbwBnAGUAbgBJAG4AUwBvAGwAaQBkAFMAdABvAHIAYQBnAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA0AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ASQBuAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA0AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ASQBuAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA0AF8ARgByAGEAYwB0AGkAbwBuAE8AZgBOAGkAdAByAG8AZwBlAG4ASQBuAFMAbwBsAGkAZABTAHQAbwByAGEAZwBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8ANABfAEYAcgBhAGMAdABpAG8AbgBPAGYATgBpAHQAcgBvAGcAZQBuAEkAbgBTAG8AbABpAGQAUwB0AG8AcgBhAGcAZQBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADUAXwBBAG4AbgB1AGEAbABOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAaQBvAG4AIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8ANQBfAEEAbgBuAHUAYQBsAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBfAFQAaQB0AGwAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA1AF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADUAXwBBAG4AbgB1AGEAbABOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADUAXwBBAG4AbgB1AGEAbABOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA1AF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8ANQBfAEEAbgBuAHUAYQBsAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8ANQBfAEEAbgBuAHUAYQBsAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADYAXwBTAHQAYQBnAGUAMgBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADYAXwBTAHQAYQBnAGUAMgBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAF8AVABpAHQAbABlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADYAXwBTAHQAYQBnAGUAMgBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADYAXwBTAHQAYQBnAGUAMgBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA2AF8AUwB0AGEAZwBlADIATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADYAXwBTAHQAYQBnAGUAMgBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8ANgBfAFMAdABhAGcAZQAyAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADYAXwBTAHQAYQBnAGUAMgBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8ANwBfAE4AaQB0AHIAbwBnAGUAbgBUAHIAYQBuAHMAZgBlAHIAcgBlAGQAVABvAFMAdABhAGcAZQAyAE0ATQBTACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADcAXwBOAGkAdAByAG8AZwBlAG4AVAByAGEAbgBzAGYAZQByAHIAZQBkAFQAbwBTAHQAYQBnAGUAMgBNAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA3AF8ATgBpAHQAcgBvAGcAZQBuAFQAcgBhAG4AcwBmAGUAcgByAGUAZABUAG8AUwB0AGEAZwBlADIATQBNAFMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AMwBfAF8ANwBfAE4AaQB0AHIAbwBnAGUAbgBUAHIAYQBuAHMAZgBlAHIAcgBlAGQAVABvAFMAdABhAGcAZQAyAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA3AF8ATgBpAHQAcgBvAGcAZQBuAFQAcgBhAG4AcwBmAGUAcgByAGUAZABUAG8AUwB0AGEAZwBlADIATQBNAFMAXwBTAG8AdQByAGMAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA3AF8ATgBpAHQAcgBvAGcAZQBuAFQAcgBhAG4AcwBmAGUAcgByAGUAZABUAG8AUwB0AGEAZwBlADIATQBNAFMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwAzAF8AXwA3AF8ATgBpAHQAcgBvAGcAZQBuAFQAcgBhAG4AcwBmAGUAcgByAGUAZABUAG8AUwB0AGEAZwBlADIATQBNAFMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADMAXwBfADcAXwBOAGkAdAByAG8AZwBlAG4AVAByAGEAbgBzAGYAZQByAHIAZQBkAFQAbwBTAHQAYQBnAGUAMgBNAE0AUwBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADUAXwBfADEAXwBBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAE0ATQBTACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADUAXwBfADEAXwBBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAE0ATQBTAF8AVABpAHQAbABlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADUAXwBfADEAXwBBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAE0ATQBTAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADUAXwBfADEAXwBBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAE0ATQBTAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA1AF8AXwAxAF8AQQBuAG4AdQBhAGwAQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBNAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADUAXwBfADEAXwBBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAE0ATQBTAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANQBfAF8AMQBfAEEAbgBuAHUAYQBsAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0ATQBNAFMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADUAXwBfADEAXwBBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAE0ATQBTAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANQBfAF8AMgBfAFQAbwB0AGEAbABOAGkAdAByAG8AZwBlAG4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAEYAcgBvAG0ATQBNAFMAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANQBfAF8AMgBfAFQAbwB0AGEAbABOAGkAdAByAG8AZwBlAG4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAEYAcgBvAG0ATQBNAFMAXwBUAGkAdABsAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANQBfAF8AMgBfAFQAbwB0AGEAbABOAGkAdAByAG8AZwBlAG4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAEYAcgBvAG0ATQBNAFMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANQBfAF8AMgBfAFQAbwB0AGEAbABOAGkAdAByAG8AZwBlAG4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAEYAcgBvAG0ATQBNAFMAXwBVAG4AaQB0ACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADUAXwBfADIAXwBUAG8AdABhAGwATgBpAHQAcgBvAGcAZQBuAFYAbwBsAGEAdABpAGwAaQBzAGUAZABGAHIAbwBtAE0ATQBTAF8AUwBvAHUAcgBjAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANQBfAF8AMgBfAFQAbwB0AGEAbABOAGkAdAByAG8AZwBlAG4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAEYAcgBvAG0ATQBNAFMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA1AF8AXwAyAF8AVABvAHQAYQBsAE4AaQB0AHIAbwBnAGUAbgBWAG8AbABhAHQAaQBsAGkAcwBlAGQARgByAG8AbQBNAE0AUwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANQBfAF8AMgBfAFQAbwB0AGEAbABOAGkAdAByAG8AZwBlAG4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAEYAcgBvAG0ATQBNAFMAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANwBfAF8AMQBfAEEAbgBuAHUAYQBsAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEYAcgBvAG0ATQBNAFMAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADcAXwBfADEAXwBBAG4AbgB1AGEAbABFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBGAHIAbwBtAE0ATQBTAF8AVABpAHQAbABlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA3AF8AXwAxAF8AQQBuAG4AdQBhAGwARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARgByAG8AbQBNAE0AUwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANwBfAF8AMQBfAEEAbgBuAHUAYQBsAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEYAcgBvAG0ATQBNAFMAXwBVAG4AaQB0ACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA3AF8AXwAxAF8AQQBuAG4AdQBhAGwARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARgByAG8AbQBNAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA3AF8AXwAxAF8AQQBuAG4AdQBhAGwARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARgByAG8AbQBNAE0AUwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA3AF8AXwAxAF8AQQBuAG4AdQBhAGwARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARgByAG8AbQBNAE0AUwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADcAXwBfADEAXwBBAG4AbgB1AGEAbABFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBGAHIAbwBtAE0ATQBTAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADcAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAG8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEYAcgBvAG0ARAByAHkAbABvAHQATQBNAFMAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADcAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAG8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEYAcgBvAG0ARAByAHkAbABvAHQATQBNAFMAXwBUAGkAdABsAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADcAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAG8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEYAcgBvAG0ARAByAHkAbABvAHQATQBNAFMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADcAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAG8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEYAcgBvAG0ARAByAHkAbABvAHQATQBNAFMAXwBVAG4AaQB0ACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA3AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABvAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBGAHIAbwBtAEQAcgB5AGwAbwB0AE0ATQBTAF8AUwBvAHUAcgBjAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADcAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAG8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEYAcgBvAG0ARAByAHkAbABvAHQATQBNAFMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8ANwBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAbwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARgByAG8AbQBEAHIAeQBsAG8AdABNAE0AUwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADcAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAG8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEYAcgBvAG0ARAByAHkAbABvAHQATQBNAFMAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AYQBuAHUAcgBlAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AOQBfAF8AMQBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADEAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGEAbgB1AHIAZQBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADkAXwBfADEAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAxAF8AVABpAHQAbABlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBhAG4AdQByAGUAQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA5AF8AXwAxAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AYQBuAHUAcgBlAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AOQBfAF8AMQBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADEAXwBVAG4AaQB0ACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBhAG4AdQByAGUAQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA5AF8AXwAxAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMQBfAFMAbwB1AHIAYwBlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBhAG4AdQByAGUAQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA5AF8AXwAxAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBhAG4AdQByAGUAQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA5AF8AXwAxAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGEAbgB1AHIAZQBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADkAXwBfADEAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAxAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGEAbgB1AHIAZQBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADkAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAzACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBhAG4AdQByAGUAQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA5AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMwBfAFQAaQB0AGwAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AYQBuAHUAcgBlAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AOQBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBTAHcAaQBuAGUAXwBNAGEAbgB1AHIAZQBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA1AF8AMQBfADkAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAzAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AYQBuAHUAcgBlAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AOQBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADMAXwBTAG8AdQByAGMAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AYQBuAHUAcgBlAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AOQBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAFMAdwBpAG4AZQBfAE0AYQBuAHUAcgBlAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADUAXwAxAF8AOQBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8AUwB3AGkAbgBlAF8ATQBhAG4AdQByAGUAQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANQBfADEAXwA5AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMwBfAEEAcgBnAHUAbQBlAG4AdABzACIAXQAsACIAbABvAGMAYQBsAGUAIgA6AHsAIgBsAGkAcwB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAcgBvAHcAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBjAG8AbAB1AG0AbgBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUABvAHMAaQB0AGkAbwBuAHMAIgA6AFsAMwBdACwAIgBkAGUAYwBpAG0AYQBsAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiAC4AIgAsACIAZABhAHQAZQBPAHIAZABlAHIAIgA6ACIARABNAFkAIgAsACIAYwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsACIAOgAiACQAIgAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbABMAGUAYQBkACIAOgB0AHIAdQBlACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAZQBwAEIAeQBTAHAAYQBjAGUAIgA6AGYAYQBsAHMAZQAsACIAcgBvAHcATABlAHQAdABlAHIAIgA6ACIAUgAiACwAIgBjAG8AbAB1AG0AbgBMAGUAdAB0AGUAcgAiADoAIgBDACIALAAiAHIAYwBMAGUAZgB0AEIAcgBhAGMAawBlAHQAIgA6ACIAWwAiACwAIgByAGMAUgBpAGcAaAB0AEIAcgBhAGMAawBlAHQAIgA6ACIAXQAiACwAIgBzAHQAYQB0AGUAbQBlAG4AdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGwAbwBjAGEAbABlAE4AYQBtAGUAIgA6ACIAZQBuAC0AdQBzACIAfQB9AA==</AFEJSONBlob>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7291119c-fce9-4911-96ae-b800be5dccd8">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{809E3D44-A88D-4EBF-A307-6B8CE77A3361}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -19328,4 +19301,31 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="09eef6d6-daa8-4301-8f9f-b1ec38079286"/>
+    <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>